<commit_message>
update excel build scripts, finalise feedlot
</commit_message>
<xml_diff>
--- a/Excel/Common_v01.xlsx
+++ b/Excel/Common_v01.xlsx
@@ -8,21 +8,38 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\htdocs\zneagcrc\GAF-VEERG-Functions\Excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AB2272D4-83D6-4782-8546-72EBE880DEA7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F1AD5D3F-FEA4-408F-B764-2A4C13D2531F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="285" yWindow="390" windowWidth="37755" windowHeight="20445" xr2:uid="{992023F3-CAB7-4E5B-A348-08D563A0EF40}"/>
+    <workbookView xWindow="1170" yWindow="1170" windowWidth="28800" windowHeight="15345" xr2:uid="{992023F3-CAB7-4E5B-A348-08D563A0EF40}"/>
   </bookViews>
   <sheets>
-    <sheet name="Constants - Common" sheetId="1" r:id="rId1"/>
+    <sheet name="Constants - Common" sheetId="14" r:id="rId1"/>
   </sheets>
+  <externalReferences>
+    <externalReference r:id="rId2"/>
+  </externalReferences>
   <definedNames>
+    <definedName name="Common_Equations.Common_ConvertCH4ToCO2e">_xlfn.LAMBDA(_xlpm.E_CH4,_xlpm.GWP_CH4, _xlpm.E_CH4 * _xlpm.GWP_CH4)</definedName>
+    <definedName name="Common_Equations.Common_ConvertCH4ToCO2e_Arguments">_xlfn.LAMBDA(_xlfn.MAKEARRAY(2, 2, _xlfn.LAMBDA(_xlpm.r,_xlpm.c, INDEX({"ECH4","Methane emissions (t CH4)";"GWPCH4","Global warming potential for methane (t CO2-e / t CH4)"}, _xlpm.r, _xlpm.c))))</definedName>
+    <definedName name="Common_Equations.Common_ConvertCH4ToCO2e_LatexEquation">_xlfn.LAMBDA("CO2_e = E_{CH4} \times GWP_{CH4}")</definedName>
+    <definedName name="Common_Equations.Common_ConvertCH4ToCO2e_NIRReference">_xlfn.LAMBDA("")</definedName>
+    <definedName name="Common_Equations.Common_ConvertCH4ToCO2e_Title">_xlfn.LAMBDA("Convert methane emissions to carbon dioxide equivalent emissions")</definedName>
+    <definedName name="Common_Equations.Common_ConvertCH4ToCO2e_Unit">_xlfn.LAMBDA("t CO2e")</definedName>
+    <definedName name="Common_Equations.Common_ConvertCH4ToCO2e_Variable">_xlfn.LAMBDA("ECH4 CO2e")</definedName>
+    <definedName name="Common_Equations.Common_ConvertN2OToCO2e">_xlfn.LAMBDA(_xlpm.E_N2O,_xlpm.GWP_N2O, _xlpm.E_N2O * _xlpm.GWP_N2O)</definedName>
+    <definedName name="Common_Equations.Common_ConvertN2OToCO2e_Arguments">_xlfn.LAMBDA(_xlfn.MAKEARRAY(2, 2, _xlfn.LAMBDA(_xlpm.r,_xlpm.c, INDEX({"EN2O","Nitrous oxide emissions (t N2O)";"GWPN2O","Global warming potential for nitrous oxide (t CO2-e / t N2O)"}, _xlpm.r, _xlpm.c))))</definedName>
+    <definedName name="Common_Equations.Common_ConvertN2OToCO2e_LatexEquation">_xlfn.LAMBDA("CO2_e = E_{N2O} \times GWP_{N2O}")</definedName>
+    <definedName name="Common_Equations.Common_ConvertN2OToCO2e_NIRReference">_xlfn.LAMBDA("")</definedName>
+    <definedName name="Common_Equations.Common_ConvertN2OToCO2e_Title">_xlfn.LAMBDA("Convert nitrous oxide emissions to carbon dioxide equivalent emissions")</definedName>
+    <definedName name="Common_Equations.Common_ConvertN2OToCO2e_Unit">_xlfn.LAMBDA("t CO2e")</definedName>
+    <definedName name="Common_Equations.Common_ConvertN2OToCO2e_Variable">_xlfn.LAMBDA("EN2O CO2e")</definedName>
     <definedName name="Common_InputFunctions.getOverlappingReportingCycles">_xlfn.LAMBDA(_xlpm.ProductionCycleStart,_xlpm.ProductionCycleEnd,_xlpm.ReportingCycleStart, _xlfn.LET(_xlpm.S, _xlpm.ProductionCycleStart, _xlpm.E, _xlpm.ProductionCycleEnd, _xlpm.m, MONTH(_xlpm.ReportingCycleStart), _xlpm.d, DAY(_xlpm.ReportingCycleStart), _xlpm.PeriodEnd, _xlfn.LAMBDA(_xlpm.st, EDATE(_xlpm.st, 12) - 1), _xlpm.A, _xlpm.S - 365, _xlpm.ya, YEAR(_xlpm.A), _xlpm.yb, YEAR(_xlpm.E), _xlpm.firstYear, _xlpm.ya + (_xlpm.PeriodEnd(DATE(_xlpm.ya, _xlpm.m, _xlpm.d)) &lt; _xlpm.S), _xlpm.lastYear, _xlpm.yb - (DATE(_xlpm.yb, _xlpm.m, _xlpm.d) &gt; _xlpm.E), MAX(0, _xlpm.lastYear - _xlpm.firstYear + 1)))</definedName>
     <definedName name="Common_InputFunctions.getOverlappingReportingPeriods">_xlfn.LAMBDA(_xlpm.ProductionCycleStart,_xlpm.ProductionCycleEnd,_xlpm.ReportingCycleStart, _xlfn.LET(_xlpm.S, _xlpm.ProductionCycleStart, _xlpm.E, _xlpm.ProductionCycleEnd, _xlpm.m, MONTH(_xlpm.ReportingCycleStart), _xlpm.d, DAY(_xlpm.ReportingCycleStart), _xlpm.PeriodEnd, _xlfn.LAMBDA(_xlpm.st, EDATE(_xlpm.st, 12) - 1), _xlpm.A, _xlpm.S - 365, _xlpm.ya, YEAR(_xlpm.A), _xlpm.yb, YEAR(_xlpm.E), _xlpm.firstYear, _xlpm.ya + (_xlpm.PeriodEnd(DATE(_xlpm.ya, _xlpm.m, _xlpm.d)) &lt; _xlpm.S), _xlpm.lastYear, _xlpm.yb - (DATE(_xlpm.yb, _xlpm.m, _xlpm.d) &gt; _xlpm.E), _xlpm.n, MAX(0, _xlpm.lastYear - _xlpm.firstYear + 1), _xlpm.yrs, _xlfn.SEQUENCE(_xlpm.n, 1, _xlpm.firstYear, 1), _xlpm.starts, DATE(_xlpm.yrs, _xlpm.m, _xlpm.d), _xlpm.ends, _xlfn.MAP(_xlpm.starts, _xlpm.PeriodEnd), _xlpm.startsText, TEXT(_xlpm.starts, "dd mmm yyyy"), _xlpm.endsText, TEXT(_xlpm.ends, "dd mmm yyyy"), IF(_xlpm.n = 0, "", _xlfn.HSTACK(_xlpm.startsText &amp; " to " &amp; _xlpm.endsText))))</definedName>
     <definedName name="Common_InputFunctions.Utility_DisplayArrayInTable">_xlfn.LAMBDA(_xlpm.ArrayData,_xlpm.TableheaderCell,_xlpm.RowsBetweenHeaderandArray,_xlop.ColumnsBetweenHeaderAndArray, IFERROR(INDEX(_xlfn.UNIQUE(_xlpm.ArrayData), ROW() - Common_InputFunctions.Utility_GetArrayTableRowStartNumber(_xlpm.TableheaderCell, _xlpm.RowsBetweenHeaderandArray), COLUMN() - Common_InputFunctions.Utility_GetArrayTableColumnStartNumber(_xlpm.TableheaderCell) + IF(_xlfn.ISOMITTED(_xlpm.ColumnsBetweenHeaderAndArray), 1, _xlpm.ColumnsBetweenHeaderAndArray)), ""))</definedName>
     <definedName name="Common_InputFunctions.Utility_DisplayFunctionName">_xlfn.LAMBDA(_xlpm.Function, _xlfn.FORMULATEXT(_xlpm.Function))</definedName>
     <definedName name="Common_InputFunctions.Utility_GetArrayTableColumnStartNumber">_xlfn.LAMBDA(_xlpm.TableHeaderCell, COLUMN(_xlpm.TableHeaderCell))</definedName>
     <definedName name="Common_InputFunctions.Utility_GetArrayTableRowStartNumber">_xlfn.LAMBDA(_xlpm.TableheaderCell,_xlpm.RowsBetweenHeaderandArray, ROW(_xlpm.TableheaderCell) + _xlpm.RowsBetweenHeaderandArray - 1)</definedName>
-    <definedName name="Common_InputFunctions.Utility_GetClimateZone">_xlfn.LAMBDA(_xlpm.avgTemp,_xlpm.avgRain,_xlpm.frostDays,_xlpm.elev,_xlpm.map_pet, _xlfn.LET(_xlpm.mask, (VALUE(Table_SourceData_ClimateZones[Min temp]) &lt;= _xlpm.avgTemp) * (VALUE(Table_SourceData_ClimateZones[Max temp]) &gt;= _xlpm.avgTemp) * (VALUE(Table_SourceData_ClimateZones[Min rainfall]) &lt;= _xlpm.avgRain) * (VALUE(Table_SourceData_ClimateZones[Max rainfall]) &gt;= _xlpm.avgRain) * (VALUE(Table_SourceData_ClimateZones[Min frost days]) &lt;= _xlpm.frostDays) * (VALUE(Table_SourceData_ClimateZones[Max frost days]) &gt;= _xlpm.frostDays) * (VALUE(Table_SourceData_ClimateZones[Min elevation]) &lt;= _xlpm.elev) * (VALUE(Table_SourceData_ClimateZones[Max elevation]) &gt;= _xlpm.elev) * (VALUE(Table_SourceData_ClimateZones[Min MAP:PET]) &lt;= _xlpm.map_pet) * (VALUE(Table_SourceData_ClimateZones[Max MAP:PET]) &gt;= _xlpm.map_pet), _xlfn.TAKE(_xlfn._xlws.FILTER(Table_SourceData_ClimateZones[Climate zone], _xlpm.mask, "No match"), 1)))</definedName>
+    <definedName name="Common_InputFunctions.Utility_GetClimateZone">_xlfn.LAMBDA(_xlpm.avgTemp,_xlpm.avgRain,_xlpm.frostDays,_xlpm.elev,_xlpm.map_pet, _xlfn.LET(_xlpm.mask, (VALUE(#REF!) &lt;= _xlpm.avgTemp) * (VALUE(#REF!) &gt;= _xlpm.avgTemp) * (VALUE(#REF!) &lt;= _xlpm.avgRain) * (VALUE(#REF!) &gt;= _xlpm.avgRain) * (VALUE(#REF!) &lt;= _xlpm.frostDays) * (VALUE(#REF!) &gt;= _xlpm.frostDays) * (VALUE(#REF!) &lt;= _xlpm.elev) * (VALUE(#REF!) &gt;= _xlpm.elev) * (VALUE(#REF!) &lt;= _xlpm.map_pet) * (VALUE(#REF!) &gt;= _xlpm.map_pet), _xlfn.TAKE(_xlfn._xlws.FILTER(#REF!, _xlpm.mask, "No match"), 1)))</definedName>
     <definedName name="Common_InputFunctions.Utility_LookupItemFromMinMax">_xlfn.LAMBDA(_xlpm.LookupValue,_xlpm.MinArray,_xlpm.MaxArray,_xlpm.ItemArray, _xlfn.LET(_xlpm.mask, (VALUE(_xlpm.MinArray) &lt;= _xlpm.LookupValue) * (VALUE(_xlpm.MaxArray) &gt;= _xlpm.LookupValue), _xlfn._xlws.FILTER(_xlpm.ItemArray, _xlpm.mask, "No match")))</definedName>
     <definedName name="Common_InputFunctions.Utility_LookupValueInTable">_xlfn.LAMBDA(_xlpm.LookupValue,_xlpm.LookupArray,_xlpm.ReturnArray, _xlfn.XLOOKUP(_xlpm.LookupValue, _xlpm.LookupArray, _xlpm.ReturnArray, ""))</definedName>
     <definedName name="Common_InputFunctions.Utility_LookupValueInTableNumber">_xlfn.LAMBDA(_xlpm.LookupValue,_xlpm.LookupArray,_xlpm.ReturnArray, IF(ISNUMBER(_xlfn.XLOOKUP(_xlpm.LookupValue, _xlpm.LookupArray, _xlpm.ReturnArray, "")), _xlfn.XLOOKUP(_xlpm.LookupValue, _xlpm.LookupArray, _xlpm.ReturnArray, ""), 0))</definedName>
@@ -66,6 +83,12 @@
     <definedName name="Common_SourceData.Common_SourceData_EFleach_Title">_xlfn.LAMBDA("Emission factor for nitrogen leaching and runoff")</definedName>
     <definedName name="Common_SourceData.Common_SourceData_EFleach_Unit">_xlfn.LAMBDA("(kg N2O-N / kg N")</definedName>
     <definedName name="Common_SourceData.Common_SourceData_EFleach_Variation">_xlfn.LAMBDA((""))</definedName>
+    <definedName name="Common_SourceData.Common_SourceData_EFN2O_Data">_xlfn.LAMBDA(_xlfn.MAKEARRAY(14, 5, _xlfn.LAMBDA(_xlpm.r,_xlpm.c, INDEX({"Production system j","EFN2O","Production system only","Irrigation method","Rainfall zone";"Irrigated pasture",0.0059,"Pasture","Any","Any";"Irrigated crop",0.007,"Crop","Any","Any";"Non-irrigated pasture",0.0018,"Pasture","Not irrigated","Low rainfall";"Non-irrigated crop (low rainfall)",0.0029,"Crop","Not irrigated","Low rainfall";"Non-irrigated crop (high rainfall)",0.008,"Crop","Not irrigated","High rainfall";"Sugar",0.0199,"Sugar","Any","Any";"Cotton",0.0053,"Cotton","Any","Any";"Horticultural crops",0.0064,"Horticultural crops","Any","Any";"Rice (continuous flooding)",0.003,"Rice","Continuous flooding","Any";"Rice (single and multiple drainage, or alternate wetting and drying)",0.005,"Rice","Single and multiple drainage, or alternate wetting and drying","Any";"Aquaculture",0.0026,"Aquaculture","Any","Any";"Forestry",0.0018,"Forestry","Any","Any"}, _xlpm.r, _xlpm.c))))</definedName>
+    <definedName name="Common_SourceData.Common_SourceData_EFN2O_NIRReference">_xlfn.LAMBDA("")</definedName>
+    <definedName name="Common_SourceData.Common_SourceData_EFN2O_Source">_xlfn.LAMBDA("VEERG 2026: Table A.2.2.1")</definedName>
+    <definedName name="Common_SourceData.Common_SourceData_EFN2O_Title">_xlfn.LAMBDA("Nitrous oxide emission factors for inorganic fertiliser application")</definedName>
+    <definedName name="Common_SourceData.Common_SourceData_EFN2O_Unit">_xlfn.LAMBDA("(kg N2O-N / kg N")</definedName>
+    <definedName name="Common_SourceData.Common_SourceData_EFN2O_Variation">_xlfn.LAMBDA(_xlfn.MAKEARRAY(4, 1, _xlfn.LAMBDA(_xlpm.r,_xlpm.c, INDEX({"VARIATION OF SOURCE DATA:";"Removed duplicate 'Aquaculture' row.";"Removed asterisks to aid lookup.";"Added 'production system only', 'rainfall zone' and 'irrigation method' columns to aid lookup."}, _xlpm.r, _xlpm.c))))</definedName>
     <definedName name="Common_SourceData.Common_SourceData_FracLEACH_Data">_xlfn.LAMBDA(_xlfn.MAKEARRAY(1, 2, _xlfn.LAMBDA(_xlpm.r,_xlpm.c, INDEX({"FracLEACH",0.24}, _xlpm.r, _xlpm.c))))</definedName>
     <definedName name="Common_SourceData.Common_SourceData_FracLEACH_NIRReference">_xlfn.LAMBDA("National Inventory Report Volume 1: Leaching and runoff (3.D.b.2)")</definedName>
     <definedName name="Common_SourceData.Common_SourceData_FracLEACH_Source">_xlfn.LAMBDA("VEERG 2026:5.5.2.3 Constant Parameters")</definedName>
@@ -114,9 +137,12 @@
     <definedName name="Common_SourceData.Common_SourceData_WetAndDryZones_Variation">_xlfn.LAMBDA(_xlfn.MAKEARRAY(3, 1, _xlfn.LAMBDA(_xlpm.r,_xlpm.c, INDEX({"VARIATION OF SOURCE DATA:";"Added warm / cool temperate moist / dry - low frost and high temp classes to accommodate climate scenarios excluded by VEERG criteria.";"Fixed typo - Changed 'Fry' to 'Dry'."}, _xlpm.r, _xlpm.c))))</definedName>
     <definedName name="CommonLivestock_InputFunctions.AverageLiveweightEndOfMonth">_xlfn.LAMBDA(_xlpm.Month,_xlpm.LivestockClass,_xlpm.HeadAtStart,_xlpm.LiveweightAtStart,_xlpm.LiveweightGain, [0]!CommonLivestock_InputFunctions.LivestockMovement_ProportionalAverageLiveweightAddedDuringMonth(_xlpm.Month, _xlpm.LivestockClass, _xlpm.HeadAtStart) + [0]!CommonLivestock_InputFunctions.LivestockMovement_ProportionalAverageLiveweightRemainingAtEndOfMonth(_xlpm.Month, _xlpm.LivestockClass, _xlpm.HeadAtStart, _xlpm.LiveweightAtStart, _xlpm.LiveweightGain))</definedName>
     <definedName name="CommonLivestock_InputFunctions.LivestockMovement_AverageLiveweightAddedDuringMonth">_xlfn.LAMBDA(_xlpm.Month,_xlpm.LivestockClass, IFERROR([0]!CommonLivestock_InputFunctions.LivestockMovement_TotalLiveweightAddedDuringMonth(_xlpm.Month, _xlpm.LivestockClass) / [0]!CommonLivestock_InputFunctions.LivestockMovement_HeadAddedDuringMonth(_xlpm.Month, _xlpm.LivestockClass), 0))</definedName>
+    <definedName name="CommonLivestock_InputFunctions.LivestockMovement_GetMovementLiveweightGain" localSheetId="0">_xlfn.LAMBDA(_xlpm.LivestockClass,_xlpm.MovementDate, _xlfn.LET(_xlpm.ym, TEXT(_xlpm.MovementDate, "yyyymm"), IFERROR(INDEX(_xlfn._xlws.FILTER(#REF!, (TEXT(#REF!, "yyyymm") = _xlpm.ym) * (#REF! = _xlpm.LivestockClass)), 1), "")))</definedName>
     <definedName name="CommonLivestock_InputFunctions.LivestockMovement_GetMovementLiveweightGain">_xlfn.LAMBDA(_xlpm.LivestockClass,_xlpm.MovementDate, _xlfn.LET(_xlpm.ym, TEXT(_xlpm.MovementDate, "yyyymm"), IFERROR(INDEX(_xlfn._xlws.FILTER(#REF!, (TEXT(#REF!, "yyyymm") = _xlpm.ym) * (#REF! = _xlpm.LivestockClass)), 1), "")))</definedName>
+    <definedName name="CommonLivestock_InputFunctions.LivestockMovement_HeadAddedDuringMonth" localSheetId="0">_xlfn.LAMBDA(_xlpm.Month,_xlpm.LivestockClass, IFERROR(SUM(_xlfn._xlws.FILTER(#REF!, (#REF! &gt;= EOMONTH(_xlpm.Month, -1) + 1) * (#REF! &lt;= EOMONTH(_xlpm.Month, 0)) * (#REF! = _xlpm.LivestockClass))), 0))</definedName>
     <definedName name="CommonLivestock_InputFunctions.LivestockMovement_HeadAddedDuringMonth">_xlfn.LAMBDA(_xlpm.Month,_xlpm.LivestockClass, IFERROR(SUM(_xlfn._xlws.FILTER(#REF!, (#REF! &gt;= EOMONTH(_xlpm.Month, -1) + 1) * (#REF! &lt;= EOMONTH(_xlpm.Month, 0)) * (#REF! = _xlpm.LivestockClass))), 0))</definedName>
     <definedName name="CommonLivestock_InputFunctions.LivestockMovement_HeadAtEndOfMonth">_xlfn.LAMBDA(_xlpm.HeadAtStart,_xlpm.Month,_xlpm.LivestockClass, _xlpm.HeadAtStart + [0]!CommonLivestock_InputFunctions.LivestockMovement_HeadAddedDuringMonth(_xlpm.Month, _xlpm.LivestockClass) - [0]!CommonLivestock_InputFunctions.LivestockMovement_HeadLostDuringMonth(_xlpm.Month, _xlpm.LivestockClass))</definedName>
+    <definedName name="CommonLivestock_InputFunctions.LivestockMovement_HeadLostDuringMonth" localSheetId="0">_xlfn.LAMBDA(_xlpm.Month,_xlpm.LivestockClass, IFERROR(SUM(_xlfn._xlws.FILTER(#REF!, (#REF! &gt;= EOMONTH(_xlpm.Month, -1) + 1) * (#REF! &lt;= EOMONTH(_xlpm.Month, 0)) * (#REF! = _xlpm.LivestockClass))), 0))</definedName>
     <definedName name="CommonLivestock_InputFunctions.LivestockMovement_HeadLostDuringMonth">_xlfn.LAMBDA(_xlpm.Month,_xlpm.LivestockClass, IFERROR(SUM(_xlfn._xlws.FILTER(#REF!, (#REF! &gt;= EOMONTH(_xlpm.Month, -1) + 1) * (#REF! &lt;= EOMONTH(_xlpm.Month, 0)) * (#REF! = _xlpm.LivestockClass))), 0))</definedName>
     <definedName name="CommonLivestock_InputFunctions.LivestockMovement_HeadRemainingAtMonthEnd">_xlfn.LAMBDA(_xlpm.Month,_xlpm.LivestockClass,_xlpm.HeadAtStartOfMonth, MAX(_xlpm.HeadAtStartOfMonth - [0]!CommonLivestock_InputFunctions.LivestockMovement_HeadLostDuringMonth(_xlpm.Month, _xlpm.LivestockClass), 0))</definedName>
     <definedName name="CommonLivestock_InputFunctions.LivestockMovement_LiveweightAddedDuringMonth">_xlfn.LAMBDA(_xlpm.LivestockClass,_xlpm.MovementDate,_xlpm.WeightAtMovementDate,_xlpm.Head, IFERROR(_xlpm.Head * (_xlpm.WeightAtMovementDate + [0]!CommonLivestock_InputFunctions.LivestockMovement_LiveweightGrownDuringMonthPerHead(_xlpm.LivestockClass, _xlpm.MovementDate)), 0))</definedName>
@@ -128,7 +154,9 @@
     <definedName name="CommonLivestock_InputFunctions.LivestockMovement_ProportionalAverageLiveweightRemainingAtEndOfMonth">_xlfn.LAMBDA(_xlpm.Month,_xlpm.LivestockClass,_xlpm.HeadAtStart,_xlpm.LiveweightAtStart,_xlpm.LiveweightGain, [0]!CommonLivestock_InputFunctions.LivestockMovement_ProportionHeadRemainingAtEndOfMonth(_xlpm.Month, _xlpm.LivestockClass, _xlpm.HeadAtStart) * CommonLivestock_InputFunctions.LivestockMovement_AverageLiveweightRemainingHead(_xlpm.Month, _xlpm.LiveweightAtStart, _xlpm.LiveweightGain))</definedName>
     <definedName name="CommonLivestock_InputFunctions.LivestockMovement_ProportionHeadAddedDuringMonth">_xlfn.LAMBDA(_xlpm.Month,_xlpm.LivestockClass,_xlpm.HeadAtStart, IFERROR(MIN(1, [0]!CommonLivestock_InputFunctions.LivestockMovement_HeadAddedDuringMonth(_xlpm.Month, _xlpm.LivestockClass) / [0]!CommonLivestock_InputFunctions.LivestockMovement_HeadAtEndOfMonth(_xlpm.HeadAtStart, _xlpm.Month, _xlpm.LivestockClass)), 0))</definedName>
     <definedName name="CommonLivestock_InputFunctions.LivestockMovement_ProportionHeadRemainingAtEndOfMonth">_xlfn.LAMBDA(_xlpm.Month,_xlpm.LivestockClass,_xlpm.HeadAtStart, IFERROR(MIN(1, [0]!CommonLivestock_InputFunctions.LivestockMovement_HeadRemainingAtMonthEnd(_xlpm.Month, _xlpm.LivestockClass, _xlpm.HeadAtStart) / [0]!CommonLivestock_InputFunctions.LivestockMovement_HeadAtEndOfMonth(_xlpm.HeadAtStart, _xlpm.Month, _xlpm.LivestockClass)), 0))</definedName>
+    <definedName name="CommonLivestock_InputFunctions.LivestockMovement_TotalLiveweightAddedDuringMonth" localSheetId="0">_xlfn.LAMBDA(_xlpm.Month,_xlpm.LivestockClass, IFERROR(SUM(_xlfn._xlws.FILTER(#REF!, (#REF! &gt;= EOMONTH(_xlpm.Month, -1) + 1) * (#REF! &lt;= EOMONTH(_xlpm.Month, 0)) * (#REF! = _xlpm.LivestockClass))), 0))</definedName>
     <definedName name="CommonLivestock_InputFunctions.LivestockMovement_TotalLiveweightAddedDuringMonth">_xlfn.LAMBDA(_xlpm.Month,_xlpm.LivestockClass, IFERROR(SUM(_xlfn._xlws.FILTER(#REF!, (#REF! &gt;= EOMONTH(_xlpm.Month, -1) + 1) * (#REF! &lt;= EOMONTH(_xlpm.Month, 0)) * (#REF! = _xlpm.LivestockClass))), 0))</definedName>
+    <definedName name="CommonLivestock_InputFunctions.LivestockMovement_TotalLiveweightGrownDuringMonth" localSheetId="0">_xlfn.LAMBDA(_xlpm.Month,_xlpm.LivestockClass, IFERROR(SUM(_xlfn._xlws.FILTER(#REF!, (#REF! &gt;= EOMONTH(_xlpm.Month, -1) + 1) * (#REF! &lt;= EOMONTH(_xlpm.Month, 0)) * (#REF! = _xlpm.LivestockClass))), 0))</definedName>
     <definedName name="CommonLivestock_InputFunctions.LivestockMovement_TotalLiveweightGrownDuringMonth">_xlfn.LAMBDA(_xlpm.Month,_xlpm.LivestockClass, IFERROR(SUM(_xlfn._xlws.FILTER(#REF!, (#REF! &gt;= EOMONTH(_xlpm.Month, -1) + 1) * (#REF! &lt;= EOMONTH(_xlpm.Month, 0)) * (#REF! = _xlpm.LivestockClass))), 0))</definedName>
     <definedName name="CommonLivestock_InputFunctions.LivestockMovement_TotalLiveweightGrownDuringMonthAddedAndRemaining">_xlfn.LAMBDA(_xlpm.Month,_xlpm.LivestockClass,_xlpm.HeadAtStart, [0]!CommonLivestock_InputFunctions.LivestockMovement_LiveweightGrownFromMonthStartTotal(_xlpm.LivestockClass, _xlpm.Month, _xlpm.HeadAtStart) + [0]!CommonLivestock_InputFunctions.LivestockMovement_TotalLiveweightGrownDuringMonth(_xlpm.Month, _xlpm.LivestockClass))</definedName>
     <definedName name="getOverlappingReportingCycles">_xlfn.LAMBDA(_xlpm.ProductionCycleStart,_xlpm.ProductionCycleEnd,_xlpm.ReportingStartMonth,_xlpm.ReportingStartDay, _xlfn.LET(_xlpm.S, _xlpm.ProductionCycleStart, _xlpm.E, _xlpm.ProductionCycleEnd, _xlpm.m, _xlpm.ReportingStartMonth, _xlpm.d, _xlpm.ReportingStartDay, _xlpm.A, _xlpm.S - 364, _xlpm.ya, YEAR(_xlpm.A), _xlpm.yb, YEAR(_xlpm.E), _xlpm.firstYear, _xlpm.ya + (DATE(_xlpm.ya, _xlpm.m, _xlpm.d) &lt; _xlpm.A), _xlpm.lastYear, _xlpm.yb - (DATE(_xlpm.yb, _xlpm.m, _xlpm.d) &gt; _xlpm.E), MAX(0, _xlpm.lastYear - _xlpm.firstYear + 1)))</definedName>
@@ -208,7 +236,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="39">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="52" uniqueCount="47">
   <si>
     <t>Climate zone</t>
   </si>
@@ -326,6 +354,30 @@
   <si>
     <t>FracWET</t>
   </si>
+  <si>
+    <t>Production system j</t>
+  </si>
+  <si>
+    <t>EFN2O</t>
+  </si>
+  <si>
+    <t>Production system only</t>
+  </si>
+  <si>
+    <t>Irrigation method</t>
+  </si>
+  <si>
+    <t>Rainfall zone</t>
+  </si>
+  <si>
+    <t>test</t>
+  </si>
+  <si>
+    <t>test 2</t>
+  </si>
+  <si>
+    <t>test 3</t>
+  </si>
 </sst>
 </file>
 
@@ -335,10 +387,10 @@
     <numFmt numFmtId="164" formatCode="0.000"/>
     <numFmt numFmtId="165" formatCode="#,##0.000"/>
     <numFmt numFmtId="166" formatCode="d/mm/yyyy;@"/>
-    <numFmt numFmtId="168" formatCode="[$-C09]dd\-mmmm\-yyyy;@"/>
-    <numFmt numFmtId="169" formatCode="#,##0.000000"/>
+    <numFmt numFmtId="167" formatCode="[$-C09]dd\-mmmm\-yyyy;@"/>
+    <numFmt numFmtId="168" formatCode="#,##0.000000"/>
   </numFmts>
-  <fonts count="33" x14ac:knownFonts="1">
+  <fonts count="32" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -468,12 +520,6 @@
       <color theme="0"/>
       <name val="Times New Roman"/>
       <family val="1"/>
-    </font>
-    <font>
-      <sz val="8"/>
-      <name val="Times New Roman"/>
-      <family val="2"/>
-      <scheme val="minor"/>
     </font>
     <font>
       <sz val="11"/>
@@ -703,16 +749,16 @@
     <xf numFmtId="0" fontId="16" fillId="3" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="4" borderId="0">
+    <xf numFmtId="0" fontId="23" fillId="4" borderId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="29" fillId="4" borderId="0">
+    <xf numFmtId="0" fontId="28" fillId="4" borderId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="27" fillId="4" borderId="0">
+    <xf numFmtId="0" fontId="26" fillId="4" borderId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="2" borderId="0">
@@ -801,65 +847,65 @@
     <xf numFmtId="0" fontId="18" fillId="8" borderId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="0">
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0">
       <alignment horizontal="left" vertical="center" indent="2"/>
     </xf>
-    <xf numFmtId="0" fontId="30" fillId="12" borderId="4">
+    <xf numFmtId="0" fontId="29" fillId="12" borderId="4">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="3" fontId="22" fillId="4" borderId="1">
+    <xf numFmtId="3" fontId="21" fillId="4" borderId="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="168" fontId="2" fillId="0" borderId="1">
+    <xf numFmtId="167" fontId="2" fillId="0" borderId="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="0"/>
-    <xf numFmtId="166" fontId="22" fillId="4" borderId="1">
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="0"/>
+    <xf numFmtId="166" fontId="21" fillId="4" borderId="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="4" fontId="22" fillId="4" borderId="1">
+    <xf numFmtId="4" fontId="21" fillId="4" borderId="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="26" fillId="4" borderId="0">
+    <xf numFmtId="0" fontId="25" fillId="4" borderId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="4" borderId="0" applyNumberFormat="0">
+    <xf numFmtId="0" fontId="24" fillId="4" borderId="0" applyNumberFormat="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="22" fillId="4" borderId="1">
+    <xf numFmtId="165" fontId="21" fillId="4" borderId="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="4" borderId="0">
+    <xf numFmtId="0" fontId="20" fillId="4" borderId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="169" fontId="22" fillId="4" borderId="1">
+    <xf numFmtId="168" fontId="21" fillId="4" borderId="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="4" borderId="1">
+    <xf numFmtId="0" fontId="21" fillId="4" borderId="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="4" borderId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="28" fillId="4" borderId="0">
+    <xf numFmtId="0" fontId="27" fillId="4" borderId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="30" fillId="4" borderId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="31" fillId="4" borderId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="32" fillId="4" borderId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellStyleXfs>
   <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="27" fillId="4" borderId="0" xfId="8">
+    <xf numFmtId="0" fontId="26" fillId="4" borderId="0" xfId="8">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="7">
@@ -868,10 +914,10 @@
     <xf numFmtId="0" fontId="16" fillId="3" borderId="0" xfId="4">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="29" fillId="4" borderId="0" xfId="6">
+    <xf numFmtId="0" fontId="28" fillId="4" borderId="0" xfId="6">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="4" borderId="0" xfId="5">
+    <xf numFmtId="0" fontId="23" fillId="4" borderId="0" xfId="5">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="7" applyFill="1">
@@ -891,7 +937,7 @@
     <xf numFmtId="0" fontId="6" fillId="4" borderId="0" xfId="53">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="28" fillId="4" borderId="0" xfId="54">
+    <xf numFmtId="0" fontId="27" fillId="4" borderId="0" xfId="54">
       <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1609,6 +1655,22 @@
 </styleSheet>
 </file>
 
+<file path=xl/externalLinks/externalLink1.xml><?xml version="1.0" encoding="utf-8"?>
+<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
+  <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
+    <xxl21:alternateUrls>
+      <xxl21:absoluteUrl r:id="rId2"/>
+    </xxl21:alternateUrls>
+    <sheetNames>
+      <sheetName val="Constants - Common"/>
+    </sheetNames>
+    <sheetDataSet>
+      <sheetData sheetId="0"/>
+    </sheetDataSet>
+  </externalBook>
+</externalLink>
+</file>
+
 <file path=xl/richData/rdRichValueTypes.xml><?xml version="1.0" encoding="utf-8"?>
 <rvTypesInfo xmlns="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" mc:Ignorable="x">
   <global>
@@ -1674,21 +1736,21 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="35" xr:uid="{E0906749-7FC7-47DE-82F6-F796C4463018}" name="Table_AustralianStates" displayName="Table_AustralianStates" ref="D6:F14" totalsRowShown="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="13" xr:uid="{70E3688E-4550-4D37-92E4-8E6D7B93986F}" name="Table_AustralianStates" displayName="Table_AustralianStates" ref="D6:F14" totalsRowShown="0">
   <autoFilter ref="D6:F14" xr:uid="{E0906749-7FC7-47DE-82F6-F796C4463018}">
     <filterColumn colId="0" hiddenButton="1"/>
     <filterColumn colId="1" hiddenButton="1"/>
     <filterColumn colId="2" hiddenButton="1"/>
   </autoFilter>
   <tableColumns count="3">
-    <tableColumn id="1" xr3:uid="{AEDF0F21-30D6-4DC6-90D9-B28878486711}" name="State/Territory">
-      <calculatedColumnFormula array="1">InputFunctions_Utilities.Utility_DisplayArrayInTable(SourceData_Common.SourceData_Common_AustralianStatesTerritories_Data(),Table_AustralianStates[[#Headers],[State/Territory]],0)</calculatedColumnFormula>
+    <tableColumn id="1" xr3:uid="{5AE544D6-6CBB-4119-B5C5-091C6E27A988}" name="State/Territory">
+      <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_AustralianStatesTerritories_Data(),Table_AustralianStates[[#Headers],[State/Territory]],0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{46746E17-67FE-4DE2-A5E2-E900B123DBAA}" name="Common Name">
-      <calculatedColumnFormula array="1">InputFunctions_Utilities.Utility_DisplayArrayInTable(SourceData_Common.SourceData_Common_AustralianStatesTerritories_Data(),Table_AustralianStates[[#Headers],[State/Territory]],0)</calculatedColumnFormula>
+    <tableColumn id="2" xr3:uid="{BF8D713A-6FD6-4CAB-AF21-DBA86B554721}" name="Common Name">
+      <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_AustralianStatesTerritories_Data(),Table_AustralianStates[[#Headers],[State/Territory]],0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="3" xr3:uid="{5C5F8341-C8D2-41BE-B1BD-34A42E441B01}" name="Abbreviation">
-      <calculatedColumnFormula array="1">InputFunctions_Utilities.Utility_DisplayArrayInTable(SourceData_Common.SourceData_Common_AustralianStatesTerritories_Data(),Table_AustralianStates[[#Headers],[State/Territory]],0)</calculatedColumnFormula>
+    <tableColumn id="3" xr3:uid="{F0BC5BA0-7D2B-4193-AAB1-4E55191B02D9}" name="Abbreviation">
+      <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_AustralianStatesTerritories_Data(),Table_AustralianStates[[#Headers],[State/Territory]],0)</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
   <tableStyleInfo name="Equation table" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
@@ -1696,16 +1758,16 @@
 </file>
 
 <file path=xl/tables/table10.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="55" xr:uid="{133D42B0-F6D2-470A-858A-37E6A7F5EC2B}" name="Table_SourceData_DataScores_Scope3" displayName="Table_SourceData_DataScores_Scope3" ref="D142:E147" totalsRowShown="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="22" xr:uid="{5EE6BF60-CE26-4377-8154-DF5907B0B692}" name="Table_SourceData_DataScores_Scope3" displayName="Table_SourceData_DataScores_Scope3" ref="D142:E147" totalsRowShown="0">
   <autoFilter ref="D142:E147" xr:uid="{133D42B0-F6D2-470A-858A-37E6A7F5EC2B}">
     <filterColumn colId="0" hiddenButton="1"/>
     <filterColumn colId="1" hiddenButton="1"/>
   </autoFilter>
   <tableColumns count="2">
-    <tableColumn id="1" xr3:uid="{A9DA4FD2-DEF5-4DC6-9632-12EB6948FD08}" name="Data source">
+    <tableColumn id="1" xr3:uid="{68EABE1B-963C-47DD-9D87-D9246D45A477}" name="Data source">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_DataScores_Scope3_Data(), Table_SourceData_DataScores_Scope3[[#Headers],[Data source]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{E2DE90A7-DD83-4933-A185-E076F73E3141}" name="Data score">
+    <tableColumn id="2" xr3:uid="{11CEB607-ADD4-4046-BF94-7934247978CD}" name="Data score">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_DataScores_Scope3_Data(), Table_SourceData_DataScores_Scope3[[#Headers],[Data source]], 0)</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -1714,16 +1776,16 @@
 </file>
 
 <file path=xl/tables/table11.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="78" xr:uid="{308E99BE-FE1F-47A4-B2CA-97217277C4E9}" name="Table_SourceData_FracWET" displayName="Table_SourceData_FracWET" ref="D134:E136" totalsRowShown="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="23" xr:uid="{43B9E031-0DAE-47E1-A28D-9CA693FDF6ED}" name="Table_SourceData_FracWET" displayName="Table_SourceData_FracWET" ref="D134:E136" totalsRowShown="0">
   <autoFilter ref="D134:E136" xr:uid="{308E99BE-FE1F-47A4-B2CA-97217277C4E9}">
     <filterColumn colId="0" hiddenButton="1"/>
     <filterColumn colId="1" hiddenButton="1"/>
   </autoFilter>
   <tableColumns count="2">
-    <tableColumn id="1" xr3:uid="{EE610985-3845-4DCC-B7C5-D8A476C71C3D}" name="Is in leaching zone">
+    <tableColumn id="1" xr3:uid="{9EAD8DDD-FB08-42A5-B9E0-6C4315AEE8B1}" name="Is in leaching zone">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_FracWET_Data(),Table_SourceData_FracWET[[#Headers],[Is in leaching zone]],0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{01250727-4553-4905-AA33-A18CFA70E7C7}" name="FracWET" dataDxfId="0">
+    <tableColumn id="2" xr3:uid="{9E8DF127-FD5D-486C-B271-7A4F84E7D5B7}" name="FracWET" dataDxfId="0">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_FracWET_Data(),Table_SourceData_FracWET[[#Headers],[Is in leaching zone]],0)</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -1731,14 +1793,44 @@
 </table>
 </file>
 
+<file path=xl/tables/table12.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="24" xr:uid="{F8ED201F-FF01-45AD-8F36-BD6B21B4BD7F}" name="Table_SourceData_Common_EFN2O" displayName="Table_SourceData_Common_EFN2O" ref="D175:H188" totalsRowShown="0">
+  <autoFilter ref="D175:H188" xr:uid="{D41FBEA4-8379-4DF7-A068-BF94D364F1A2}">
+    <filterColumn colId="0" hiddenButton="1"/>
+    <filterColumn colId="1" hiddenButton="1"/>
+    <filterColumn colId="2" hiddenButton="1"/>
+    <filterColumn colId="3" hiddenButton="1"/>
+    <filterColumn colId="4" hiddenButton="1"/>
+  </autoFilter>
+  <tableColumns count="5">
+    <tableColumn id="1" xr3:uid="{83D0A318-3C7C-411A-B48E-8C101797A5D1}" name="Production system j">
+      <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_EFN2O_Data(), Table_SourceData_Common_EFN2O[[#Headers],[Production system j]], 0)</calculatedColumnFormula>
+    </tableColumn>
+    <tableColumn id="2" xr3:uid="{5CD5D5AB-7A74-4746-AB6D-BAA01B8181B4}" name="EFN2O">
+      <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_EFN2O_Data(), Table_SourceData_Common_EFN2O[[#Headers],[Production system j]], 0)</calculatedColumnFormula>
+    </tableColumn>
+    <tableColumn id="3" xr3:uid="{AFC49662-E901-416F-8B07-CB0A6B3B7409}" name="Production system only">
+      <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_EFN2O_Data(), Table_SourceData_Common_EFN2O[[#Headers],[Production system j]], 0)</calculatedColumnFormula>
+    </tableColumn>
+    <tableColumn id="4" xr3:uid="{2D5EAFB0-7F67-4E2A-AFEC-589CDA2640D7}" name="Irrigation method">
+      <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_EFN2O_Data(), Table_SourceData_Common_EFN2O[[#Headers],[Production system j]], 0)</calculatedColumnFormula>
+    </tableColumn>
+    <tableColumn id="5" xr3:uid="{FE8A229D-4ABE-4DE7-977F-336F28BA8FFD}" name="Rainfall zone">
+      <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_EFN2O_Data(), Table_SourceData_Common_EFN2O[[#Headers],[Production system j]], 0)</calculatedColumnFormula>
+    </tableColumn>
+  </tableColumns>
+  <tableStyleInfo name="Equation table" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="36" xr:uid="{5FA81339-C6C8-4D36-BEEA-6C4AEDD9E676}" name="Table_WASA4Areas" displayName="Table_WASA4Areas" ref="D20:D30" totalsRowShown="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="14" xr:uid="{200A0681-B1CE-43A0-9C2C-E63A2F4C8176}" name="Table_WASA4Areas" displayName="Table_WASA4Areas" ref="D20:D30" totalsRowShown="0">
   <autoFilter ref="D20:D30" xr:uid="{5FA81339-C6C8-4D36-BEEA-6C4AEDD9E676}">
     <filterColumn colId="0" hiddenButton="1"/>
   </autoFilter>
   <tableColumns count="1">
-    <tableColumn id="1" xr3:uid="{BA0BFB2C-353C-4FA0-A43A-0C86271AC72D}" name="SA 4 Name">
-      <calculatedColumnFormula array="1">InputFunctions_Utilities.Utility_DisplayArrayInTable(SourceData_Common.SourceData_Common_WASA4Areas_Data(), Table_WASA4Areas[[#Headers],[SA 4 Name]], 0)</calculatedColumnFormula>
+    <tableColumn id="1" xr3:uid="{099E98CA-54FE-4A54-9A7A-47F29FDE5C39}" name="SA 4 Name">
+      <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_WASA4Areas_Data(), Table_WASA4Areas[[#Headers],[SA 4 Name]], 0)</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
   <tableStyleInfo name="Equation table" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
@@ -1746,17 +1838,17 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="17" xr:uid="{B8E87A66-3E41-4AD3-925D-01EE21B43D7A}" name="Table_GWPData" displayName="Table_GWPData" ref="D36:E43" totalsRowShown="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="15" xr:uid="{0DE30BBE-2E67-4C99-93B9-5650B3570310}" name="Table_GWPData" displayName="Table_GWPData" ref="D36:E43" totalsRowShown="0">
   <autoFilter ref="D36:E43" xr:uid="{B8E87A66-3E41-4AD3-925D-01EE21B43D7A}">
     <filterColumn colId="0" hiddenButton="1"/>
     <filterColumn colId="1" hiddenButton="1"/>
   </autoFilter>
   <tableColumns count="2">
-    <tableColumn id="1" xr3:uid="{D3EC5F11-79A1-4A25-8E52-628D1910D761}" name="Gas">
-      <calculatedColumnFormula array="1">InputFunctions_Utilities.Utility_DisplayArrayInTable(SourceData_Common.SourceData_Common_GWP_Data(), Table_GWPData[[#Headers],[Gas]], 0)</calculatedColumnFormula>
+    <tableColumn id="1" xr3:uid="{54ED2520-7DCD-4AEB-9D61-39C29BBB211D}" name="Gas">
+      <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_GWP_Data(), Table_GWPData[[#Headers],[Gas]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{7C22FC98-4FBA-41C9-A44A-5811DB9E3402}" name="CO2-e factor">
-      <calculatedColumnFormula array="1">InputFunctions_Utilities.Utility_DisplayArrayInTable(SourceData_Common.SourceData_Common_GWP_Data(), Table_GWPData[[#Headers],[Gas]], 0)</calculatedColumnFormula>
+    <tableColumn id="2" xr3:uid="{90B16C7B-E1D7-496E-9F5E-7B399B4EB76E}" name="CO2-e factor">
+      <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_GWP_Data(), Table_GWPData[[#Headers],[Gas]], 0)</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
   <tableStyleInfo name="Equation table" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
@@ -1764,7 +1856,7 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="25" xr:uid="{C1F562BB-DAA6-45BB-951A-7BAFA5B64B45}" name="Table_GasToMolecularConversionFactor" displayName="Table_GasToMolecularConversionFactor" ref="D47:H54" totalsRowShown="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="16" xr:uid="{527CC946-57F5-4D57-9741-4E5839209E66}" name="Table_GasToMolecularConversionFactor" displayName="Table_GasToMolecularConversionFactor" ref="D47:H54" totalsRowShown="0">
   <autoFilter ref="D47:H54" xr:uid="{C1F562BB-DAA6-45BB-951A-7BAFA5B64B45}">
     <filterColumn colId="0" hiddenButton="1"/>
     <filterColumn colId="1" hiddenButton="1"/>
@@ -1773,19 +1865,19 @@
     <filterColumn colId="4" hiddenButton="1"/>
   </autoFilter>
   <tableColumns count="5">
-    <tableColumn id="1" xr3:uid="{DD533D11-7BC1-47AF-9AAC-8EC81432FA5B}" name="Gas">
-      <calculatedColumnFormula array="1">InputFunctions_Utilities.Utility_DisplayArrayInTable(SourceData_Common.SourceData_Common_ConvertGasElementalToMolecular_Data(),Table_GasToMolecularConversionFactor[[#Headers],[Gas]], 0)</calculatedColumnFormula>
+    <tableColumn id="1" xr3:uid="{3AF87ECF-AD12-40D9-9A34-B8C322351989}" name="Gas">
+      <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_ConvertGasElementalToMolecular_Data(),Table_GasToMolecularConversionFactor[[#Headers],[Gas]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="5" xr3:uid="{547883D7-1288-4839-9925-11EC372CE88D}" name="Conversion factor">
-      <calculatedColumnFormula array="1">InputFunctions_Utilities.Utility_DisplayArrayInTable(SourceData_Common.SourceData_Common_ConvertGasElementalToMolecular_Data(),Table_GasToMolecularConversionFactor[[#Headers],[Gas]], 0)</calculatedColumnFormula>
+    <tableColumn id="5" xr3:uid="{C2128F92-CB50-4903-8EF0-40843A63E8E2}" name="Conversion factor">
+      <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_ConvertGasElementalToMolecular_Data(),Table_GasToMolecularConversionFactor[[#Headers],[Gas]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{F4A922C9-B30F-4AB7-9D59-89F81921D5E7}" name="Conversion factor 1">
-      <calculatedColumnFormula array="1">InputFunctions_Utilities.Utility_DisplayArrayInTable(SourceData_Common.SourceData_Common_ConvertGasElementalToMolecular_Data(),Table_GasToMolecularConversionFactor[[#Headers],[Gas]], 0)</calculatedColumnFormula>
+    <tableColumn id="2" xr3:uid="{935334FD-4E47-4440-BE5C-5503DA853552}" name="Conversion factor 1">
+      <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_ConvertGasElementalToMolecular_Data(),Table_GasToMolecularConversionFactor[[#Headers],[Gas]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="3" xr3:uid="{B9BE2574-25AA-4F1B-AF93-4C5D0D5D9DB8}" name="Conversion factor 2">
-      <calculatedColumnFormula array="1">InputFunctions_Utilities.Utility_DisplayArrayInTable(SourceData_Common.SourceData_Common_ConvertGasElementalToMolecular_Data(),Table_GasToMolecularConversionFactor[[#Headers],[Gas]], 0)</calculatedColumnFormula>
+    <tableColumn id="3" xr3:uid="{FFB95828-61BC-4516-AA27-A6946CD503CE}" name="Conversion factor 2">
+      <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_ConvertGasElementalToMolecular_Data(),Table_GasToMolecularConversionFactor[[#Headers],[Gas]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="4" xr3:uid="{052E6F6E-0B83-44BB-8210-F23D2612CABD}" name="Conversion factor combined">
+    <tableColumn id="4" xr3:uid="{D7065489-B161-49B8-8A59-08BDFD64E159}" name="Conversion factor combined">
       <calculatedColumnFormula>Table_GasToMolecularConversionFactor[[#This Row],[Conversion factor 1]]/Table_GasToMolecularConversionFactor[[#This Row],[Conversion factor 2]]</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -1794,7 +1886,7 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="50" xr:uid="{5A437AE9-7724-4CF2-ACCF-291078682FB9}" name="Table_SourceData_ClimateZones" displayName="Table_SourceData_ClimateZones" ref="D89:S97" totalsRowShown="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="17" xr:uid="{E2F324C3-5204-4DB7-90EA-1335F81926F8}" name="Table_SourceData_ClimateZones" displayName="Table_SourceData_ClimateZones" ref="D89:S97" totalsRowShown="0">
   <autoFilter ref="D89:S97" xr:uid="{5A437AE9-7724-4CF2-ACCF-291078682FB9}">
     <filterColumn colId="0" hiddenButton="1"/>
     <filterColumn colId="1" hiddenButton="1"/>
@@ -1814,53 +1906,53 @@
     <filterColumn colId="15" hiddenButton="1"/>
   </autoFilter>
   <tableColumns count="16">
-    <tableColumn id="1" xr3:uid="{EC53732C-A9F9-48AD-A3CB-B4760097606E}" name="Climate zone" totalsRowCellStyle="Content bold">
-      <calculatedColumnFormula array="1">InputFunctions_Utilities.Utility_DisplayArrayInTable(SourceData_Common.SourceData_Common_ClimateZones_Data(), Table_SourceData_ClimateZones[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
+    <tableColumn id="1" xr3:uid="{3A3D3818-A5A1-48AD-9BB8-7D638C1E32AE}" name="Climate zone" totalsRowCellStyle="Content bold">
+      <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_ClimateZones_Data(), Table_SourceData_ClimateZones[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{AD0DEE0C-10DC-47BF-872F-7DE7910DB3B7}" name="MAT" totalsRowDxfId="16" totalsRowCellStyle="Content bold">
-      <calculatedColumnFormula array="1">InputFunctions_Utilities.Utility_DisplayArrayInTable(SourceData_Common.SourceData_Common_ClimateZones_Data(), Table_SourceData_ClimateZones[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
+    <tableColumn id="2" xr3:uid="{59814154-9022-4047-A927-D808F88DD7DD}" name="MAT" totalsRowDxfId="16" totalsRowCellStyle="Content bold">
+      <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_ClimateZones_Data(), Table_SourceData_ClimateZones[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="3" xr3:uid="{F5413B88-DBB1-4866-917E-9175D1ABD29E}" name="MAP" totalsRowDxfId="15" totalsRowCellStyle="Content bold">
-      <calculatedColumnFormula array="1">InputFunctions_Utilities.Utility_DisplayArrayInTable(SourceData_Common.SourceData_Common_ClimateZones_Data(), Table_SourceData_ClimateZones[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
+    <tableColumn id="3" xr3:uid="{F6B768A6-9933-4CD7-8DDB-C32DE40C5D5D}" name="MAP" totalsRowDxfId="15" totalsRowCellStyle="Content bold">
+      <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_ClimateZones_Data(), Table_SourceData_ClimateZones[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="4" xr3:uid="{51AA9590-F173-4D3B-9691-BEB628B2816C}" name="Frost days per year" totalsRowDxfId="14" totalsRowCellStyle="Content bold">
-      <calculatedColumnFormula array="1">InputFunctions_Utilities.Utility_DisplayArrayInTable(SourceData_Common.SourceData_Common_ClimateZones_Data(), Table_SourceData_ClimateZones[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
+    <tableColumn id="4" xr3:uid="{75A564B3-D32E-4FD0-9D03-FE7B38188305}" name="Frost days per year" totalsRowDxfId="14" totalsRowCellStyle="Content bold">
+      <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_ClimateZones_Data(), Table_SourceData_ClimateZones[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="5" xr3:uid="{B8CB7CAF-BA1F-405C-A3B9-7EE8AC22A7AC}" name="Elevation" totalsRowDxfId="13" totalsRowCellStyle="Content bold">
-      <calculatedColumnFormula array="1">InputFunctions_Utilities.Utility_DisplayArrayInTable(SourceData_Common.SourceData_Common_ClimateZones_Data(), Table_SourceData_ClimateZones[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
+    <tableColumn id="5" xr3:uid="{CB8E024E-D313-4C2D-B662-87F82486AB46}" name="Elevation" totalsRowDxfId="13" totalsRowCellStyle="Content bold">
+      <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_ClimateZones_Data(), Table_SourceData_ClimateZones[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="6" xr3:uid="{638398A3-9C3E-4C73-8D73-A0F308FE488E}" name="MAP:PET" totalsRowDxfId="12" totalsRowCellStyle="Content bold">
-      <calculatedColumnFormula array="1">InputFunctions_Utilities.Utility_DisplayArrayInTable(SourceData_Common.SourceData_Common_ClimateZones_Data(), Table_SourceData_ClimateZones[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
+    <tableColumn id="6" xr3:uid="{B8680258-7B8E-4065-9919-C817ABC192DB}" name="MAP:PET" totalsRowDxfId="12" totalsRowCellStyle="Content bold">
+      <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_ClimateZones_Data(), Table_SourceData_ClimateZones[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="7" xr3:uid="{05CE54D0-9014-4670-99F1-E324A16D94DE}" name="Min temp" totalsRowDxfId="11" totalsRowCellStyle="Content bold">
-      <calculatedColumnFormula array="1">InputFunctions_Utilities.Utility_DisplayArrayInTable(SourceData_Common.SourceData_Common_ClimateZones_Data(), Table_SourceData_ClimateZones[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
+    <tableColumn id="7" xr3:uid="{D566E839-40A6-45F8-A27A-903F8E28119B}" name="Min temp" totalsRowDxfId="11" totalsRowCellStyle="Content bold">
+      <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_ClimateZones_Data(), Table_SourceData_ClimateZones[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="8" xr3:uid="{2CB0184B-3F70-4F6A-95F6-6F2E9492F09A}" name="Max temp" totalsRowDxfId="10" totalsRowCellStyle="Content bold">
-      <calculatedColumnFormula array="1">InputFunctions_Utilities.Utility_DisplayArrayInTable(SourceData_Common.SourceData_Common_ClimateZones_Data(), Table_SourceData_ClimateZones[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
+    <tableColumn id="8" xr3:uid="{C3BED548-D2DC-484C-A3E3-D473E29A0F40}" name="Max temp" totalsRowDxfId="10" totalsRowCellStyle="Content bold">
+      <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_ClimateZones_Data(), Table_SourceData_ClimateZones[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="9" xr3:uid="{7F3184EE-4EC3-458E-AAFB-DB279F02C494}" name="Min rainfall" totalsRowDxfId="9" totalsRowCellStyle="Content bold">
-      <calculatedColumnFormula array="1">InputFunctions_Utilities.Utility_DisplayArrayInTable(SourceData_Common.SourceData_Common_ClimateZones_Data(), Table_SourceData_ClimateZones[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
+    <tableColumn id="9" xr3:uid="{ABFA4E14-3EFF-4B09-9163-389BA2CD0048}" name="Min rainfall" totalsRowDxfId="9" totalsRowCellStyle="Content bold">
+      <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_ClimateZones_Data(), Table_SourceData_ClimateZones[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="10" xr3:uid="{2466BB77-E1A0-4018-A3CF-2C0CC0466491}" name="Max rainfall" totalsRowDxfId="8" totalsRowCellStyle="Content bold">
-      <calculatedColumnFormula array="1">InputFunctions_Utilities.Utility_DisplayArrayInTable(SourceData_Common.SourceData_Common_ClimateZones_Data(), Table_SourceData_ClimateZones[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
+    <tableColumn id="10" xr3:uid="{82CF3AA9-82DF-4E8C-95D8-383DCA73B8E3}" name="Max rainfall" totalsRowDxfId="8" totalsRowCellStyle="Content bold">
+      <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_ClimateZones_Data(), Table_SourceData_ClimateZones[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="11" xr3:uid="{0F0EFB18-D235-42F9-8CFF-00C67495994A}" name="Min frost days" totalsRowDxfId="7" totalsRowCellStyle="Content bold">
-      <calculatedColumnFormula array="1">InputFunctions_Utilities.Utility_DisplayArrayInTable(SourceData_Common.SourceData_Common_ClimateZones_Data(), Table_SourceData_ClimateZones[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
+    <tableColumn id="11" xr3:uid="{55BCA9BE-1159-4A67-A5AF-0F536700B79E}" name="Min frost days" totalsRowDxfId="7" totalsRowCellStyle="Content bold">
+      <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_ClimateZones_Data(), Table_SourceData_ClimateZones[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="15" xr3:uid="{44DE5C86-B4DC-4280-82BA-D5DC51D3D97F}" name="Max frost days" totalsRowDxfId="6" totalsRowCellStyle="Content bold">
-      <calculatedColumnFormula array="1">InputFunctions_Utilities.Utility_DisplayArrayInTable(SourceData_Common.SourceData_Common_ClimateZones_Data(), Table_SourceData_ClimateZones[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
+    <tableColumn id="15" xr3:uid="{B6BE0FB2-9310-4EED-BE2B-DF6EDC7FB16A}" name="Max frost days" totalsRowDxfId="6" totalsRowCellStyle="Content bold">
+      <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_ClimateZones_Data(), Table_SourceData_ClimateZones[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="12" xr3:uid="{C682AF37-CAEC-4E35-81E8-C6AB50735245}" name="Min elevation" totalsRowDxfId="5" totalsRowCellStyle="Content bold">
-      <calculatedColumnFormula array="1">InputFunctions_Utilities.Utility_DisplayArrayInTable(SourceData_Common.SourceData_Common_ClimateZones_Data(), Table_SourceData_ClimateZones[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
+    <tableColumn id="12" xr3:uid="{297E9969-647C-4F5F-9784-5E9CAA919D1D}" name="Min elevation" totalsRowDxfId="5" totalsRowCellStyle="Content bold">
+      <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_ClimateZones_Data(), Table_SourceData_ClimateZones[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="16" xr3:uid="{3B35E945-FFA7-4785-B1EB-DE4BD0488436}" name="Max elevation" totalsRowDxfId="4" totalsRowCellStyle="Content bold">
-      <calculatedColumnFormula array="1">InputFunctions_Utilities.Utility_DisplayArrayInTable(SourceData_Common.SourceData_Common_ClimateZones_Data(), Table_SourceData_ClimateZones[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
+    <tableColumn id="16" xr3:uid="{CC3A75C9-813A-4CAD-9C83-E7324450F9DB}" name="Max elevation" totalsRowDxfId="4" totalsRowCellStyle="Content bold">
+      <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_ClimateZones_Data(), Table_SourceData_ClimateZones[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="13" xr3:uid="{5999F275-917F-4A04-98ED-E40FD63B6DB6}" name="Min MAP:PET" totalsRowDxfId="3" totalsRowCellStyle="Content bold">
-      <calculatedColumnFormula array="1">InputFunctions_Utilities.Utility_DisplayArrayInTable(SourceData_Common.SourceData_Common_ClimateZones_Data(), Table_SourceData_ClimateZones[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
+    <tableColumn id="13" xr3:uid="{92CCD05C-2CE4-4A45-B22F-316F9E8A4294}" name="Min MAP:PET" totalsRowDxfId="3" totalsRowCellStyle="Content bold">
+      <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_ClimateZones_Data(), Table_SourceData_ClimateZones[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="17" xr3:uid="{94F10080-9531-4F63-AD9E-ED0BE040D333}" name="Max MAP:PET" totalsRowDxfId="2" totalsRowCellStyle="Content bold">
-      <calculatedColumnFormula array="1">InputFunctions_Utilities.Utility_DisplayArrayInTable(SourceData_Common.SourceData_Common_ClimateZones_Data(), Table_SourceData_ClimateZones[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
+    <tableColumn id="17" xr3:uid="{78DAEF96-486C-4AF9-B29C-89ACF0044AC2}" name="Max MAP:PET" totalsRowDxfId="2" totalsRowCellStyle="Content bold">
+      <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_ClimateZones_Data(), Table_SourceData_ClimateZones[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
   <tableStyleInfo name="Equation table" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
@@ -1868,17 +1960,17 @@
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="51" xr:uid="{3597E019-B21E-4B76-BCC8-D02D497BCFA9}" name="Table_SourceData_WetDryZones" displayName="Table_SourceData_WetDryZones" ref="D63:E77" totalsRowShown="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="18" xr:uid="{CE5AF498-03AE-41D0-840D-C52401CE2071}" name="Table_SourceData_WetDryZones" displayName="Table_SourceData_WetDryZones" ref="D63:E77" totalsRowShown="0">
   <autoFilter ref="D63:E77" xr:uid="{3597E019-B21E-4B76-BCC8-D02D497BCFA9}">
     <filterColumn colId="0" hiddenButton="1"/>
     <filterColumn colId="1" hiddenButton="1"/>
   </autoFilter>
   <tableColumns count="2">
-    <tableColumn id="1" xr3:uid="{2730A065-413F-4034-BFED-94FC80ACEF7C}" name="Climate zone" totalsRowCellStyle="Content bold">
-      <calculatedColumnFormula array="1">InputFunctions_Utilities.Utility_DisplayArrayInTable(SourceData_Common.SourceData_Common_WetAndDryZones_Data(), Table_SourceData_WetDryZones[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
+    <tableColumn id="1" xr3:uid="{19694A92-0DEE-4A6E-BC51-982D6E854911}" name="Climate zone" totalsRowCellStyle="Content bold">
+      <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_WetAndDryZones_Data(), Table_SourceData_WetDryZones[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{15428E11-9167-40B3-A71A-9D0BF558F1BE}" name="Wet or Dry Zone" totalsRowDxfId="1" totalsRowCellStyle="Content bold">
-      <calculatedColumnFormula array="1">InputFunctions_Utilities.Utility_DisplayArrayInTable(SourceData_Common.SourceData_Common_WetAndDryZones_Data(), Table_SourceData_WetDryZones[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
+    <tableColumn id="2" xr3:uid="{D0A70713-973B-422D-918B-ABC10BCB175D}" name="Wet or Dry Zone" totalsRowDxfId="1" totalsRowCellStyle="Content bold">
+      <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_WetAndDryZones_Data(), Table_SourceData_WetDryZones[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
   <tableStyleInfo name="Equation table" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
@@ -1886,7 +1978,7 @@
 </file>
 
 <file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="54" xr:uid="{AB16FEAB-AB03-45E1-BBD4-66D29CD412DF}" name="Table_SourceData_TemperatureZones" displayName="Table_SourceData_TemperatureZones" ref="D109:G112" totalsRowShown="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="19" xr:uid="{50B17EFA-36F5-4688-90AC-4736DA174794}" name="Table_SourceData_TemperatureZones" displayName="Table_SourceData_TemperatureZones" ref="D109:G112" totalsRowShown="0">
   <autoFilter ref="D109:G112" xr:uid="{AB16FEAB-AB03-45E1-BBD4-66D29CD412DF}">
     <filterColumn colId="0" hiddenButton="1"/>
     <filterColumn colId="1" hiddenButton="1"/>
@@ -1894,17 +1986,17 @@
     <filterColumn colId="3" hiddenButton="1"/>
   </autoFilter>
   <tableColumns count="4">
-    <tableColumn id="1" xr3:uid="{96C3C322-2156-4255-AAB2-50D379E8314F}" name="Temperature Zone">
-      <calculatedColumnFormula array="1">InputFunctions_Utilities.Utility_DisplayArrayInTable(SourceData_Common.SourceData_Common_TemperatureZones_Data(),Table_SourceData_TemperatureZones[[#Headers],[Temperature Zone]],0)</calculatedColumnFormula>
+    <tableColumn id="1" xr3:uid="{39A3E798-B6F6-4E8D-8F88-A99C8EA054AF}" name="Temperature Zone">
+      <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_TemperatureZones_Data(),Table_SourceData_TemperatureZones[[#Headers],[Temperature Zone]],0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{439934D3-101E-4FFD-B79E-1CF004533D9F}" name="MAT">
-      <calculatedColumnFormula array="1">InputFunctions_Utilities.Utility_DisplayArrayInTable(SourceData_Common.SourceData_Common_TemperatureZones_Data(),Table_SourceData_TemperatureZones[[#Headers],[Temperature Zone]],0)</calculatedColumnFormula>
+    <tableColumn id="2" xr3:uid="{716FBAFC-9EF8-4F89-8B6A-9456ED64AB2A}" name="MAT">
+      <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_TemperatureZones_Data(),Table_SourceData_TemperatureZones[[#Headers],[Temperature Zone]],0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="3" xr3:uid="{B9C6925C-8859-447A-9033-026808DCCFDE}" name="Min MAT">
-      <calculatedColumnFormula array="1">InputFunctions_Utilities.Utility_DisplayArrayInTable(SourceData_Common.SourceData_Common_TemperatureZones_Data(),Table_SourceData_TemperatureZones[[#Headers],[Temperature Zone]],0)</calculatedColumnFormula>
+    <tableColumn id="3" xr3:uid="{8EBDDF1B-E2B1-469E-9A0F-3097B9182F3D}" name="Min MAT">
+      <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_TemperatureZones_Data(),Table_SourceData_TemperatureZones[[#Headers],[Temperature Zone]],0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="4" xr3:uid="{A71D2833-8D0B-4018-ADB5-A980B546381D}" name="Max MAT">
-      <calculatedColumnFormula array="1">InputFunctions_Utilities.Utility_DisplayArrayInTable(SourceData_Common.SourceData_Common_TemperatureZones_Data(),Table_SourceData_TemperatureZones[[#Headers],[Temperature Zone]],0)</calculatedColumnFormula>
+    <tableColumn id="4" xr3:uid="{4D6211F2-492C-4681-BEDD-4CF0E003C60C}" name="Max MAT">
+      <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_TemperatureZones_Data(),Table_SourceData_TemperatureZones[[#Headers],[Temperature Zone]],0)</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
   <tableStyleInfo name="Equation table" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
@@ -1912,7 +2004,7 @@
 </file>
 
 <file path=xl/tables/table8.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="52" xr:uid="{E08772F3-2E8C-40A8-B755-08A5BBDF4130}" name="Table_SourceData_RainfallZones" displayName="Table_SourceData_RainfallZones" ref="D119:G121" totalsRowShown="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="20" xr:uid="{4D9D7934-770E-4FA0-B3A9-313B4333ABCE}" name="Table_SourceData_RainfallZones" displayName="Table_SourceData_RainfallZones" ref="D119:G121" totalsRowShown="0">
   <autoFilter ref="D119:G121" xr:uid="{E08772F3-2E8C-40A8-B755-08A5BBDF4130}">
     <filterColumn colId="0" hiddenButton="1"/>
     <filterColumn colId="1" hiddenButton="1"/>
@@ -1920,17 +2012,17 @@
     <filterColumn colId="3" hiddenButton="1"/>
   </autoFilter>
   <tableColumns count="4">
-    <tableColumn id="1" xr3:uid="{8D528D96-99E0-4B73-862C-72B864EE99DC}" name="Rainfall Zone">
-      <calculatedColumnFormula array="1">InputFunctions_Utilities.Utility_DisplayArrayInTable(SourceData_Common.SourceData_Common_RainfallZones_Data(),Table_SourceData_RainfallZones[[#Headers],[Rainfall Zone]],0)</calculatedColumnFormula>
+    <tableColumn id="1" xr3:uid="{A2B3A07F-70DF-4FBB-BED6-38DB0B294353}" name="Rainfall Zone">
+      <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_RainfallZones_Data(),Table_SourceData_RainfallZones[[#Headers],[Rainfall Zone]],0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{4CBBC8D3-E963-45E4-9BC9-FC10B677B877}" name="Annual rainfall">
-      <calculatedColumnFormula array="1">InputFunctions_Utilities.Utility_DisplayArrayInTable(SourceData_Common.SourceData_Common_RainfallZones_Data(),Table_SourceData_RainfallZones[[#Headers],[Rainfall Zone]],0)</calculatedColumnFormula>
+    <tableColumn id="2" xr3:uid="{D0314575-5F75-4E7F-BCDF-E543D94DBE99}" name="Annual rainfall">
+      <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_RainfallZones_Data(),Table_SourceData_RainfallZones[[#Headers],[Rainfall Zone]],0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="3" xr3:uid="{956E7C3A-DE83-4483-B43E-C6D4A7BC4BC1}" name="Min rainfall">
-      <calculatedColumnFormula array="1">InputFunctions_Utilities.Utility_DisplayArrayInTable(SourceData_Common.SourceData_Common_RainfallZones_Data(),Table_SourceData_RainfallZones[[#Headers],[Rainfall Zone]],0)</calculatedColumnFormula>
+    <tableColumn id="3" xr3:uid="{E8EC7B10-93C4-4C08-A0A5-221C22CABCE2}" name="Min rainfall">
+      <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_RainfallZones_Data(),Table_SourceData_RainfallZones[[#Headers],[Rainfall Zone]],0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="4" xr3:uid="{5797AA9E-22BA-4D6A-A09F-C98233F711CE}" name="Max rainfall">
-      <calculatedColumnFormula array="1">InputFunctions_Utilities.Utility_DisplayArrayInTable(SourceData_Common.SourceData_Common_RainfallZones_Data(),Table_SourceData_RainfallZones[[#Headers],[Rainfall Zone]],0)</calculatedColumnFormula>
+    <tableColumn id="4" xr3:uid="{132159D6-AB45-4D4A-B6E2-FCBD4D3AAA39}" name="Max rainfall">
+      <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_RainfallZones_Data(),Table_SourceData_RainfallZones[[#Headers],[Rainfall Zone]],0)</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
   <tableStyleInfo name="Equation table" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
@@ -1938,17 +2030,17 @@
 </file>
 
 <file path=xl/tables/table9.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="53" xr:uid="{A159E140-02ED-4547-B6E1-6695D8B16A11}" name="Table_SourceData_LeachingZones" displayName="Table_SourceData_LeachingZones" ref="D127:E129" totalsRowShown="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="21" xr:uid="{CB2DE042-FB5F-4D99-A8D1-0CF6E232CFF8}" name="Table_SourceData_LeachingZones" displayName="Table_SourceData_LeachingZones" ref="D127:E129" totalsRowShown="0">
   <autoFilter ref="D127:E129" xr:uid="{A159E140-02ED-4547-B6E1-6695D8B16A11}">
     <filterColumn colId="0" hiddenButton="1"/>
     <filterColumn colId="1" hiddenButton="1"/>
   </autoFilter>
   <tableColumns count="2">
-    <tableColumn id="1" xr3:uid="{848865A1-4E92-40ED-B0C2-5BFD4E72D24A}" name="Leaching Zone">
-      <calculatedColumnFormula array="1">InputFunctions_Utilities.Utility_DisplayArrayInTable(SourceData_Common.SourceData_Common_LeachingZones_Data(), Table_SourceData_LeachingZones[[#Headers],[Leaching Zone]], 0)</calculatedColumnFormula>
+    <tableColumn id="1" xr3:uid="{F0D5BDD2-F81C-4E8F-B8B5-0CC8BEDBC472}" name="Leaching Zone">
+      <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_LeachingZones_Data(), Table_SourceData_LeachingZones[[#Headers],[Leaching Zone]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{549D2E4C-1B28-48F1-94DE-5374E4E37B32}" name="Leaching criteria">
-      <calculatedColumnFormula array="1">InputFunctions_Utilities.Utility_DisplayArrayInTable(SourceData_Common.SourceData_Common_LeachingZones_Data(), Table_SourceData_LeachingZones[[#Headers],[Leaching Zone]], 0)</calculatedColumnFormula>
+    <tableColumn id="2" xr3:uid="{34942F55-5E31-4A20-9926-1B41D505AAD4}" name="Leaching criteria">
+      <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_LeachingZones_Data(), Table_SourceData_LeachingZones[[#Headers],[Leaching Zone]], 0)</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
   <tableStyleInfo name="Equation table" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
@@ -2209,9 +2301,8 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{41C7EF23-0CE2-4D86-AA37-C6D78B995C56}">
-  <sheetPr codeName="Sheet2"/>
-  <dimension ref="A1:BX179"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2A280EEB-088F-4A37-9670-186703ED1DFE}">
+  <dimension ref="A1:BX196"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="30.7109375" style="6" customWidth="1"/>
@@ -3718,24 +3809,24 @@
       </c>
       <c r="BM115" s="6"/>
     </row>
-    <row r="116" spans="4:65" x14ac:dyDescent="0.25">
+    <row r="116" spans="4:65" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D116" s="4" t="str" cm="1">
         <f t="array" ref="D116">Common_SourceData.Common_SourceData_RainfallZones_Source()</f>
         <v>VEERG 2026: Table 1.3: Climate and Rainfall zone classifications and definitions</v>
       </c>
       <c r="BM116" s="6"/>
     </row>
-    <row r="117" spans="4:65" x14ac:dyDescent="0.25">
+    <row r="117" spans="4:65" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D117" s="13" t="str" cm="1">
         <f t="array" ref="D117">"⚠️" &amp; Common_SourceData.Common_SourceData_RainfallZones_Variation()</f>
         <v>⚠️VARIATION OF SOURCE DATA: Added extra Rainfall min and Rainfall max columns to calculate zone from real rainfall data.</v>
       </c>
       <c r="BM117" s="6"/>
     </row>
-    <row r="118" spans="4:65" x14ac:dyDescent="0.25">
+    <row r="118" spans="4:65" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="BM118" s="6"/>
     </row>
-    <row r="119" spans="4:65" x14ac:dyDescent="0.25">
+    <row r="119" spans="4:65" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D119" s="11" t="s">
         <v>30</v>
       </c>
@@ -3750,7 +3841,7 @@
       </c>
       <c r="BM119" s="6"/>
     </row>
-    <row r="120" spans="4:65" x14ac:dyDescent="0.25">
+    <row r="120" spans="4:65" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D120" s="11" t="str" cm="1">
         <f t="array" ref="D120">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_RainfallZones_Data(),Table_SourceData_RainfallZones[[#Headers],[Rainfall Zone]],0)</f>
         <v>High rainfall</v>
@@ -3769,7 +3860,7 @@
       </c>
       <c r="BM120" s="6"/>
     </row>
-    <row r="121" spans="4:65" x14ac:dyDescent="0.25">
+    <row r="121" spans="4:65" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D121" s="11" t="str" cm="1">
         <f t="array" ref="D121">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_RainfallZones_Data(),Table_SourceData_RainfallZones[[#Headers],[Rainfall Zone]],0)</f>
         <v>Low rainfall</v>
@@ -3788,22 +3879,24 @@
       </c>
       <c r="BM121" s="6"/>
     </row>
-    <row r="122" spans="4:65" x14ac:dyDescent="0.25">
+    <row r="122" spans="4:65" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="BM122" s="6"/>
     </row>
-    <row r="124" spans="4:65" ht="23.25" x14ac:dyDescent="0.25">
+    <row r="123" spans="4:65" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="124" spans="4:65" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D124" s="5" t="str" cm="1">
         <f t="array" ref="D124">Common_SourceData.Common_SourceData_LeachingZones_Title()</f>
         <v>VEERG Australian leaching zones</v>
       </c>
     </row>
-    <row r="125" spans="4:65" x14ac:dyDescent="0.25">
+    <row r="125" spans="4:65" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D125" s="4" t="str" cm="1">
         <f t="array" ref="D125">Common_SourceData.Common_SourceData_LeachingZones_Source()</f>
         <v>VEERG 2026: Table 1.3: Climate and Rainfall zone classifications and definitions</v>
       </c>
     </row>
-    <row r="127" spans="4:65" x14ac:dyDescent="0.25">
+    <row r="126" spans="4:65" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="127" spans="4:65" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D127" s="11" t="s">
         <v>32</v>
       </c>
@@ -3811,7 +3904,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="128" spans="4:65" x14ac:dyDescent="0.25">
+    <row r="128" spans="4:65" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D128" s="11" t="str" cm="1">
         <f t="array" ref="D128">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_LeachingZones_Data(), Table_SourceData_LeachingZones[[#Headers],[Leaching Zone]], 0)</f>
         <v>Leaching occurs</v>
@@ -3821,7 +3914,7 @@
         <v>Σ(𝑟𝑎𝑖𝑛)&gt;Σ(𝐸𝑇0)+𝑠𝑜𝑖𝑙 𝑤𝑎𝑡𝑒𝑟 ℎ𝑜𝑙𝑑𝑖𝑛𝑔 𝑐𝑎𝑝𝑎𝑐𝑖𝑡𝑦</v>
       </c>
     </row>
-    <row r="129" spans="4:76" x14ac:dyDescent="0.25">
+    <row r="129" spans="4:76" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D129" s="11" t="str" cm="1">
         <f t="array" ref="D129">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_LeachingZones_Data(), Table_SourceData_LeachingZones[[#Headers],[Leaching Zone]], 0)</f>
         <v>Leaching does not occur</v>
@@ -3831,21 +3924,23 @@
         <v>Σ(𝑟𝑎𝑖𝑛)≤Σ(𝐸𝑇0)+𝑠𝑜𝑖𝑙 𝑤𝑎𝑡𝑒𝑟 ℎ𝑜𝑙𝑑𝑖𝑛𝑔 𝑐𝑎𝑝𝑎𝑐𝑖𝑡𝑦</v>
       </c>
     </row>
-    <row r="132" spans="4:76" ht="23.25" x14ac:dyDescent="0.25">
+    <row r="130" spans="4:76" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="131" spans="4:76" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="132" spans="4:76" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D132" s="5" t="str" cm="1">
         <f t="array" ref="D132">Common_SourceData.Common_SourceData_FracWET_Title()</f>
         <v>Fraction of N that is available for leaching and runoff</v>
       </c>
       <c r="E132" s="10"/>
     </row>
-    <row r="133" spans="4:76" x14ac:dyDescent="0.25">
+    <row r="133" spans="4:76" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D133" s="4" t="str" cm="1">
         <f t="array" ref="D133">Common_SourceData.Common_SourceData_FracWET_Source()</f>
         <v>VEERG 2026:5.5.2.3 Constant Parameters</v>
       </c>
       <c r="E133" s="10"/>
     </row>
-    <row r="134" spans="4:76" x14ac:dyDescent="0.25">
+    <row r="134" spans="4:76" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D134" t="s">
         <v>37</v>
       </c>
@@ -3853,7 +3948,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="135" spans="4:76" x14ac:dyDescent="0.25">
+    <row r="135" spans="4:76" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D135" t="str" cm="1">
         <f t="array" ref="D135">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_FracWET_Data(),Table_SourceData_FracWET[[#Headers],[Is in leaching zone]],0)</f>
         <v>Yes - in leaching zone</v>
@@ -3863,7 +3958,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="136" spans="4:76" x14ac:dyDescent="0.25">
+    <row r="136" spans="4:76" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D136" s="1" t="str" cm="1">
         <f t="array" ref="D136">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_FracWET_Data(),Table_SourceData_FracWET[[#Headers],[Is in leaching zone]],0)</f>
         <v>No - not in leaching zone</v>
@@ -3873,7 +3968,8 @@
         <v>0</v>
       </c>
     </row>
-    <row r="138" spans="4:76" x14ac:dyDescent="0.25">
+    <row r="137" spans="4:76" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="138" spans="4:76" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="BM138" s="6"/>
       <c r="BN138" s="6"/>
       <c r="BO138" s="6"/>
@@ -3887,7 +3983,7 @@
       <c r="BW138" s="6"/>
       <c r="BX138" s="6"/>
     </row>
-    <row r="139" spans="4:76" ht="23.25" x14ac:dyDescent="0.25">
+    <row r="139" spans="4:76" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D139" s="5" t="str" cm="1">
         <f t="array" ref="D139">Common_SourceData.Common_SourceData_DataScores_Scope3_Title()</f>
         <v>Australian data scores for scope 3</v>
@@ -3905,7 +4001,7 @@
       <c r="BW139" s="6"/>
       <c r="BX139" s="6"/>
     </row>
-    <row r="140" spans="4:76" x14ac:dyDescent="0.25">
+    <row r="140" spans="4:76" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D140" s="4" t="str" cm="1">
         <f t="array" ref="D140">Common_SourceData.Common_SourceData_DataScores_Scope3_Source()</f>
         <v>VEERG 2026: XXXXXXXX</v>
@@ -3923,10 +4019,10 @@
       <c r="BW140" s="6"/>
       <c r="BX140" s="6"/>
     </row>
-    <row r="141" spans="4:76" x14ac:dyDescent="0.25">
+    <row r="141" spans="4:76" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="BM141" s="6"/>
     </row>
-    <row r="142" spans="4:76" x14ac:dyDescent="0.25">
+    <row r="142" spans="4:76" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D142" s="11" t="s">
         <v>34</v>
       </c>
@@ -3935,7 +4031,7 @@
       </c>
       <c r="BM142" s="6"/>
     </row>
-    <row r="143" spans="4:76" x14ac:dyDescent="0.25">
+    <row r="143" spans="4:76" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D143" s="11" t="str" cm="1">
         <f t="array" ref="D143">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_DataScores_Scope3_Data(), Table_SourceData_DataScores_Scope3[[#Headers],[Data source]], 0)</f>
         <v>International scope 3 database</v>
@@ -3946,7 +4042,7 @@
       </c>
       <c r="BM143" s="6"/>
     </row>
-    <row r="144" spans="4:76" x14ac:dyDescent="0.25">
+    <row r="144" spans="4:76" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D144" s="11" t="str" cm="1">
         <f t="array" ref="D144">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_DataScores_Scope3_Data(), Table_SourceData_DataScores_Scope3[[#Headers],[Data source]], 0)</f>
         <v>Australian scope 3 database</v>
@@ -3957,7 +4053,7 @@
       </c>
       <c r="BM144" s="6"/>
     </row>
-    <row r="145" spans="4:65" x14ac:dyDescent="0.25">
+    <row r="145" spans="4:65" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D145" s="11" t="str" cm="1">
         <f t="array" ref="D145">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_DataScores_Scope3_Data(), Table_SourceData_DataScores_Scope3[[#Headers],[Data source]], 0)</f>
         <v>State or regional scope 3 database</v>
@@ -3968,7 +4064,7 @@
       </c>
       <c r="BM145" s="6"/>
     </row>
-    <row r="146" spans="4:65" x14ac:dyDescent="0.25">
+    <row r="146" spans="4:65" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D146" s="11" t="str" cm="1">
         <f t="array" ref="D146">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_DataScores_Scope3_Data(), Table_SourceData_DataScores_Scope3[[#Headers],[Data source]], 0)</f>
         <v>Emissions intensity calculated from approved method</v>
@@ -3979,7 +4075,7 @@
       </c>
       <c r="BM146" s="6"/>
     </row>
-    <row r="147" spans="4:65" x14ac:dyDescent="0.25">
+    <row r="147" spans="4:65" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D147" s="11" t="str" cm="1">
         <f t="array" ref="D147">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_DataScores_Scope3_Data(), Table_SourceData_DataScores_Scope3[[#Headers],[Data source]], 0)</f>
         <v>Verified credential matching ISO14067</v>
@@ -3990,13 +4086,13 @@
       </c>
       <c r="BM147" s="6"/>
     </row>
-    <row r="148" spans="4:65" x14ac:dyDescent="0.25">
+    <row r="148" spans="4:65" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="BM148" s="6"/>
     </row>
-    <row r="149" spans="4:65" x14ac:dyDescent="0.25">
+    <row r="149" spans="4:65" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="BM149" s="6"/>
     </row>
-    <row r="150" spans="4:65" ht="23.25" x14ac:dyDescent="0.25">
+    <row r="150" spans="4:65" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D150" s="5" t="str" cm="1">
         <f t="array" ref="D150">Common_SourceData.Common_SourceData_FracLEACH_Title()</f>
         <v>Fraction of N that is available for leaching and runoff</v>
@@ -4004,7 +4100,7 @@
       <c r="E150" s="10"/>
       <c r="BM150" s="6"/>
     </row>
-    <row r="151" spans="4:65" x14ac:dyDescent="0.25">
+    <row r="151" spans="4:65" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D151" s="4" t="str" cm="1">
         <f t="array" ref="D151">Common_SourceData.Common_SourceData_FracLEACH_Source()</f>
         <v>VEERG 2026:5.5.2.3 Constant Parameters</v>
@@ -4012,7 +4108,7 @@
       <c r="E151" s="10"/>
       <c r="BM151" s="6"/>
     </row>
-    <row r="152" spans="4:65" x14ac:dyDescent="0.25">
+    <row r="152" spans="4:65" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D152" s="4" t="str" cm="1">
         <f t="array" ref="D152">Common_SourceData.Common_SourceData_FracLEACH_NIRReference()</f>
         <v>National Inventory Report Volume 1: Leaching and runoff (3.D.b.2)</v>
@@ -4020,7 +4116,7 @@
       <c r="E152" s="10"/>
       <c r="BM152" s="6"/>
     </row>
-    <row r="153" spans="4:65" x14ac:dyDescent="0.25">
+    <row r="153" spans="4:65" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D153" s="10" t="str" cm="1">
         <f t="array" ref="D153:E153">Common_SourceData.Common_SourceData_FracLEACH_Data()</f>
         <v>FracLEACH</v>
@@ -4040,7 +4136,7 @@
       <c r="BK153" s="2"/>
       <c r="BL153" s="2"/>
     </row>
-    <row r="154" spans="4:65" x14ac:dyDescent="0.25">
+    <row r="154" spans="4:65" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="BB154" s="2"/>
       <c r="BC154" s="2"/>
       <c r="BD154" s="2"/>
@@ -4053,7 +4149,7 @@
       <c r="BK154" s="2"/>
       <c r="BL154" s="2"/>
     </row>
-    <row r="155" spans="4:65" x14ac:dyDescent="0.25">
+    <row r="155" spans="4:65" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="BB155" s="2"/>
       <c r="BC155" s="2"/>
       <c r="BD155" s="2"/>
@@ -4066,25 +4162,25 @@
       <c r="BK155" s="2"/>
       <c r="BL155" s="2"/>
     </row>
-    <row r="156" spans="4:65" ht="23.25" x14ac:dyDescent="0.25">
+    <row r="156" spans="4:65" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D156" s="5" t="str" cm="1">
         <f t="array" ref="D156">Common_SourceData.Common_SourceData_EFleach_Title()</f>
         <v>Emission factor for nitrogen leaching and runoff</v>
       </c>
     </row>
-    <row r="157" spans="4:65" x14ac:dyDescent="0.25">
+    <row r="157" spans="4:65" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D157" s="4" t="str" cm="1">
         <f t="array" ref="D157">Common_SourceData.Common_SourceData_EFleach_Source()</f>
         <v>VEERG 2026:5.5.2.3 Constant Parameters</v>
       </c>
     </row>
-    <row r="158" spans="4:65" x14ac:dyDescent="0.25">
+    <row r="158" spans="4:65" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D158" s="4" t="str" cm="1">
         <f t="array" ref="D158">Common_SourceData.Common_SourceData_EFleach_NIRReference()</f>
         <v>National Inventory Report Volume 1: Equation 3.D.B_10</v>
       </c>
     </row>
-    <row r="159" spans="4:65" x14ac:dyDescent="0.25">
+    <row r="159" spans="4:65" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D159" s="1" t="str" cm="1">
         <f t="array" ref="D159:E159">Common_SourceData.Common_SourceData_EFleach_Data()</f>
         <v>EFleach</v>
@@ -4093,19 +4189,21 @@
         <v>1.0999999999999999E-2</v>
       </c>
     </row>
-    <row r="162" spans="4:67" ht="23.25" x14ac:dyDescent="0.25">
+    <row r="160" spans="4:65" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="161" spans="4:67" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="162" spans="4:67" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D162" s="5" t="str" cm="1">
         <f t="array" ref="D162">Common_SourceData.Common_SourceData_DensityOfMethane_Title()</f>
         <v>p = density of methane</v>
       </c>
     </row>
-    <row r="163" spans="4:67" x14ac:dyDescent="0.25">
+    <row r="163" spans="4:67" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D163" s="4" t="str" cm="1">
         <f t="array" ref="D163">Common_SourceData.Common_SourceData_DensityOfMethane_Source()</f>
         <v>National Inventory Report 2023 Volume 1: Equations 3.B.1a_2, 3.B.1c_2, 3.B.3_1, 3.B.4g_2</v>
       </c>
     </row>
-    <row r="164" spans="4:67" x14ac:dyDescent="0.25">
+    <row r="164" spans="4:67" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D164" s="1" cm="1">
         <f t="array" ref="D164">Common_SourceData.Common_SourceData_DensityOfMethane_Data()</f>
         <v>0.6784</v>
@@ -4115,85 +4213,420 @@
         <v>kg/m3</v>
       </c>
     </row>
-    <row r="165" spans="4:67" x14ac:dyDescent="0.25">
+    <row r="165" spans="4:67" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="BM165" s="6"/>
       <c r="BN165" s="6"/>
       <c r="BO165" s="6"/>
     </row>
-    <row r="166" spans="4:67" x14ac:dyDescent="0.25">
+    <row r="166" spans="4:67" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="BM166" s="6"/>
       <c r="BN166" s="6"/>
       <c r="BO166" s="6"/>
     </row>
-    <row r="167" spans="4:67" x14ac:dyDescent="0.25">
+    <row r="167" spans="4:67" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="D167" s="5" t="str" cm="1">
+        <f t="array" ref="D167">Common_SourceData.Common_SourceData_EFN2O_Title()</f>
+        <v>Nitrous oxide emission factors for inorganic fertiliser application</v>
+      </c>
       <c r="BM167" s="6"/>
       <c r="BN167" s="6"/>
       <c r="BO167" s="6"/>
     </row>
-    <row r="168" spans="4:67" x14ac:dyDescent="0.25">
+    <row r="168" spans="4:67" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="D168" s="4" t="str" cm="1">
+        <f t="array" ref="D168">Common_SourceData.Common_SourceData_EFN2O_Source()</f>
+        <v>VEERG 2026: Table A.2.2.1</v>
+      </c>
       <c r="BM168" s="6"/>
       <c r="BN168" s="6"/>
       <c r="BO168" s="6"/>
     </row>
-    <row r="169" spans="4:67" x14ac:dyDescent="0.25">
+    <row r="169" spans="4:67" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="D169" s="12" t="str" cm="1">
+        <f t="array" ref="D169">Common_SourceData.Common_SourceData_EFN2O_Unit()</f>
+        <v>(kg N2O-N / kg N</v>
+      </c>
       <c r="BM169" s="6"/>
       <c r="BN169" s="6"/>
       <c r="BO169" s="6"/>
     </row>
-    <row r="170" spans="4:67" x14ac:dyDescent="0.25">
+    <row r="170" spans="4:67" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="D170" s="13" t="str" cm="1">
+        <f t="array" ref="D170:D173">Common_SourceData.Common_SourceData_EFN2O_Variation()</f>
+        <v>VARIATION OF SOURCE DATA:</v>
+      </c>
       <c r="BM170" s="6"/>
       <c r="BN170" s="6"/>
       <c r="BO170" s="6"/>
     </row>
-    <row r="171" spans="4:67" x14ac:dyDescent="0.25">
+    <row r="171" spans="4:67" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="D171" s="13" t="str">
+        <v>Removed duplicate 'Aquaculture' row.</v>
+      </c>
       <c r="BM171" s="6"/>
       <c r="BN171" s="6"/>
       <c r="BO171" s="6"/>
     </row>
-    <row r="172" spans="4:67" x14ac:dyDescent="0.25">
+    <row r="172" spans="4:67" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="D172" s="13" t="str">
+        <v>Removed asterisks to aid lookup.</v>
+      </c>
       <c r="BM172" s="6"/>
       <c r="BN172" s="6"/>
       <c r="BO172" s="6"/>
     </row>
-    <row r="173" spans="4:67" x14ac:dyDescent="0.25">
+    <row r="173" spans="4:67" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="D173" s="13" t="str">
+        <v>Added 'production system only', 'rainfall zone' and 'irrigation method' columns to aid lookup.</v>
+      </c>
       <c r="BM173" s="6"/>
       <c r="BN173" s="6"/>
       <c r="BO173" s="6"/>
     </row>
-    <row r="174" spans="4:67" x14ac:dyDescent="0.25">
+    <row r="174" spans="4:67" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="D174" s="13"/>
       <c r="BM174" s="6"/>
       <c r="BN174" s="6"/>
       <c r="BO174" s="6"/>
     </row>
-    <row r="175" spans="4:67" x14ac:dyDescent="0.25">
+    <row r="175" spans="4:67" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="D175" s="11" t="s">
+        <v>39</v>
+      </c>
+      <c r="E175" s="11" t="s">
+        <v>40</v>
+      </c>
+      <c r="F175" s="11" t="s">
+        <v>41</v>
+      </c>
+      <c r="G175" s="11" t="s">
+        <v>42</v>
+      </c>
+      <c r="H175" s="11" t="s">
+        <v>43</v>
+      </c>
+      <c r="J175" s="1" t="s">
+        <v>44</v>
+      </c>
       <c r="BM175" s="6"/>
       <c r="BN175" s="6"/>
       <c r="BO175" s="6"/>
     </row>
-    <row r="176" spans="4:67" x14ac:dyDescent="0.25">
+    <row r="176" spans="4:67" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="D176" s="11" t="str" cm="1">
+        <f t="array" ref="D176">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_EFN2O_Data(), Table_SourceData_Common_EFN2O[[#Headers],[Production system j]], 0)</f>
+        <v>Irrigated pasture</v>
+      </c>
+      <c r="E176" s="11" cm="1">
+        <f t="array" ref="E176">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_EFN2O_Data(), Table_SourceData_Common_EFN2O[[#Headers],[Production system j]], 0)</f>
+        <v>5.8999999999999999E-3</v>
+      </c>
+      <c r="F176" s="11" t="str" cm="1">
+        <f t="array" ref="F176">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_EFN2O_Data(), Table_SourceData_Common_EFN2O[[#Headers],[Production system j]], 0)</f>
+        <v>Pasture</v>
+      </c>
+      <c r="G176" s="11" t="str" cm="1">
+        <f t="array" ref="G176">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_EFN2O_Data(), Table_SourceData_Common_EFN2O[[#Headers],[Production system j]], 0)</f>
+        <v>Any</v>
+      </c>
+      <c r="H176" s="11" t="str" cm="1">
+        <f t="array" ref="H176">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_EFN2O_Data(), Table_SourceData_Common_EFN2O[[#Headers],[Production system j]], 0)</f>
+        <v>Any</v>
+      </c>
+      <c r="J176" s="1" t="s">
+        <v>45</v>
+      </c>
       <c r="BM176" s="6"/>
       <c r="BN176" s="6"/>
       <c r="BO176" s="6"/>
     </row>
-    <row r="177" spans="65:67" x14ac:dyDescent="0.25">
+    <row r="177" spans="4:67" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="D177" s="11" t="str" cm="1">
+        <f t="array" ref="D177">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_EFN2O_Data(), Table_SourceData_Common_EFN2O[[#Headers],[Production system j]], 0)</f>
+        <v>Irrigated crop</v>
+      </c>
+      <c r="E177" s="11" cm="1">
+        <f t="array" ref="E177">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_EFN2O_Data(), Table_SourceData_Common_EFN2O[[#Headers],[Production system j]], 0)</f>
+        <v>7.0000000000000001E-3</v>
+      </c>
+      <c r="F177" s="11" t="str" cm="1">
+        <f t="array" ref="F177">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_EFN2O_Data(), Table_SourceData_Common_EFN2O[[#Headers],[Production system j]], 0)</f>
+        <v>Crop</v>
+      </c>
+      <c r="G177" s="11" t="str" cm="1">
+        <f t="array" ref="G177">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_EFN2O_Data(), Table_SourceData_Common_EFN2O[[#Headers],[Production system j]], 0)</f>
+        <v>Any</v>
+      </c>
+      <c r="H177" s="11" t="str" cm="1">
+        <f t="array" ref="H177">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_EFN2O_Data(), Table_SourceData_Common_EFN2O[[#Headers],[Production system j]], 0)</f>
+        <v>Any</v>
+      </c>
+      <c r="J177" s="1" t="s">
+        <v>46</v>
+      </c>
       <c r="BM177" s="6"/>
       <c r="BN177" s="6"/>
       <c r="BO177" s="6"/>
     </row>
-    <row r="178" spans="65:67" x14ac:dyDescent="0.25">
+    <row r="178" spans="4:67" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="D178" s="11" t="str" cm="1">
+        <f t="array" ref="D178">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_EFN2O_Data(), Table_SourceData_Common_EFN2O[[#Headers],[Production system j]], 0)</f>
+        <v>Non-irrigated pasture</v>
+      </c>
+      <c r="E178" s="11" cm="1">
+        <f t="array" ref="E178">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_EFN2O_Data(), Table_SourceData_Common_EFN2O[[#Headers],[Production system j]], 0)</f>
+        <v>1.8E-3</v>
+      </c>
+      <c r="F178" s="11" t="str" cm="1">
+        <f t="array" ref="F178">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_EFN2O_Data(), Table_SourceData_Common_EFN2O[[#Headers],[Production system j]], 0)</f>
+        <v>Pasture</v>
+      </c>
+      <c r="G178" s="11" t="str" cm="1">
+        <f t="array" ref="G178">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_EFN2O_Data(), Table_SourceData_Common_EFN2O[[#Headers],[Production system j]], 0)</f>
+        <v>Not irrigated</v>
+      </c>
+      <c r="H178" s="11" t="str" cm="1">
+        <f t="array" ref="H178">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_EFN2O_Data(), Table_SourceData_Common_EFN2O[[#Headers],[Production system j]], 0)</f>
+        <v>Low rainfall</v>
+      </c>
       <c r="BM178" s="6"/>
       <c r="BN178" s="6"/>
       <c r="BO178" s="6"/>
     </row>
-    <row r="179" spans="65:67" x14ac:dyDescent="0.25">
+    <row r="179" spans="4:67" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="D179" s="11" t="str" cm="1">
+        <f t="array" ref="D179">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_EFN2O_Data(), Table_SourceData_Common_EFN2O[[#Headers],[Production system j]], 0)</f>
+        <v>Non-irrigated crop (low rainfall)</v>
+      </c>
+      <c r="E179" s="11" cm="1">
+        <f t="array" ref="E179">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_EFN2O_Data(), Table_SourceData_Common_EFN2O[[#Headers],[Production system j]], 0)</f>
+        <v>2.8999999999999998E-3</v>
+      </c>
+      <c r="F179" s="11" t="str" cm="1">
+        <f t="array" ref="F179">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_EFN2O_Data(), Table_SourceData_Common_EFN2O[[#Headers],[Production system j]], 0)</f>
+        <v>Crop</v>
+      </c>
+      <c r="G179" s="11" t="str" cm="1">
+        <f t="array" ref="G179">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_EFN2O_Data(), Table_SourceData_Common_EFN2O[[#Headers],[Production system j]], 0)</f>
+        <v>Not irrigated</v>
+      </c>
+      <c r="H179" s="11" t="str" cm="1">
+        <f t="array" ref="H179">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_EFN2O_Data(), Table_SourceData_Common_EFN2O[[#Headers],[Production system j]], 0)</f>
+        <v>Low rainfall</v>
+      </c>
       <c r="BM179" s="6"/>
       <c r="BN179" s="6"/>
       <c r="BO179" s="6"/>
     </row>
+    <row r="180" spans="4:67" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="D180" s="11" t="str" cm="1">
+        <f t="array" ref="D180">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_EFN2O_Data(), Table_SourceData_Common_EFN2O[[#Headers],[Production system j]], 0)</f>
+        <v>Non-irrigated crop (high rainfall)</v>
+      </c>
+      <c r="E180" s="11" cm="1">
+        <f t="array" ref="E180">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_EFN2O_Data(), Table_SourceData_Common_EFN2O[[#Headers],[Production system j]], 0)</f>
+        <v>8.0000000000000002E-3</v>
+      </c>
+      <c r="F180" s="11" t="str" cm="1">
+        <f t="array" ref="F180">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_EFN2O_Data(), Table_SourceData_Common_EFN2O[[#Headers],[Production system j]], 0)</f>
+        <v>Crop</v>
+      </c>
+      <c r="G180" s="11" t="str" cm="1">
+        <f t="array" ref="G180">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_EFN2O_Data(), Table_SourceData_Common_EFN2O[[#Headers],[Production system j]], 0)</f>
+        <v>Not irrigated</v>
+      </c>
+      <c r="H180" s="11" t="str" cm="1">
+        <f t="array" ref="H180">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_EFN2O_Data(), Table_SourceData_Common_EFN2O[[#Headers],[Production system j]], 0)</f>
+        <v>High rainfall</v>
+      </c>
+    </row>
+    <row r="181" spans="4:67" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="D181" s="11" t="str" cm="1">
+        <f t="array" ref="D181">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_EFN2O_Data(), Table_SourceData_Common_EFN2O[[#Headers],[Production system j]], 0)</f>
+        <v>Sugar</v>
+      </c>
+      <c r="E181" s="11" cm="1">
+        <f t="array" ref="E181">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_EFN2O_Data(), Table_SourceData_Common_EFN2O[[#Headers],[Production system j]], 0)</f>
+        <v>1.9900000000000001E-2</v>
+      </c>
+      <c r="F181" s="11" t="str" cm="1">
+        <f t="array" ref="F181">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_EFN2O_Data(), Table_SourceData_Common_EFN2O[[#Headers],[Production system j]], 0)</f>
+        <v>Sugar</v>
+      </c>
+      <c r="G181" s="11" t="str" cm="1">
+        <f t="array" ref="G181">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_EFN2O_Data(), Table_SourceData_Common_EFN2O[[#Headers],[Production system j]], 0)</f>
+        <v>Any</v>
+      </c>
+      <c r="H181" s="11" t="str" cm="1">
+        <f t="array" ref="H181">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_EFN2O_Data(), Table_SourceData_Common_EFN2O[[#Headers],[Production system j]], 0)</f>
+        <v>Any</v>
+      </c>
+    </row>
+    <row r="182" spans="4:67" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="D182" s="11" t="str" cm="1">
+        <f t="array" ref="D182">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_EFN2O_Data(), Table_SourceData_Common_EFN2O[[#Headers],[Production system j]], 0)</f>
+        <v>Cotton</v>
+      </c>
+      <c r="E182" s="11" cm="1">
+        <f t="array" ref="E182">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_EFN2O_Data(), Table_SourceData_Common_EFN2O[[#Headers],[Production system j]], 0)</f>
+        <v>5.3E-3</v>
+      </c>
+      <c r="F182" s="11" t="str" cm="1">
+        <f t="array" ref="F182">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_EFN2O_Data(), Table_SourceData_Common_EFN2O[[#Headers],[Production system j]], 0)</f>
+        <v>Cotton</v>
+      </c>
+      <c r="G182" s="11" t="str" cm="1">
+        <f t="array" ref="G182">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_EFN2O_Data(), Table_SourceData_Common_EFN2O[[#Headers],[Production system j]], 0)</f>
+        <v>Any</v>
+      </c>
+      <c r="H182" s="11" t="str" cm="1">
+        <f t="array" ref="H182">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_EFN2O_Data(), Table_SourceData_Common_EFN2O[[#Headers],[Production system j]], 0)</f>
+        <v>Any</v>
+      </c>
+    </row>
+    <row r="183" spans="4:67" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="D183" s="11" t="str" cm="1">
+        <f t="array" ref="D183">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_EFN2O_Data(), Table_SourceData_Common_EFN2O[[#Headers],[Production system j]], 0)</f>
+        <v>Horticultural crops</v>
+      </c>
+      <c r="E183" s="11" cm="1">
+        <f t="array" ref="E183">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_EFN2O_Data(), Table_SourceData_Common_EFN2O[[#Headers],[Production system j]], 0)</f>
+        <v>6.4000000000000003E-3</v>
+      </c>
+      <c r="F183" s="11" t="str" cm="1">
+        <f t="array" ref="F183">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_EFN2O_Data(), Table_SourceData_Common_EFN2O[[#Headers],[Production system j]], 0)</f>
+        <v>Horticultural crops</v>
+      </c>
+      <c r="G183" s="11" t="str" cm="1">
+        <f t="array" ref="G183">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_EFN2O_Data(), Table_SourceData_Common_EFN2O[[#Headers],[Production system j]], 0)</f>
+        <v>Any</v>
+      </c>
+      <c r="H183" s="11" t="str" cm="1">
+        <f t="array" ref="H183">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_EFN2O_Data(), Table_SourceData_Common_EFN2O[[#Headers],[Production system j]], 0)</f>
+        <v>Any</v>
+      </c>
+    </row>
+    <row r="184" spans="4:67" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="D184" s="11" t="str" cm="1">
+        <f t="array" ref="D184">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_EFN2O_Data(), Table_SourceData_Common_EFN2O[[#Headers],[Production system j]], 0)</f>
+        <v>Rice (continuous flooding)</v>
+      </c>
+      <c r="E184" s="11" cm="1">
+        <f t="array" ref="E184">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_EFN2O_Data(), Table_SourceData_Common_EFN2O[[#Headers],[Production system j]], 0)</f>
+        <v>3.0000000000000001E-3</v>
+      </c>
+      <c r="F184" s="11" t="str" cm="1">
+        <f t="array" ref="F184">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_EFN2O_Data(), Table_SourceData_Common_EFN2O[[#Headers],[Production system j]], 0)</f>
+        <v>Rice</v>
+      </c>
+      <c r="G184" s="11" t="str" cm="1">
+        <f t="array" ref="G184">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_EFN2O_Data(), Table_SourceData_Common_EFN2O[[#Headers],[Production system j]], 0)</f>
+        <v>Continuous flooding</v>
+      </c>
+      <c r="H184" s="11" t="str" cm="1">
+        <f t="array" ref="H184">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_EFN2O_Data(), Table_SourceData_Common_EFN2O[[#Headers],[Production system j]], 0)</f>
+        <v>Any</v>
+      </c>
+    </row>
+    <row r="185" spans="4:67" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="D185" s="11" t="str" cm="1">
+        <f t="array" ref="D185">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_EFN2O_Data(), Table_SourceData_Common_EFN2O[[#Headers],[Production system j]], 0)</f>
+        <v>Rice (single and multiple drainage, or alternate wetting and drying)</v>
+      </c>
+      <c r="E185" s="11" cm="1">
+        <f t="array" ref="E185">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_EFN2O_Data(), Table_SourceData_Common_EFN2O[[#Headers],[Production system j]], 0)</f>
+        <v>5.0000000000000001E-3</v>
+      </c>
+      <c r="F185" s="11" t="str" cm="1">
+        <f t="array" ref="F185">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_EFN2O_Data(), Table_SourceData_Common_EFN2O[[#Headers],[Production system j]], 0)</f>
+        <v>Rice</v>
+      </c>
+      <c r="G185" s="11" t="str" cm="1">
+        <f t="array" ref="G185">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_EFN2O_Data(), Table_SourceData_Common_EFN2O[[#Headers],[Production system j]], 0)</f>
+        <v>Single and multiple drainage, or alternate wetting and drying</v>
+      </c>
+      <c r="H185" s="11" t="str" cm="1">
+        <f t="array" ref="H185">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_EFN2O_Data(), Table_SourceData_Common_EFN2O[[#Headers],[Production system j]], 0)</f>
+        <v>Any</v>
+      </c>
+    </row>
+    <row r="186" spans="4:67" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="D186" s="11" t="str" cm="1">
+        <f t="array" ref="D186">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_EFN2O_Data(), Table_SourceData_Common_EFN2O[[#Headers],[Production system j]], 0)</f>
+        <v>Aquaculture</v>
+      </c>
+      <c r="E186" s="11" cm="1">
+        <f t="array" ref="E186">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_EFN2O_Data(), Table_SourceData_Common_EFN2O[[#Headers],[Production system j]], 0)</f>
+        <v>2.5999999999999999E-3</v>
+      </c>
+      <c r="F186" s="11" t="str" cm="1">
+        <f t="array" ref="F186">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_EFN2O_Data(), Table_SourceData_Common_EFN2O[[#Headers],[Production system j]], 0)</f>
+        <v>Aquaculture</v>
+      </c>
+      <c r="G186" s="11" t="str" cm="1">
+        <f t="array" ref="G186">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_EFN2O_Data(), Table_SourceData_Common_EFN2O[[#Headers],[Production system j]], 0)</f>
+        <v>Any</v>
+      </c>
+      <c r="H186" s="11" t="str" cm="1">
+        <f t="array" ref="H186">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_EFN2O_Data(), Table_SourceData_Common_EFN2O[[#Headers],[Production system j]], 0)</f>
+        <v>Any</v>
+      </c>
+    </row>
+    <row r="187" spans="4:67" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="D187" s="11" t="str" cm="1">
+        <f t="array" ref="D187">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_EFN2O_Data(), Table_SourceData_Common_EFN2O[[#Headers],[Production system j]], 0)</f>
+        <v>Forestry</v>
+      </c>
+      <c r="E187" s="11" cm="1">
+        <f t="array" ref="E187">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_EFN2O_Data(), Table_SourceData_Common_EFN2O[[#Headers],[Production system j]], 0)</f>
+        <v>1.8E-3</v>
+      </c>
+      <c r="F187" s="11" t="str" cm="1">
+        <f t="array" ref="F187">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_EFN2O_Data(), Table_SourceData_Common_EFN2O[[#Headers],[Production system j]], 0)</f>
+        <v>Forestry</v>
+      </c>
+      <c r="G187" s="11" t="str" cm="1">
+        <f t="array" ref="G187">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_EFN2O_Data(), Table_SourceData_Common_EFN2O[[#Headers],[Production system j]], 0)</f>
+        <v>Any</v>
+      </c>
+      <c r="H187" s="11" t="str" cm="1">
+        <f t="array" ref="H187">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_EFN2O_Data(), Table_SourceData_Common_EFN2O[[#Headers],[Production system j]], 0)</f>
+        <v>Any</v>
+      </c>
+    </row>
+    <row r="188" spans="4:67" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="D188" s="11" t="str" cm="1">
+        <f t="array" ref="D188">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_EFN2O_Data(), Table_SourceData_Common_EFN2O[[#Headers],[Production system j]], 0)</f>
+        <v/>
+      </c>
+      <c r="E188" s="11" t="str" cm="1">
+        <f t="array" ref="E188">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_EFN2O_Data(), Table_SourceData_Common_EFN2O[[#Headers],[Production system j]], 0)</f>
+        <v/>
+      </c>
+      <c r="F188" s="11" t="str" cm="1">
+        <f t="array" ref="F188">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_EFN2O_Data(), Table_SourceData_Common_EFN2O[[#Headers],[Production system j]], 0)</f>
+        <v/>
+      </c>
+      <c r="G188" s="11" t="str" cm="1">
+        <f t="array" ref="G188">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_EFN2O_Data(), Table_SourceData_Common_EFN2O[[#Headers],[Production system j]], 0)</f>
+        <v/>
+      </c>
+      <c r="H188" s="11" t="str" cm="1">
+        <f t="array" ref="H188">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_EFN2O_Data(), Table_SourceData_Common_EFN2O[[#Headers],[Production system j]], 0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="189" spans="4:67" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="190" spans="4:67" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="191" spans="4:67" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="192" spans="4:67" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="193" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="194" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="195" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="196" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25"/>
   </sheetData>
-  <phoneticPr fontId="19" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <tableParts count="11">
+  <tableParts count="12">
     <tablePart r:id="rId1"/>
     <tablePart r:id="rId2"/>
     <tablePart r:id="rId3"/>
@@ -4205,17 +4638,20 @@
     <tablePart r:id="rId9"/>
     <tablePart r:id="rId10"/>
     <tablePart r:id="rId11"/>
+    <tablePart r:id="rId12"/>
   </tableParts>
 </worksheet>
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="09eef6d6-daa8-4301-8f9f-b1ec38079286" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="7291119c-fce9-4911-96ae-b800be5dccd8">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -4414,24 +4850,25 @@
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="09eef6d6-daa8-4301-8f9f-b1ec38079286" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="7291119c-fce9-4911-96ae-b800be5dccd8">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/item4.xml><?xml version="1.0" encoding="utf-8"?>
-<AFEJSONBlob xmlns="http://schemas.advancedformulaenvironment.officeapps.live.com/afejsonblob/1.0">ewAiAHMAYwBoAGUAbQBhACIAOgAiAGgAdAB0AHAAOgAvAC8AcwBjAGgAZQBtAGEAcwAuAGEAZAB2AGEAbgBjAGUAZABmAG8AcgBtAHUAbABhAGUAbgB2AGkAcgBvAG4AbQBlAG4AdAAuAG8AZgBmAGkAYwBlAGEAcABwAHMALgBsAGkAdgBlAC4AYwBvAG0ALwBhAGYAZQBwAHIAbwBqAGUAYwB0AHMALwAwAC4AMgAiACwAIgBmAGkAbABlAHMAIgA6AFsAewAiAHAAYQB0AGgAIgA6ACIALwBwAHIAbwBqAGUAYwB0AHMALwBXAG8AcgBrAGIAbwBvAGsAIgAsACIAdABlAHgAdAAiADoAIgAvAC8AIAAtAC0ALQAgAFcAbwByAGsAYgBvAG8AawAgAG0AbwBkAHUAbABlACAALQAtAC0AXABuAC8ALwAgAEEAIABmAGkAbABlACAAbwBmACAAbgBhAG0AZQAgAGQAZQBmAGkAbgBpAHQAaQBvAG4AcwAgAG8AZgAgAHQAaABlACAAZgBvAHIAbQA6AFwAbgAvAC8AIAAgACAAIABuAGEAbQBlACAAPQAgAGQAZQBmAGkAbgBpAHQAaQBvAG4AOwBcAG4AIgB9ACwAewAiAHAAYQB0AGgAIgA6ACIALwBwAHIAbwBqAGUAYwB0AHMALwBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAIgAsACIAdABlAHgAdAAiADoAIgAvACoAXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuAFMAbwB1AHIAYwBlACAAZABhAHQAYQAgAHQAaABhAHQAIABpAHMAIABjAG8AbQBtAG8AbgAgAGEAYwByAG8AcwBzACAAYQBsAGwAIABlAG4AdABlAHIAcAByAGkAcwBlACAAdAB5AHAAZQBzAFwAbgBFAHgAYwBlAGwAIABtAG8AZAB1AGwAZQAgAG4AYQBtAGUAOgAgAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBcAG4APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQBcAG4APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQBcAG4AKgAvAFwAbgBcAG4ALwAqAFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQBcAG4AUwBvAHUAcgBjAGUAOgAgAE4AYQB0AGkAbwBuAGEAbAAgAEkAbgB2AGUAbgB0AG8AcgB5ACAAUgBlAHAAbwByAHQAIAAyADAAMgAzACAAVgBvAGwAdQBtAGUAIAAxAFwAbgBOAEkAUgBfADIAMAAyADMAXwBWAG8AbAAxAFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQBcAG4AKgAvAFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABlAG4AcwBpAHQAeQBPAGYATQBlAHQAaABhAG4AZQBcAG4AcAAgAD0AIABkAGUAbgBzAGkAdAB5ACAAbwBmACAAbQBlAHQAaABhAG4AZQAgACgAMAAuADYANwA4ADQAIABrAGcALwBtADMAKQBcAG4AVABhAGsAZQBuACAAZgByAG8AbQAgAHQAaABlACAATgBhAHQAaQBvAG4AYQBsACAARwByAGUAZQBuAGgAbwB1AHMAZQAgAGEAbgBkACAARQBuAGUAcgBnAHkAIABSAGUAcABvAHIAdABpAG4AZwAgAFwAbgAoAE0AZQBhAHMAdQByAGUAbQBlAG4AdAApACAARABlAHQAZQByAG0AaQBuAGEAdABpAG8AbgAgADIAMAAwADgAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABlAG4AcwBpAHQAeQBPAGYATQBlAHQAaABhAG4AZQBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAcAAgAD0AIABkAGUAbgBzAGkAdAB5ACAAbwBmACAAbQBlAHQAaABhAG4AZQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABlAG4AcwBpAHQAeQBPAGYATQBlAHQAaABhAG4AZQBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAGsAZwAvAG0AMwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABlAG4AcwBpAHQAeQBPAGYATQBlAHQAaABhAG4AZQBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBOAGEAdABpAG8AbgBhAGwAIABJAG4AdgBlAG4AdABvAHIAeQAgAFIAZQBwAG8AcgB0ACAAMgAwADIAMwAgAFYAbwBsAHUAbQBlACAAMQA6ACAARQBxAHUAYQB0AGkAbwBuAHMAIAAzAC4AQgAuADEAYQBfADIALAAgADMALgBCAC4AMQBjAF8AMgAsACAAMwAuAEIALgAzAF8AMQAsACAAMwAuAEIALgA0AGcAXwAyAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGUAbgBzAGkAdAB5AE8AZgBNAGUAdABoAGEAbgBlAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKAAwAC4ANgA3ADgANAApADsAXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AE4AMgBvAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBDAGcAXABuAEMAZwAgAD0AIAA0ADQALwAyADgAIABmAGEAYwB0AG8AcgAgAHQAbwAgAGMAbwBuAHYAZQByAHQAIABlAGwAZQBtAGUAbgB0AGEAbAAgAG0AYQBzAHMAIABvAGYAIABOADIATwAgAHQAbwAgAG0AbwBsAGUAYwB1AGwAYQByACAAbQBhAHMAcwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AE4AMgBvAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBDAGcAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEYAYQBjAHQAbwByACAAdABvACAAYwBvAG4AdgBlAHIAdAAgAGUAbABlAG0AZQBuAHQAYQBsACAAbQBhAHMAcwAgAG8AZgAgAE4AMgBPACAAdABvACAAbQBvAGwAZQBjAHUAbABhAHIAIABtAGEAcwBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AE4AMgBvAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBDAGcAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEMAZwBOADIATwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABOADIAbwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAQwBnAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAZgBhAGMAdABvAHIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQATgAyAG8ARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAEMAZwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBOAGEAdABpAG8AbgBhAGwAIABJAG4AdgBlAG4AdABvAHIAeQAgAFIAZQBwAG8AcgB0ACAAMgAwADIAMwAgAFYAbwBsAHUAbQBlACAAMQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABOADIAbwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAQwBnAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKAA0ADQALwAyADgAKQA7AFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXABuAEYAYQBjAHQAbwByACAAdABvACAAYwBvAG4AdgBlAHIAdAAgAGUAbABlAG0AZQBuAHQAYQBsACAAbQBhAHMAcwAgAG8AZgAgAGcAYQBzACAAdABvACAAbQBvAGwAZQBjAHUAbABhAHIAIABtAGEAcwBzAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQARwBhAHMARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBGAGEAYwB0AG8AcgAgAHQAbwAgAGMAbwBuAHYAZQByAHQAIABlAGwAZQBtAGUAbgB0AGEAbAAgAG0AYQBzAHMAIABvAGYAIABnAGEAcwAgAHQAbwAgAG0AbwBsAGUAYwB1AGwAYQByACAAbQBhAHMAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEMAZwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBmAGEAYwB0AG8AcgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAWABYAFgAWABYAFgAWABcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAOAAsACAANAAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARwBhAHMAXAAiACwAIABcACIAQwBvAG4AdgBlAHIAcwBpAG8AbgAgAGYAYQBjAHQAbwByAFwAIgAsACAAXAAiAEMAbwBuAHYAZQByAHMAaQBvAG4AIABmAGEAYwB0AG8AcgAgADEAXAAiACwAIABcACIAQwBvAG4AdgBlAHIAcwBpAG8AbgAgAGYAYQBjAHQAbwByACAAMgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBPADIAXAAiACwAIABcACIANAA0AC8AMQAyAFwAIgAsACAANAA0ACwAIAAxADIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBIADQAXAAiACwAIABcACIAMQA2AC8AMQAyAFwAIgAsACAAMQA2ACwAIAAxADIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgAyAE8AXAAiACwAIABcACIANAA0AC8AMgA4AFwAIgAsACAANAA0ACwAIAAyADgAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgBvAHgAXAAiACwAIABcACIANAA2AC8AMQA0AFwAIgAsACAANAA2ACwAIAAxADQAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBPAFwAIgAsACAAXAAiADIAOAAvADEAMgBcACIALAAgADIAOAAsACAAMQAyADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMATwAyACAATABpAG0AZQBcACIALAAgAFwAIgA0ADQALwAxADIAXAAiACwAIAA0ADQALAAgADEAMgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOAE0AVgBPAEMAXAAiACwAIABcACIAMQA0AC8AMQAyAFwAIgAsACAAMQA0ACwAIAAxADIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEcAVwBQAE4AMgBPAFwAbgBHAGwAbwBiAGEAbAAgAHcAYQByAG0AaQBuAGcAIABwAG8AdABlAG4AdABpAGEAbAAgAGYAbwByACAAZwByAGUAZQBuAGgAbwB1AHMAZQAgAGcAYQBzAGUAcwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBHAFcAUABfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARwBsAG8AYgBhAGwAIAB3AGEAcgBtAGkAbgBnACAAcABvAHQAZQBuAHQAaQBhAGwAIABmAG8AcgAgAGcAcgBlAGUAbgBoAG8AdQBzAGUAIABnAGEAcwBlAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEcAVwBQAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBHAFcAUABOADIATwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARwBXAFAAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBmAGEAYwB0AG8AcgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARwBXAFAAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAWABYAFgAWABYAFgAWABcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARwBXAFAAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAOAAsACAAMgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARwBhAHMAXAAiACwAIABcACIAQwBPADIALQBlACAAZgBhAGMAdABvAHIAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMATwAyAFwAIgAsACAAMQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAEgANABcACIALAAgADIAOAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOADIATwBcACIALAAgADIANgA1ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMARgA0AFwAIgAsACAANgA2ADMAMAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDADIARgA2AFwAIgAsACAAMQAyADIAMAAwADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFMARgA2AFwAIgAsACAAMgAyADgAMAAwADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE4ARgAzAFwAIgAsACAAMQA3ADIAMAAwAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQQB1AHMAdAByAGEAbABpAGEAbgBTAHQAYQB0AGUAcwBUAGUAcgByAGkAdABvAHIAaQBlAHMAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQQB1AHMAdAByAGEAbABpAGEAbgBTAHQAYQB0AGUAcwBUAGUAcgByAGkAdABvAHIAaQBlAHMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEEAdQBzAHQAcgBhAGwAaQBhAG4AIABzAHQAYQB0AGUAcwAgAGEAbgBkACAAdABlAHIAcgBpAHQAbwByAGkAZQBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBBAHUAcwB0AHIAYQBsAGkAYQBuAFMAdABhAHQAZQBzAFQAZQByAHIAaQB0AG8AcgBpAGUAcwBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEEAdQBzAHQAcgBhAGwAaQBhAG4AUwB0AGEAdABlAHMAVABlAHIAcgBpAHQAbwByAGkAZQBzAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEEAdQBzAHQAcgBhAGwAaQBhAG4AUwB0AGEAdABlAHMAVABlAHIAcgBpAHQAbwByAGkAZQBzAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBBAHUAcwB0AHIAYQBsAGkAYQBuAFMAdABhAHQAZQBzAFQAZQByAHIAaQB0AG8AcgBpAGUAcwBfAEQAYQB0AGEAXABuACAAIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADkALAAgADMALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFMAdABhAHQAZQAvAFQAZQByAHIAaQB0AG8AcgB5AFwAIgAsACAAXAAiAEMAbwBtAG0AbwBuACAATgBhAG0AZQBcACIALAAgAFwAIgBBAGIAYgByAGUAdgBpAGEAdABpAG8AbgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgBlAHcAIABTAG8AdQB0AGgAIABXAGEAbABlAHMAXAAiACwAIABcACIATgBlAHcAIABTAG8AdQB0AGgAIABXAGEAbABlAHMAXAAiACwAIABcACIATgBTAFcAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEEAdQBzAHQAcgBhAGwAaQBhAG4AIABDAGEAcABpAHQAYQBsACAAVABlAHIAcgBpAHQAbwByAHkAXAAiACwAIABcACIAQQBDAFQAXAAiACwAIABcACIAQQBDAFQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFYAaQBjAHQAbwByAGkAYQBcACIALAAgAFwAIgBWAGkAYwB0AG8AcgBpAGEAXAAiACwAIABcACIAVgBJAEMAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFEAdQBlAGUAbgBzAGwAYQBuAGQAXAAiACwAIABcACIAUQB1AGUAZQBuAHMAbABhAG4AZABcACIALAAgAFwAIgBRAEwARABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUwBvAHUAdABoACAAQQB1AHMAdAByAGEAbABpAGEAXAAiACwAIABcACIAUwBvAHUAdABoACAAQQB1AHMAdAByAGEAbABpAGEAXAAiACwAIABcACIAUwBBAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGUAcwB0AGUAcgBuACAAQQB1AHMAdAByAGEAbABpAGEAXAAiACwAIABcACIAVwBlAHMAdABlAHIAbgAgAEEAdQBzAHQAcgBhAGwAaQBhAFwAIgAsACAAXAAiAFcAQQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVABhAHMAbQBhAG4AaQBhAFwAIgAsACAAXAAiAFQAYQBzAG0AYQBuAGkAYQBcACIALAAgAFwAIgBUAEEAUwBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgBvAHIAdABoAGUAcgBuACAAVABlAHIAcgBpAHQAbwByAHkAXAAiACwAIABcACIATgBvAHIAdABoAGUAcgBuACAAVABlAHIAcgBpAHQAbwByAHkAXAAiACwAIABcACIATgBUAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBBAFMAQQA0AEEAcgBlAGEAcwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAEEAUwBBADQAQQByAGUAYQBzAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBBAEIAUwAgAFMAdABhAHQAaQBzAHQAYwBhAGwAIABBAHIAZQBhAHMAIABMAGUAdgBlAGwAIAA0ACAALQAgAFcAZQBzAHQAZQByAG4AIABBAHUAcwB0AHIAYQBsAGkAYQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBBAFMAQQA0AEEAcgBlAGEAcwBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAQQBTAEEANABBAHIAZQBhAHMAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBBAFMAQQA0AEEAcgBlAGEAcwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBBAHUAcwB0AHIAYQBsAGkAYQBuACAAQgB1AHIAZQBhAHUAIABvAGYAIABTAHQAYQB0AGkAcwB0AGkAYwBzACAAKABBAEIAUwApACAALQAgAFMAdABhAHQAaQBzAHQAaQBjAGEAbAAgAEEAcgBlAGEAcwAgAEwAZQB2AGUAbAAgADIAIAAtACAAMgAwADIAMQAgAC0AIABTAGgAYQBwAGUAZgBpAGwAZQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBBAFMAQQA0AEEAcgBlAGEAcwBfAEQAYQB0AGEAXABuACAAIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADEAMQAsACAAMQAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUwBBACAANAAgAE4AYQBtAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEIAdQBuAGIAdQByAHkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE0AYQBuAGQAdQByAGEAaABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUABlAHIAdABoACAALQAgAEkAbgBuAGUAcgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUABlAHIAdABoACAALQAgAE4AbwByAHQAaAAgAEUAYQBzAHQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFAAZQByAHQAaAAgAC0AIABOAG8AcgB0AGgAIABXAGUAcwB0AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBQAGUAcgB0AGgAIAAtACAAUwBvAHUAdABoACAARQBhAHMAdABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUABlAHIAdABoACAALQAgAFMAbwB1AHQAaAAgAFcAZQBzAHQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAZQBzAHQAZQByAG4AIABBAHUAcwB0AHIAYQBsAGkAYQAgAC0AIABXAGgAZQBhAHQAIABCAGUAbAB0AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGUAcwB0AGUAcgBuACAAQQB1AHMAdAByAGEAbABpAGEAIAAtACAATwB1AHQAYgBhAGMAawAgACgATgBvAHIAdABoACkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAZQBzAHQAZQByAG4AIABBAHUAcwB0AHIAYQBsAGkAYQAgAC0AIABPAHUAdABiAGEAYwBrACAAKABTAG8AdQB0AGgAKQBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAZQB0AEEAbgBkAEQAcgB5AFoAbwBuAGUAcwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAGUAdABBAG4AZABEAHIAeQBaAG8AbgBlAHMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgAEEAdQBzAHQAcgBhAGwAaQBhAG4AIAB3AGUAdAAgAGEAbgBkACAAZAByAHkAIAB6AG8AbgBlAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAZQB0AEEAbgBkAEQAcgB5AFoAbwBuAGUAcwBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAZQB0AEEAbgBkAEQAcgB5AFoAbwBuAGUAcwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAGUAdABBAG4AZABEAHIAeQBaAG8AbgBlAHMAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAVABhAGIAbABlACAAMQAuADIAOgAgAFQAcgBhAG4AcwBsAGEAdABpAG4AZwAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAHMAIAB0AG8AIAB3AGUAdAAgAGEAbgBkACAAZAByAHkAIAB6AG8AbgBlAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAZQB0AEEAbgBkAEQAcgB5AFoAbwBuAGUAcwBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAzACwAIAAxACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBWAEEAUgBJAEEAVABJAE8ATgAgAE8ARgAgAFMATwBVAFIAQwBFACAARABBAFQAQQA6AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBBAGQAZABlAGQAIAB3AGEAcgBtACAALwAgAGMAbwBvAGwAIAB0AGUAbQBwAGUAcgBhAHQAZQAgAG0AbwBpAHMAdAAgAC8AIABkAHIAeQAgAC0AIABsAG8AdwAgAGYAcgBvAHMAdAAgAGEAbgBkACAAaABpAGcAaAAgAHQAZQBtAHAAIABjAGwAYQBzAHMAZQBzACAAdABvACAAYQBjAGMAbwBtAG0AbwBkAGEAdABlACAAYwBsAGkAbQBhAHQAZQAgAHMAYwBlAG4AYQByAGkAbwBzACAAZQB4AGMAbAB1AGQAZQBkACAAYgB5ACAAVgBFAEUAUgBHACAAYwByAGkAdABlAHIAaQBhAC4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEYAaQB4AGUAZAAgAHQAeQBwAG8AIAAtACAAQwBoAGEAbgBnAGUAZAAgAFwAdQAwADAAMgA3AEYAcgB5AFwAdQAwADAAMgA3ACAAdABvACAAXAB1ADAAMAAyADcARAByAHkAXAB1ADAAMAAyADcALgBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAZQB0AEEAbgBkAEQAcgB5AFoAbwBuAGUAcwBfAEQAYQB0AGEAXABuACAAIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADEANQAsACAAMgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBsAGkAbQBhAHQAZQAgAFoAbwBuAGUAXAAiACwAIABcACIAVwBlAHQAIABvAHIAIABEAHIAeQAgAFoAbwBuAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAcgBvAHAAaQBjAGEAbAAgAG0AbwBuAHQAYQBuAGUAXAAiACwAIABcACIAVwBlAHQAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVAByAG8AcABpAGMAYQBsACAAdwBlAHQAXAAiACwAIABcACIAVwBlAHQAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVAByAG8AcABpAGMAYQBsACAAbQBvAGkAcwB0AFwAIgAsACAAXAAiAFcAZQB0ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAcgBvAHAAaQBjAGEAbAAgAGQAcgB5AFwAIgAsACAAXAAiAEQAcgB5ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAYQByAG0AIAB0AGUAbQBwAGUAcgBhAHQAZQAgAG0AbwBpAHMAdABcACIALAAgAFwAIgBXAGUAdAAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGEAcgBtACAAdABlAG0AcABlAHIAYQB0AGUAIABkAHIAeQBcACIALAAgAFwAIgBEAHIAeQAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AbwBsACAAdABlAG0AcABlAHIAYQB0AGUAIABtAG8AaQBzAHQAXAAiACwAIABcACIAVwBlAHQAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBvAG8AbAAgAHQAZQBtAHAAZQByAGEAdABlACAAZAByAHkAXAAiACwAIABcACIARAByAHkAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBhAHIAbQAgAHQAZQBtAHAAZQByAGEAdABlACAAbQBvAGkAcwB0ACAALQAgAGwAbwB3ACAAZgByAG8AcwB0AFwAIgAsACAAXAAiAFcAZQB0ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAYQByAG0AIAB0AGUAbQBwAGUAcgBhAHQAZQAgAGQAcgB5ACAALQAgAGwAbwB3ACAAZgByAG8AcwB0AFwAIgAsACAAXAAiAEQAcgB5ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAYQByAG0AIAB0AGUAbQBwAGUAcgBhAHQAZQAgAG0AbwBpAHMAdAAgAC0AIABoAGkAZwBoACAAdABlAG0AcABcACIALAAgAFwAIgBXAGUAdAAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGEAcgBtACAAdABlAG0AcABlAHIAYQB0AGUAIABkAHIAeQAgAC0AIABoAGkAZwBoACAAdABlAG0AcABcACIALAAgAFwAIgBEAHIAeQAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AbwBsACAAdABlAG0AcABlAHIAYQB0AGUAIABtAG8AaQBzAHQAIAAtACAAbABvAHcAIABmAHIAbwBzAHQAXAAiACwAIABcACIAVwBlAHQAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBvAG8AbAAgAHQAZQBtAHAAZQByAGEAdABlACAAZAByAHkAIAAtACAAbABvAHcAIABmAHIAbwBzAHQAXAAiACwAIABcACIARAByAHkAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbABpAG0AYQB0AGUAWgBvAG4AZQBzAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbABpAG0AYQB0AGUAWgBvAG4AZQBzAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIABBAHUAcwB0AHIAYQBsAGkAYQBuACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBsAGkAbQBhAHQAZQBaAG8AbgBlAHMAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABUAGEAYgBsAGUAIAAxAC4AMwA6ACAAQwBsAGkAbQBhAHQAZQAgAGEAbgBkACAAUgBhAGkAbgBmAGEAbABsACAAegBvAG4AZQAgAGMAbABhAHMAcwBpAGYAaQBjAGEAdABpAG8AbgBzACAAYQBuAGQAIABkAGUAZgBpAG4AaQB0AGkAbwBuAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbABpAG0AYQB0AGUAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADUALAAgADEALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFYAQQBSAEkAQQBUAEkATwBOACAATwBGACAAUwBPAFUAUgBDAEUAIABEAEEAVABBADoAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEEAZABkAGUAZAAgAHcAYQByAG0AIAAvACAAYwBvAG8AbAAgAHQAZQBtAHAAZQByAGEAdABlACAAbQBvAGkAcwB0ACAALwAgAGQAcgB5ACAALQAgAGwAbwB3ACAAZgByAG8AcwB0ACAAYQBuAGQAIABoAGkAZwBoACAAdABlAG0AcAAgAGMAbABhAHMAcwBlAHMAIAB0AG8AIABhAGMAYwBvAG0AbQBvAGQAYQB0AGUAIABjAGwAaQBtAGEAdABlACAAcwBjAGUAbgBhAHIAaQBvAHMAIABlAHgAYwBsAHUAZABlAGQAIABiAHkAIABWAEUARQBSAEcAIABjAHIAaQB0AGUAcgBpAGEALgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARgBpAHgAZQBkACAAdAB5AHAAbwAgAGkAbgAgAE0AQQBUACAAdgBhAGwAdQBlACAAZgBvAHIAIAB3AGEAcgBtACAAdABlAG0AcABlAHIAYQB0AGUAIABkAHIAeQAgAC0AIABjAGgAYQBuAGcAZQBkACAAMQAwACAAdABvACAAMQAxAC4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEEAZABkAGUAZAAgAG0AaQBuACAAYQBuAGQAIABtAGEAeAAgAGMAbwBsAHUAbQBuAHMAIABmAG8AcgAgAE0AQQBUACwAIABNAEEAUAAsACAAZgByAG8AcwB0ACAAZABhAHkAcwAgAHAAZQByACAAeQBlAGEAcgAsACAAZQBsAGUAdgBhAHQAaQBvAG4ALAAgAE0AQQBQADoAUABFAFQAIAB0AG8AIABjAGEAbABjAHUAbABhAHQAZQAgAHoAbwBuAGUAcwAgAGYAcgBvAG0AIAByAGUAYQBsACAAYwBsAGkAbQBhAHQAZQAgAGQAYQB0AGEALgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARwBBAEYAIABhAGMAYwBlAHAAdABzACAAcgBhAGkAbgBmAGEAbABsACAAYQBzACAAYQAgAHAAcgBvAHgAeQAgAGYAbwByACAAcAByAGUAYwBpAHAAaQB0AGEAdABpAG8AbgAuAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBsAGkAbQBhAHQAZQBaAG8AbgBlAHMAXwBEAGEAdABhAFwAbgAgACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAA5ACwAIAAxADYALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAbABpAG0AYQB0AGUAIABaAG8AbgBlAFwAIgAsACAAXAAiAE0AQQBUAFwAIgAsACAAXAAiAE0AQQBQAFwAIgAsACAAXAAiAEYAcgBvAHMAdAAgAGQAYQB5AHMAIABwAGUAcgAgAHkAZQBhAHIAXAAiACwAIABcACIARQBsAGUAdgBhAHQAaQBvAG4AXAAiACwAIABcACIATQBBAFAAOgBQAEUAVABcACIALAAgAFwAIgBNAGkAbgAgAHQAZQBtAHAAXAAiACwAIABcACIATQBhAHgAIAB0AGUAbQBwAFwAIgAsACAAXAAiAE0AaQBuACAAcgBhAGkAbgBmAGEAbABsAFwAIgAsACAAXAAiAE0AYQB4ACAAcgBhAGkAbgBmAGEAbABsAFwAIgAsACAAXAAiAE0AaQBuACAAZgByAG8AcwB0ACAAZABhAHkAcwBcACIALAAgAFwAIgBNAGEAeAAgAGYAcgBvAHMAdAAgAGQAYQB5AHMAXAAiACwAIABcACIATQBpAG4AIABlAGwAZQB2AGEAdABpAG8AbgBcACIALAAgAFwAIgBNAGEAeAAgAGUAbABlAHYAYQB0AGkAbwBuAFwAIgAsACAAXAAiAE0AaQBuACAATQBBAFAAOgBQAEUAVABcACIALAAgAFwAIgBNAGkAbgAgAE0AQQBQADoAUABFAFQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAcgBvAHAAaQBjAGEAbAAgAG0AbwBuAHQAYQBuAGUAXAAiACwAIABcACIAXAB1ADAAMAAzAGUAIAAxADgAIABDAFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAGQiIAA3AFwAIgAsACAAXAAiAFwAdQAwADAAMwBlACAAMQAwADAAMAAgAG0AXAAiACwAIABcACIAQQBuAHkAXAAiACwAIAAxADgALgAwADAAMQAsACAAOQA5ADkAOQA5ADkALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA3ACwAIAAxADAAMAAwACwAIAA5ADkAOQA5ADkAOQAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVAByAG8AcABpAGMAYQBsACAAdwBlAHQAXAAiACwAIABcACIAXAB1ADAAMAAzAGUAIAAxADgAIABDAFwAIgAsACAAXAAiAFwAdQAwADAAMwBlACAAMgAwADAAMAAgAG0AbQBcACIALAAgAFwAIgBkIiAANwBcACIALAAgAFwAIgBkIiAAMQAwADAAMAAgAG0AXAAiACwAIABcACIAQQBuAHkAXAAiACwAIAAxADgALgAwADAAMQAsACAAOQA5ADkAOQA5ADkALAAgADIAMAAwADAALgAwADAAMQAsACAAOQA5ADkAOQA5ADkALAAgAC0AOQA5ADkAOQA5ADkALAAgADcALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5AC4AOQA5ADkALAAgACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVAByAG8AcABpAGMAYQBsACAAbQBvAGkAcwB0AFwAIgAsACAAXAAiAFwAdQAwADAAMwBlACAAMQA4ACAAQwBcACIALAAgAFwAIgBcAHUAMAAwADMAZQAgADEAMAAwADAAIABtAG0AIAAtACAAZCIgADIAMAAwADAAIABtAG0AXAAiACwAIABcACIAZCIgADcAXAAiACwAIABcACIAZCIgADEAMAAwADAAIABtAFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAMQA4AC4AMAAwADEALAAgADkAOQA5ADkAOQA5ACwAIAAxADAAMAAwAC4AMAAwADEALAAgADIAMAAwADAALAAgAC0AOQA5ADkAOQA5ADkALAAgADcALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5AC4AOQA5ADkALAAgACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVAByAG8AcABpAGMAYQBsACAAZAByAHkAXAAiACwAIABcACIAXAB1ADAAMAAzAGUAIAAxADgAIABDAFwAIgAsACAAXAAiAGQiIAAxADAAMAAwACAAbQBtAFwAIgAsACAAXAAiAGQiIAA3AFwAIgAsACAAXAAiAGQiIAAxADAAMAAwACAAbQBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgADEAOAAuADAAMAAxACwAIAA5ADkAOQA5ADkAOQAsACAALQA5ADkAOQA5ADkAOQAsACAAMQAwADAAMAAsACAALQA5ADkAOQA5ADkAOQAsACAANwAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkALgA5ADkAOQAsACAAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQA5ADkAOQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGEAcgBtACAAdABlAG0AcABlAHIAYQB0AGUAIABtAG8AaQBzAHQAXAAiACwAIABcACIAXAB1ADAAMAAzAGUAIAAxADAAIABDAFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAFwAdQAwADAAMwBlACAAMQBcACIALAAgADEAMAAuADAAMAAxACwAIAA5ADkAOQA5ADkAOQAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQA5ADkAOQAsACAAMQAuADAAMAAxACwAIAA5ADkAOQA5ADkAOQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGEAcgBtACAAdABlAG0AcABlAHIAYQB0AGUAIABkAHIAeQBcACIALAAgAFwAIgBcAHUAMAAwADMAZQAgADEAMAAgAEMAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAZCIgADEAXAAiACwAIAAxADAALgAwADAAMQAsACAAOQA5ADkAOQA5ADkALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQA5ADkAOQAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkALAAgACAALQA5ADkAOQA5ADkAOQAsACAAMQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AbwBsACAAdABlAG0AcABlAHIAYQB0AGUAIABtAG8AaQBzAHQAXAAiACwAIABcACIAXAB1ADAAMAAzAGUAIAAwACAAQwAgAC0AIABkIiAAMQAwACAAQwBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBcAHUAMAAwADMAZQAgADEAXAAiACwAIAAtADkAOQA5ADkAOQA5ACwAIAAxADAALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQA5ADkAOQAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkALAAgADEALgAwADAAMQAsACAAOQA5ADkAOQA5ADkAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBvAG8AbAAgAHQAZQBtAHAAZQByAGEAdABlACAAZAByAHkAXAAiACwAIABcACIAXAB1ADAAMAAzAGUAIAAwACAAQwAgAC0AIABkIiAAMQAwACAAQwBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBkIiAAMQBcACIALAAgAC0AOQA5ADkAOQA5ADkALAAgADEAMAAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQA5ADkAOQAsACAAIAAtADkAOQA5ADkAOQA5ACwAIAAxAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAEEAcABwAGUAbgBkAGkAYwBlAHMAXABuACAAIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADQALAAgADEALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE4AbwB0AGUAOgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATQBBAFQAIAA9ACAAbQBlAGEAbgAgAGEAbgBuAHUAYQBsACAAdABlAG0AcABlAHIAYQB0AHUAcgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBNAEEAUAAgAD0AIABtAGUAYQBuACAAYQBuAG4AdQBhAGwAIABwAHIAZQBjAGkAcABpAHQAYQB0AGkAbwBuAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBQAEUAVAAgAD0AIABwAG8AdABlAG4AdABpAGEAbAAgAGUAdgBhAHAAbwB0AHIAYQBuAHMAcABpAHIAYQB0AGkAbwBuAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAHMAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAcwBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAQQB1AHMAdAByAGEAbABpAGEAbgAgAHQAZQBtAHAAZQByAGEAdAB1AHIAZQAgAHoAbwBuAGUAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAcwBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAHMAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAcwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABUAGEAYgBsAGUAIAAxAC4AMwA6ACAAQwBsAGkAbQBhAHQAZQAgAGEAbgBkACAAUgBhAGkAbgBmAGEAbABsACAAegBvAG4AZQAgAGMAbABhAHMAcwBpAGYAaQBjAGEAdABpAG8AbgBzACAAYQBuAGQAIABkAGUAZgBpAG4AaQB0AGkAbwBuAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAHMAXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBBAFIASQBBAFQASQBPAE4AIABPAEYAIABTAE8AVQBSAEMARQAgAEQAQQBUAEEAOgAgAEEAZABkAGUAZAAgAGUAeAB0AHIAYQAgAE0AQQBUACAAbQBpAG4AIABhAG4AZAAgAE0AQQBUACAAbQBhAHgAIABjAG8AbAB1AG0AbgBzACAAdABvACAAYwBhAGwAYwB1AGwAYQB0AGUAIAB6AG8AbgBlACAAZgByAG8AbQAgAHIAZQBhAGwAIAB0AGUAbQBwAGUAcgBhAHQAdQByAGUAIABkAGEAdABhAC4AXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAHMAXwBEAGEAdABhAFwAbgAgACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAA0ACwAIAA0ACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAGUAbQBwAGUAcgBhAHQAdQByAGUAIABaAG8AbgBlAFwAIgAsACAAXAAiAE0AZQBkAGkAYQBuACAAQQBuAG4AdQBhAGwAIABUAGUAbQBwAGUAcgBhAHQAdQByAGUAIAAoAE0AQQBUACkAXAAiACwAIABcACIATQBpAG4AIABNAEEAVABcACIALAAgAFwAIgBNAGEAeAAgAE0AQQBUAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGEAcgBtAFwAIgAsACAAXAAiAGUiIAAyADYAIABDAFwAIgAsACAAMgA2ACwAIAA5ADkAOQA5ADkAOQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAGUAbQBwAGUAcgBhAHQAZQBcACIALAAgAFwAIgAxADUAIAAtACAAMgA1ACAAQwBcACIALAAgADEANQAsACAAMgA1AC4AOQA5ADkAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBvAG8AbABcACIALAAgAFwAIgBkIiAAMQA0ACAAQwBcACIALAAgAC0AOQA5ADkAOQA5ADkALAAgADEANAAuADkAOQA5AFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBzAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlAHMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgAEEAdQBzAHQAcgBhAGwAaQBhAG4AIAByAGEAaQBuAGYAYQBsAGwAIAB6AG8AbgBlAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlAHMAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBzAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlAHMAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAVABhAGIAbABlACAAMQAuADMAOgAgAEMAbABpAG0AYQB0AGUAIABhAG4AZAAgAFIAYQBpAG4AZgBhAGwAbAAgAHoAbwBuAGUAIABjAGwAYQBzAHMAaQBmAGkAYwBhAHQAaQBvAG4AcwAgAGEAbgBkACAAZABlAGYAaQBuAGkAdABpAG8AbgBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYAQQBSAEkAQQBUAEkATwBOACAATwBGACAAUwBPAFUAUgBDAEUAIABEAEEAVABBADoAIABBAGQAZABlAGQAIABlAHgAdAByAGEAIABSAGEAaQBuAGYAYQBsAGwAIABtAGkAbgAgAGEAbgBkACAAUgBhAGkAbgBmAGEAbABsACAAbQBhAHgAIABjAG8AbAB1AG0AbgBzACAAdABvACAAYwBhAGwAYwB1AGwAYQB0AGUAIAB6AG8AbgBlACAAZgByAG8AbQAgAHIAZQBhAGwAIAByAGEAaQBuAGYAYQBsAGwAIABkAGEAdABhAC4AXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlAHMAXwBEAGEAdABhAFwAbgAgACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAzACwAIAA0ACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBSAGEAaQBuAGYAYQBsAGwAIABaAG8AbgBlAFwAIgAsACAAXAAiAEEAbgBuAHUAYQBsACAAcgBhAGkAbgBmAGEAbABsAFwAIgAsACAAXAAiAFIAYQBpAG4AZgBhAGwAbAAgAG0AaQBuAFwAIgAsACAAXAAiAFIAYQBpAG4AZgBhAGwAbAAgAG0AYQB4AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBIAGkAZwBoACAAcgBhAGkAbgBmAGEAbABsAFwAIgAsACAAXAAiAEEAbgBuAHUAYQBsACAAcgBhAGkAbgBmAGEAbABsACAAXAB1ADAAMAAzAGUAIAA2ADAAMABtAG0AXAAiACwAIAA2ADAAMAAuADAAMAAxACwAIAA5ADkAOQA5ADkAOQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBMAG8AdwAgAHIAYQBpAG4AZgBhAGwAbABcACIALAAgAFwAIgBBAG4AbgB1AGEAbAAgAHIAYQBpAG4AZgBhAGwAbAAgAGQiIAA2ADAAMABtAG0AXAAiACwAIAAtADkAOQA5ADkAOQA5ACwAIAA2ADAAMABcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBzAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIABBAHUAcwB0AHIAYQBsAGkAYQBuACAAbABlAGEAYwBoAGkAbgBnACAAegBvAG4AZQBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBzAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgAFQAYQBiAGwAZQAgADEALgAzADoAIABDAGwAaQBtAGEAdABlACAAYQBuAGQAIABSAGEAaQBuAGYAYQBsAGwAIAB6AG8AbgBlACAAYwBsAGEAcwBzAGkAZgBpAGMAYQB0AGkAbwBuAHMAIABhAG4AZAAgAGQAZQBmAGkAbgBpAHQAaQBvAG4AcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBfAEQAYQB0AGEAXABuACAAIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADQALAAgADIALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEwAZQBhAGMAaABpAG4AZwAgAFoAbwBuAGUAXAAiACwAIABcACIATABlAGEAYwBoAGkAbgBnACAAYwByAGkAdABlAHIAaQBhAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBMAGUAYQBjAGgAaQBuAGcAIABvAGMAYwB1AHIAcwBcACIALAAgAFwAIgCjAygANdhf3DXYTtw12FbcNdhb3CkAXAB1ADAAMAAzAGUAowMoADXYONw12EfcMAApACsANdhg3DXYXNw12FbcNdhZ3CAANdhk3DXYTtw12GHcNdhS3DXYX9wgAA4hNdhc3DXYWdw12FHcNdhW3DXYW9w12FTcIAA12FDcNdhO3DXYXdw12E7cNdhQ3DXYVtw12GHcNdhm3FwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBMAGUAYQBjAGgAaQBuAGcAIABkAG8AZQBzACAAbgBvAHQAIABvAGMAYwB1AHIAXAAiACwAIABcACIAowMoADXYX9w12E7cNdhW3DXYW9wpAGQiowMoADXYONw12EfcMAApACsANdhg3DXYXNw12FbcNdhZ3CAANdhk3DXYTtw12GHcNdhS3DXYX9wgAA4hNdhc3DXYWdw12FHcNdhW3DXYW9w12FTcIAA12FDcNdhO3DXYXdw12E7cNdhQ3DXYVtw12GHcNdhm3FwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABcAG4ANQAuADUALgAyAC4AMwAgAEMAbwBuAHMAdABhAG4AdAAgAFAAYQByAGEAbQBlAHQAZQByAHMAXABuAEYAcgBhAGMAdABpAG8AbgAgAG8AZgAgAE4AIAB0AGgAYQB0ACAAaQBzACAAYQB2AGEAaQBsAGEAYgBsAGUAIABmAG8AcgAgAGwAZQBhAGMAaABpAG4AZwAgAGEAbgBkACAAcgB1AG4AbwBmAGYAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARgByAGEAYwB0AGkAbwBuACAAbwBmACAATgAgAHQAaABhAHQAIABpAHMAIABhAHYAYQBpAGwAYQBiAGwAZQAgAGYAbwByACAAbABlAGEAYwBoAGkAbgBnACAAYQBuAGQAIAByAHUAbgBvAGYAZgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiACgARABpAG0AZQBuAHMAaQBvAG4AbABlAHMAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoANQAuADUALgAyAC4AMwAgAEMAbwBuAHMAdABhAG4AdAAgAFAAYQByAGEAbQBlAHQAZQByAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMwAsACAAMgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIASQBzACAAaQBuACAAbABlAGEAYwBoAGkAbgBnACAAegBvAG4AZQBcACIALABcACIARgByAGEAYwBXAEUAVABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAWQBlAHMAIAAtACAAaQBuACAAbABlAGEAYwBoAGkAbgBnACAAegBvAG4AZQBcACIALAAgADEAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgBvACAALQAgAG4AbwB0ACAAaQBuACAAbABlAGEAYwBoAGkAbgBnACAAegBvAG4AZQBcACIALAAgADAAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuACAAIABDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAKABcACIAXAAiACkAKQA7AFwAbgBcAG4AXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAdABhAFMAYwBvAHIAZQBzAF8AUwBjAG8AcABlADMAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAHQAYQBTAGMAbwByAGUAcwBfAFMAYwBvAHAAZQAzAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBBAHUAcwB0AHIAYQBsAGkAYQBuACAAZABhAHQAYQAgAHMAYwBvAHIAZQBzACAAZgBvAHIAIABzAGMAbwBwAGUAIAAzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAdABhAFMAYwBvAHIAZQBzAF8AUwBjAG8AcABlADMAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAdABhAFMAYwBvAHIAZQBzAF8AUwBjAG8AcABlADMAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAHQAYQBTAGMAbwByAGUAcwBfAFMAYwBvAHAAZQAzAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgAFgAWABYAFgAWABYAFgAWABcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAHQAYQBTAGMAbwByAGUAcwBfAFMAYwBvAHAAZQAzAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAdABhAFMAYwBvAHIAZQBzAF8AUwBjAG8AcABlADMAXwBEAGEAdABhAFwAbgAgACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAA2ACwAIAAyACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBEAGEAdABhACAAcwBvAHUAcgBjAGUAXAAiACwAIABcACIARABhAHQAYQAgAHMAYwBvAHIAZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIASQBuAHQAZQByAG4AYQB0AGkAbwBuAGEAbAAgAHMAYwBvAHAAZQAgADMAIABkAGEAdABhAGIAYQBzAGUAXAAiACwAIAAxADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEEAdQBzAHQAcgBhAGwAaQBhAG4AIABzAGMAbwBwAGUAIAAzACAAZABhAHQAYQBiAGEAcwBlAFwAIgAsACAAMgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBTAHQAYQB0AGUAIABvAHIAIAByAGUAZwBpAG8AbgBhAGwAIABzAGMAbwBwAGUAIAAzACAAZABhAHQAYQBiAGEAcwBlAFwAIgAsACAAMwA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBFAG0AaQBzAHMAaQBvAG4AcwAgAGkAbgB0AGUAbgBzAGkAdAB5ACAAYwBhAGwAYwB1AGwAYQB0AGUAZAAgAGYAcgBvAG0AIABhAHAAcAByAG8AdgBlAGQAIABtAGUAdABoAG8AZABcACIALAAgADQAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVgBlAHIAaQBmAGkAZQBkACAAYwByAGUAZABlAG4AdABpAGEAbAAgAG0AYQB0AGMAaABpAG4AZwAgAEkAUwBPADEANAAwADYANwBcACIALAAgADUAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAFwAbgAgACAALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBMAEUAQQBDAEgAXABuADUALgA1AC4AMgAuADMAIABDAG8AbgBzAHQAYQBuAHQAIABQAGEAcgBhAG0AZQB0AGUAcgBzAFwAbgBGAHIAYQBjAHQAaQBvAG4AIABvAGYAIABOACAAdABoAGEAdAAgAGkAcwAgAGEAdgBhAGkAbABhAGIAbABlACAAZgBvAHIAIABsAGUAYQBjAGgAaQBuAGcAIABhAG4AZAAgAHIAdQBuAG8AZgBmAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMATABFAEEAQwBIAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBGAHIAYQBjAHQAaQBvAG4AIABvAGYAIABOACAAdABoAGEAdAAgAGkAcwAgAGEAdgBhAGkAbABhAGIAbABlACAAZgBvAHIAIABsAGUAYQBjAGgAaQBuAGcAIABhAG4AZAAgAHIAdQBuAG8AZgBmAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAEwARQBBAEMASABfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiACgARABpAG0AZQBuAHMAaQBvAG4AbABlAHMAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ADUALgA1AC4AMgAuADMAIABDAG8AbgBzAHQAYQBuAHQAIABQAGEAcgBhAG0AZQB0AGUAcgBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAEwARQBBAEMASABfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBOAGEAdABpAG8AbgBhAGwAIABJAG4AdgBlAG4AdABvAHIAeQAgAFIAZQBwAG8AcgB0ACAAVgBvAGwAdQBtAGUAIAAxADoAIABMAGUAYQBjAGgAaQBuAGcAIABhAG4AZAAgAHIAdQBuAG8AZgBmACAAKAAzAC4ARAAuAGIALgAyACkAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMATABFAEEAQwBIAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADEALAAgADIALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEYAcgBhAGMATABFAEEAQwBIAFwAIgAsADAALgAyADQAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuACAAIABDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAEwARQBBAEMASABfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoACgAXAAiAFwAIgApACkAOwBcAG4AXABuAFwAbgBcAG4AIAAgAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBsAGUAYQBjAGgAXABuADUALgA1AC4AMgAuADMAIABDAG8AbgBzAHQAYQBuAHQAIABQAGEAcgBhAG0AZQB0AGUAcgBzAFwAbgBFAG0AaQBzAHMAaQBvAG4AIABmAGEAYwB0AG8AcgAgAGYAbwByACAAbgBpAHQAcgBvAGcAZQBuACAAbABlAGEAYwBoAGkAbgBnACAAYQBuAGQAIAByAHUAbgBvAGYAZgBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAbABlAGEAYwBoAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBFAG0AaQBzAHMAaQBvAG4AIABmAGEAYwB0AG8AcgAgAGYAbwByACAAbgBpAHQAcgBvAGcAZQBuACAAbABlAGEAYwBoAGkAbgBnACAAYQBuAGQAIAByAHUAbgBvAGYAZgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAGwAZQBhAGMAaABfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiACgAawBnACAATgAyAE8ALQBOACAALwAgAGsAZwAgAE4AXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBsAGUAYQBjAGgAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ADUALgA1AC4AMgAuADMAIABDAG8AbgBzAHQAYQBuAHQAIABQAGEAcgBhAG0AZQB0AGUAcgBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAbABlAGEAYwBoAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAE4AYQB0AGkAbwBuAGEAbAAgAEkAbgB2AGUAbgB0AG8AcgB5ACAAUgBlAHAAbwByAHQAIABWAG8AbAB1AG0AZQAgADEAOgAgAEUAcQB1AGEAdABpAG8AbgAgADMALgBEAC4AQgBfADEAMABcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAGwAZQBhAGMAaABfAEQAYQB0AGEAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAxACwAIAAyACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBFAEYAbABlAGEAYwBoAFwAIgAsADAALgAwADEAMQBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AIAAgAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBsAGUAYQBjAGgAXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKAAoAFwAIgBcACIAKQApADsAXABuACIAfQAsAHsAIgBwAGEAdABoACIAOgAiAC8AcAByAG8AagBlAGMAdABzAC8AQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMAIgAsACIAdABlAHgAdAAiADoAIgBVAHQAaQBsAGkAdAB5AF8ARwBlAHQAQQByAHIAYQB5AFQAYQBiAGwAZQBSAG8AdwBTAHQAYQByAHQATgB1AG0AYgBlAHIAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABUAGEAYgBsAGUAaABlAGEAZABlAHIAQwBlAGwAbAAsAFIAbwB3AHMAQgBlAHQAdwBlAGUAbgBIAGUAYQBkAGUAcgBhAG4AZABBAHIAcgBhAHkALABcAG4AIAAgACAAIABSAE8AVwAoAFQAYQBiAGwAZQBoAGUAYQBkAGUAcgBDAGUAbABsACkAIAArACAAUgBvAHcAcwBCAGUAdAB3AGUAZQBuAEgAZQBhAGQAZQByAGEAbgBkAEEAcgByAGEAeQAgAC0AIAAxAFwAbgApADsAXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8ARwBlAHQAQQByAHIAYQB5AFQAYQBiAGwAZQBDAG8AbAB1AG0AbgBTAHQAYQByAHQATgB1AG0AYgBlAHIAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgAFQAYQBiAGwAZQBIAGUAYQBkAGUAcgBDAGUAbABsACwAXABuACAAIABDAE8ATABVAE0ATgAoAFQAYQBiAGwAZQBIAGUAYQBkAGUAcgBDAGUAbABsACkAXABuACkAOwBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBEAGkAcwBwAGwAYQB5AEEAcgByAGEAeQBJAG4AVABhAGIAbABlAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAQQByAHIAYQB5AEQAYQB0AGEALAAgAFQAYQBiAGwAZQBoAGUAYQBkAGUAcgBDAGUAbABsACwAIABSAG8AdwBzAEIAZQB0AHcAZQBlAG4ASABlAGEAZABlAHIAYQBuAGQAQQByAHIAYQB5ACwAIABbAEMAbwBsAHUAbQBuAHMAQgBlAHQAdwBlAGUAbgBIAGUAYQBkAGUAcgBBAG4AZABBAHIAcgBhAHkAXQAsAFwAbgAgAEkARgBFAFIAUgBPAFIAKABcAG4AIAAgACAAIAAgAEkATgBEAEUAWAAoAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABVAE4ASQBRAFUARQAoAEEAcgByAGEAeQBEAGEAdABhACkALAAgAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABSAE8AVwAoACkALQBVAHQAaQBsAGkAdAB5AF8ARwBlAHQAQQByAHIAYQB5AFQAYQBiAGwAZQBSAG8AdwBTAHQAYQByAHQATgB1AG0AYgBlAHIAKABUAGEAYgBsAGUAaABlAGEAZABlAHIAQwBlAGwAbAAsACAAUgBvAHcAcwBCAGUAdAB3AGUAZQBuAEgAZQBhAGQAZQByAGEAbgBkAEEAcgByAGEAeQApACwAIABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAQwBPAEwAVQBNAE4AKAApAC0AVQB0AGkAbABpAHQAeQBfAEcAZQB0AEEAcgByAGEAeQBUAGEAYgBsAGUAQwBvAGwAdQBtAG4AUwB0AGEAcgB0AE4AdQBtAGIAZQByACgAVABhAGIAbABlAGgAZQBhAGQAZQByAEMAZQBsAGwAKQAgACsAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAEkARgAoAEkAUwBPAE0ASQBUAFQARQBEACgAQwBvAGwAdQBtAG4AcwBCAGUAdAB3AGUAZQBuAEgAZQBhAGQAZQByAEEAbgBkAEEAcgByAGEAeQApACwAIAAxACwAIABDAG8AbAB1AG0AbgBzAEIAZQB0AHcAZQBlAG4ASABlAGEAZABlAHIAQQBuAGQAQQByAHIAYQB5ACkAXABuACAAIAAgACAAIAAgACAAIAApACwAIABcACIAXAAiAFwAbgAgACAAIAAgACkAXABuACkAOwBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBMAG8AbwBrAHUAcABWAGEAbAB1AGUASQBuAFQAYQBiAGwAZQBcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQAsACAATABvAG8AawB1AHAAQQByAHIAYQB5ACwAIABSAGUAdAB1AHIAbgBBAHIAcgBhAHkALABcAG4AIAAgACAAIABYAEwATwBPAEsAVQBQACgATABvAG8AawB1AHAAVgBhAGwAdQBlACwAIABMAG8AbwBrAHUAcABBAHIAcgBhAHkALAAgAFIAZQB0AHUAcgBuAEEAcgByAGEAeQAsACAAXAAiAFwAIgApAFwAbgApADsAXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8ATABvAG8AawB1AHAAVgBhAGwAdQBlAEkAbgBUAGEAYgBsAGUATgB1AG0AYgBlAHIAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABMAG8AbwBrAHUAcABWAGEAbAB1AGUALAAgAEwAbwBvAGsAdQBwAEEAcgByAGEAeQAsACAAUgBlAHQAdQByAG4AQQByAHIAYQB5ACwAXABuACAAIAAgACAASQBGACgASQBTAE4AVQBNAEIARQBSACgAXABuACAAIAAgACAAIAAgACAAIABYAEwATwBPAEsAVQBQACgATABvAG8AawB1AHAAVgBhAGwAdQBlACwAIABMAG8AbwBrAHUAcABBAHIAcgBhAHkALAAgAFIAZQB0AHUAcgBuAEEAcgByAGEAeQAsACAAXAAiAFwAIgApAFwAbgAgACAAIAAgACkALAAgAFgATABPAE8ASwBVAFAAKABMAG8AbwBrAHUAcABWAGEAbAB1AGUALAAgAEwAbwBvAGsAdQBwAEEAcgByAGEAeQAsACAAUgBlAHQAdQByAG4AQQByAHIAYQB5ACwAIABcACIAXAAiACkALAAgADAAKQBcAG4AKQA7AFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAFMAcABsAGkAdABTAHQAcgBpAG4AZwBJAG4AdABvAEEAcgByAGEAeQBcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAEMAZQBsAGwALAAgAEQAZQBsAGkAbQBpAHQAZQByACwAIABbAEMAaABhAHIAYQBjAHQAZQByAFQAbwBSAGUAbQBvAHYAZQAxAF0ALAAgAFsAQwBoAGEAcgBhAGMAdABlAHIAVABvAFIAZQBtAG8AdgBlADIAXQAsAFwAbgAgACAAIAAgACAAIAAgACAARgBJAEwAVABFAFIAWABNAEwAKABcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBcAHUAMAAwADMAYwB0AFwAdQAwADAAMwBlAFwAdQAwADAAMwBjAHMAXAB1ADAAMAAzAGUAXAAiACAAXAB1ADAAMAAyADYAXABuACAAIAAgACAAIAAgACAAIABTAFUAQgBTAFQASQBUAFUAVABFACgAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFMAVQBCAFMAVABJAFQAVQBUAEUAKABTAFUAQgBTAFQASQBUAFUAVABFACgAQwBlAGwAbAAsAEMAaABhAHIAYQBjAHQAZQByAFQAbwBSAGUAbQBvAHYAZQAxACwAXAAiAFwAIgApACwAQwBoAGEAcgBhAGMAdABlAHIAVABvAFIAZQBtAG8AdgBlADIALABcACIAXAAiACkALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAARABlAGwAaQBtAGkAdABlAHIALABcACIAXAB1ADAAMAAzAGMALwBzAFwAdQAwADAAMwBlAFwAdQAwADAAMwBjAHMAXAB1ADAAMAAzAGUAXAAiAFwAbgAgACAAIAAgACAAIAAgACAAKQAgAFwAdQAwADAAMgA2AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAFwAdQAwADAAMwBjAC8AcwBcAHUAMAAwADMAZQBcAHUAMAAwADMAYwAvAHQAXAB1ADAAMAAzAGUAXAAiACwAXABuACAAIAAgACAAIAAgACAAIABcACIALwAvAHMAXAAiAFwAbgAgACAAIAAgACkAXABuACkAOwBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBHAGUAdABDAGwAaQBtAGEAdABlAFoAbwBuAGUAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABhAHYAZwBUAGUAbQBwACwAYQB2AGcAUgBhAGkAbgAsAGYAcgBvAHMAdABEAGEAeQBzACwAZQBsAGUAdgAsAG0AYQBwAF8AcABlAHQALABcAG4AIAAgACAAIABMAEUAVAAoAFwAbgAgACAAIAAgACAAIAAgACAAbQBhAHMAawAsAFwAbgAgACAAIAAgACAAIAAgACAAKABWAEEATABVAEUAKABUAGEAYgBsAGUAXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBsAGkAbQBhAHQAZQBaAG8AbgBlAHMAWwBNAGkAbgAgAHQAZQBtAHAAXQApAFwAdQAwADAAMwBjAD0AYQB2AGcAVABlAG0AcAApACoAXABuACAAIAAgACAAIAAgACAAIAAoAFYAQQBMAFUARQAoAFQAYQBiAGwAZQBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBbAE0AYQB4ACAAdABlAG0AcABdACkAXAB1ADAAMAAzAGUAPQBhAHYAZwBUAGUAbQBwACkAKgBcAG4AIAAgACAAIAAgACAAIAAgACgAVgBBAEwAVQBFACgAVABhAGIAbABlAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbABpAG0AYQB0AGUAWgBvAG4AZQBzAFsATQBpAG4AIAByAGEAaQBuAGYAYQBsAGwAXQApAFwAdQAwADAAMwBjAD0AYQB2AGcAUgBhAGkAbgApACoAXABuACAAIAAgACAAIAAgACAAIAAoAFYAQQBMAFUARQAoAFQAYQBiAGwAZQBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBbAE0AYQB4ACAAcgBhAGkAbgBmAGEAbABsAF0AKQBcAHUAMAAwADMAZQA9AGEAdgBnAFIAYQBpAG4AKQAqAFwAbgAgACAAIAAgACAAIAAgACAAKABWAEEATABVAEUAKABUAGEAYgBsAGUAXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBsAGkAbQBhAHQAZQBaAG8AbgBlAHMAWwBNAGkAbgAgAGYAcgBvAHMAdAAgAGQAYQB5AHMAXQApAFwAdQAwADAAMwBjAD0AZgByAG8AcwB0AEQAYQB5AHMAKQAqAFwAbgAgACAAIAAgACAAIAAgACAAKABWAEEATABVAEUAKABUAGEAYgBsAGUAXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBsAGkAbQBhAHQAZQBaAG8AbgBlAHMAWwBNAGEAeAAgAGYAcgBvAHMAdAAgAGQAYQB5AHMAXQApAFwAdQAwADAAMwBlAD0AZgByAG8AcwB0AEQAYQB5AHMAKQAqAFwAbgAgACAAIAAgACAAIAAgACAAKABWAEEATABVAEUAKABUAGEAYgBsAGUAXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBsAGkAbQBhAHQAZQBaAG8AbgBlAHMAWwBNAGkAbgAgAGUAbABlAHYAYQB0AGkAbwBuAF0AKQBcAHUAMAAwADMAYwA9AGUAbABlAHYAKQAqAFwAbgAgACAAIAAgACAAIAAgACAAKABWAEEATABVAEUAKABUAGEAYgBsAGUAXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBsAGkAbQBhAHQAZQBaAG8AbgBlAHMAWwBNAGEAeAAgAGUAbABlAHYAYQB0AGkAbwBuAF0AKQBcAHUAMAAwADMAZQA9AGUAbABlAHYAKQAqAFwAbgAgACAAIAAgACAAIAAgACAAKABWAEEATABVAEUAKABUAGEAYgBsAGUAXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBsAGkAbQBhAHQAZQBaAG8AbgBlAHMAWwBNAGkAbgAgAE0AQQBQADoAUABFAFQAXQApAFwAdQAwADAAMwBjAD0AbQBhAHAAXwBwAGUAdAApACoAXABuACAAIAAgACAAIAAgACAAIAAoAFYAQQBMAFUARQAoAFQAYQBiAGwAZQBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBbAE0AYQB4ACAATQBBAFAAOgBQAEUAVABdACkAXAB1ADAAMAAzAGUAPQBtAGEAcABfAHAAZQB0ACkALABcAG4AIAAgACAAIAAgACAAIAAgAC8AKgAgAEkAZgAgAHQAaABlACAAdABlAG0AcAAgAGkAcwAgAG8AdgBlAHIAIAAxADgAIABhAG4AZAAgAGYAcgBvAHMAdAAgAGQAYQB5AHMAIABhAHIAZQAgADcAIABvAHIAIABiAGUAbABvAHcAIAB3AGUAIABnAGUAdAAgAG0AdQBsAHQAaQBwAGwAZQAgAHIAZQBzAHUAbAB0AHMALgBcAG4AIAAgACAAIAAgACAAIAAgAEkAbgAgAHQAaABpAHMAIABjAGEAcwBlACAAXAB1ADAAMAAyADcAdAByAG8AcABpAGMAYQBsAFwAdQAwADAAMgA3ACAAcgBlAHMAdQBsAHQAcwAgAHMAaABvAHUAbABkACAAYgBlACAAdQBzAGUAZAAsACAAcwBvACAAdwBlACAAdABhAGsAZQAgAHQAaABlACAAZgBpAHIAcwB0ACAAcgBlAHMAdQBsAHQAXABuACAAIAAgACAAIAAgACAAIABiAGUAYwBhAHUAcwBlACAAdAByAG8AcABpAGMAYQBsACAAdgBhAGwAdQBlAHMAIABhAHIAZQAgAGYAaQByAHMAdAAgAGkAbgAgAHQAaABlACAAdABhAGIAbABlACAAKgAvAFwAbgAgACAAIAAgACAAIAAgACAAVABBAEsARQAoAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABGAEkATABUAEUAUgAoAFQAYQBiAGwAZQBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBbAEMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAF0ALABtAGEAcwBrACwAIABcACIATgBvACAAbQBhAHQAYwBoAFwAIgApACwAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgADEAXABuACAAIAAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACkAOwBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBMAG8AbwBrAHUAcABJAHQAZQBtAEYAcgBvAG0ATQBpAG4ATQBhAHgAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABMAG8AbwBrAHUAcABWAGEAbAB1AGUALAAgAE0AaQBuAEEAcgByAGEAeQAsACAATQBhAHgAQQByAHIAYQB5ACwAIABJAHQAZQBtAEEAcgByAGEAeQAsAFwAbgAgACAAIAAgAEwARQBUACgAXABuACAAIAAgACAAIAAgACAAIABtAGEAcwBrACwAXABuACAAIAAgACAAIAAgACAAIAAoAFYAQQBMAFUARQAoAE0AaQBuAEEAcgByAGEAeQApAFwAdQAwADAAMwBjAD0ATABvAG8AawB1AHAAVgBhAGwAdQBlACkAKgBcAG4AIAAgACAAIAAgACAAIAAgACgAVgBBAEwAVQBFACgATQBhAHgAQQByAHIAYQB5ACkAXAB1ADAAMAAzAGUAPQBMAG8AbwBrAHUAcABWAGEAbAB1AGUAKQAsAFwAbgAgACAAIAAgACAAIAAgACAARgBJAEwAVABFAFIAKABJAHQAZQBtAEEAcgByAGEAeQAsACAAbQBhAHMAawAsACAAXAAiAE4AbwAgAG0AYQB0AGMAaABcACIAKQBcAG4AIAAgACAAIAApAFwAbgApADsAXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8AUwB1AG0AUQB1AGEAbgB0AGkAdAB5AEYAcgBvAG0AQwByAGkAdABlAHIAaQBhAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIABDAHIAaQB0AGUAcgBpAGEAMQAsACAAQwByAGkAdABlAHIAaQBhADEAVAB5AHAAZQBBAHIAcgBhAHkALAAgAFEAdQBhAG4AdABpAHQAeQAsACAAWwBNAHUAbAB0AGkAcABsAGkAZQByAF0ALAAgAFsAQwByAGkAdABlAHIAaQBhADIAXQAsAFsAQwByAGkAdABlAHIAaQBhADIAQQByAHIAYQB5AF0ALABcAG4AIAAgAEwARQBUACgAXABuACAAIAAgACAAbQB1AGwAdABpAHAAbABpAGUAcgAsACAASQBGACgASQBTAE8ATQBJAFQAVABFAEQAKABNAHUAbAB0AGkAcABsAGkAZQByACkALAAxACwATQB1AGwAdABpAHAAbABpAGUAcgApACwAXABuACAAIAAgACAAcQB1AGEAbgB0AGkAdAB5ACwAIABRAHUAYQBuAHQAaQB0AHkAKgBNAHUAbAB0AGkAcABsAGkAZQByACwAXABuACAAIAAgACAAYwByAGkAdABlAHIAaQBhADEALAAtAC0AKABDAHIAaQB0AGUAcgBpAGEAMQBUAHkAcABlAEEAcgByAGEAeQA9AEMAcgBpAHQAZQByAGkAYQAxACkALABcAG4AIAAgACAAIABjAHIAaQB0AGUAcgBpAGEAMgAsAEkARgAoAEkAUwBPAE0ASQBUAFQARQBEACgAQwByAGkAdABlAHIAaQBhADIAKQAsADEALAAtAC0AKABDAHIAaQB0AGUAcgBpAGEAMgBBAHIAcgBhAHkAPQBDAHIAaQB0AGUAcgBpAGEAMgApACkALABcAG4AIAAgACAAIABTAFUATQBQAFIATwBEAFUAQwBUACgAYwByAGkAdABlAHIAaQBhADEAKgBjAHIAaQB0AGUAcgBpAGEAMgAqAHEAdQBhAG4AdABpAHQAeQApAFwAbgAgACAAKQBcAG4AKQA7AFwAbgBcAG4AZwBlAHQATwB2AGUAcgBsAGEAcABwAGkAbgBnAFIAZQBwAG8AcgB0AGkAbgBnAEMAeQBjAGwAZQBzAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAAUAByAG8AZAB1AGMAdABpAG8AbgBDAHkAYwBsAGUAUwB0AGEAcgB0ACwAUAByAG8AZAB1AGMAdABpAG8AbgBDAHkAYwBsAGUARQBuAGQALABSAGUAcABvAHIAdABpAG4AZwBDAHkAYwBsAGUAUwB0AGEAcgB0ACwAXABuACAAIAAgACAATABFAFQAKABcAG4AIAAgACAAIAAgACAAIAAgAFMALABQAHIAbwBkAHUAYwB0AGkAbwBuAEMAeQBjAGwAZQBTAHQAYQByAHQALABcAG4AIAAgACAAIAAgACAAIAAgAEUALABQAHIAbwBkAHUAYwB0AGkAbwBuAEMAeQBjAGwAZQBFAG4AZAAsAFwAbgAgACAAIAAgACAAIAAgACAAbQAsAE0ATwBOAFQASAAoAFIAZQBwAG8AcgB0AGkAbgBnAEMAeQBjAGwAZQBTAHQAYQByAHQAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAZAAsAEQAQQBZACgAUgBlAHAAbwByAHQAaQBuAGcAQwB5AGMAbABlAFMAdABhAHIAdAApACwAXABuACAAIAAgACAAIAAgACAAIABQAGUAcgBpAG8AZABFAG4AZAAsAEwAQQBNAEIARABBACgAcwB0ACwARQBEAEEAVABFACgAcwB0ACwAMQAyACkALQAxACkALABcAG4AIAAgACAAIAAgACAAIAAgAEEALABTAC0AMwA2ADUALABcAG4AIAAgACAAIAAgACAAIAAgAHkAYQAsAFkARQBBAFIAKABBACkALABcAG4AIAAgACAAIAAgACAAIAAgAHkAYgAsAFkARQBBAFIAKABFACkALABcAG4AIAAgACAAIAAgACAAIAAgAGYAaQByAHMAdABZAGUAYQByACwAeQBhACsAKABQAGUAcgBpAG8AZABFAG4AZAAoAEQAQQBUAEUAKAB5AGEALABtACwAZAApACkAXAB1ADAAMAAzAGMAIABTACkALABcAG4AIAAgACAAIAAgACAAIAAgAGwAYQBzAHQAWQBlAGEAcgAsAHkAYgAtACgARABBAFQARQAoAHkAYgAsAG0ALABkACkAXAB1ADAAMAAzAGUAIABFACkALABcAG4AIAAgACAAIAAgACAAIAAgAE0AQQBYACgAMAAsAGwAYQBzAHQAWQBlAGEAcgAtAGYAaQByAHMAdABZAGUAYQByACsAMQApAFwAbgAgACAAIAAgACkAXABuACkAOwBcAG4AXABuAGcAZQB0AE8AdgBlAHIAbABhAHAAcABpAG4AZwBSAGUAcABvAHIAdABpAG4AZwBQAGUAcgBpAG8AZABzAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAAUAByAG8AZAB1AGMAdABpAG8AbgBDAHkAYwBsAGUAUwB0AGEAcgB0ACwAUAByAG8AZAB1AGMAdABpAG8AbgBDAHkAYwBsAGUARQBuAGQALABSAGUAcABvAHIAdABpAG4AZwBDAHkAYwBsAGUAUwB0AGEAcgB0ACwAXABuACAAIAAgACAATABFAFQAKABcAG4AIAAgACAAIAAgACAAIAAgAFMALABQAHIAbwBkAHUAYwB0AGkAbwBuAEMAeQBjAGwAZQBTAHQAYQByAHQALABcAG4AIAAgACAAIAAgACAAIAAgAEUALABQAHIAbwBkAHUAYwB0AGkAbwBuAEMAeQBjAGwAZQBFAG4AZAAsAFwAbgAgACAAIAAgACAAIAAgACAAbQAsAE0ATwBOAFQASAAoAFIAZQBwAG8AcgB0AGkAbgBnAEMAeQBjAGwAZQBTAHQAYQByAHQAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAZAAsAEQAQQBZACgAUgBlAHAAbwByAHQAaQBuAGcAQwB5AGMAbABlAFMAdABhAHIAdAApACwAIAAvACoAaABlAGwAcABlAHIAOgAgAGUAbgBkACAAZABhAHQAZQAgAGYAbwByACAAYQAgAHIAZQBwAG8AcgB0AGkAbgBnACAAcABlAHIAaQBvAGQAIABzAHQAYQByAHQAaQBuAGcAIABhAHQAIABhACAAZwBpAHYAZQBuACAAZABhAHQAZQAqAC8AXABuACAAIAAgACAAIAAgACAAIABQAGUAcgBpAG8AZABFAG4AZAAsAEwAQQBNAEIARABBACgAcwB0ACwARQBEAEEAVABFACgAcwB0ACwAMQAyACkALQAxACkALAAgAC8AKgBvAG4AbAB5ACAAbgBlAGUAZAAgAHQAbwAgAGwAbwBvAGsAIABiAGEAYwBrACAAMwA2ADUAIABkAGEAeQBzACgAbQBhAHgAIABvAHYAZQByAGwAYQBwACAAdwBpAG4AZABvAHcAKQAqAC8AXABuACAAIAAgACAAIAAgACAAIABBACwAUwAtADMANgA1ACwAXABuACAAIAAgACAAIAAgACAAIAB5AGEALABZAEUAQQBSACgAQQApACwAXABuACAAIAAgACAAIAAgACAAIAB5AGIALABZAEUAQQBSACgARQApACwAIAAvACoAaQBmACAAdABoAGUAIABhAG4AYwBoAG8AcgAgAGYAbwByACAAeQBhACAAZQBuAGQAcwAgAGIAZQBmAG8AcgBlACAAUwAsAGkAdAAgAGMAYQBuAFwAdQAwADAAMgA3AHQAIABvAHYAZQByAGwAYQBwADsAIABtAG8AdgBlACAAdABvACAAbgBlAHgAdAAgAHkAZQBhAHIAKgAvAFwAbgAgACAAIAAgACAAIAAgACAAZgBpAHIAcwB0AFkAZQBhAHIALAB5AGEAKwAoAFAAZQByAGkAbwBkAEUAbgBkACgARABBAFQARQAoAHkAYQAsAG0ALABkACkAKQBcAHUAMAAwADMAYwBTACkALAAgAC8AKgBpAGYAIAB0AGgAZQAgAGEAbgBjAGgAbwByACAAZgBvAHIAIAB5AGIAIABzAHQAYQByAHQAcwAgAGEAZgB0AGUAcgAgAEUALABpAHQAIABjAGEAbgBcAHUAMAAwADIANwB0ACAAbwB2AGUAcgBsAGEAcAA7ACAAbQBvAHYAZQAgAHQAbwAgAHAAcgBlAHYAaQBvAHUAcwAgAHkAZQBhAHIAKgAvAFwAbgAgACAAIAAgACAAIAAgACAAbABhAHMAdABZAGUAYQByACwAeQBiAC0AKABEAEEAVABFACgAeQBiACwAbQAsAGQAKQBcAHUAMAAwADMAZQBFACkALABcAG4AIAAgACAAIAAgACAAIAAgAG4ALABNAEEAWAAoADAALABsAGEAcwB0AFkAZQBhAHIALQBmAGkAcgBzAHQAWQBlAGEAcgArADEAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAeQByAHMALABTAEUAUQBVAEUATgBDAEUAKABuACwAMQAsAGYAaQByAHMAdABZAGUAYQByACwAMQApACwAXABuACAAIAAgACAAIAAgACAAIABzAHQAYQByAHQAcwAsAEQAQQBUAEUAKAB5AHIAcwAsAG0ALABkACkALABcAG4AIAAgACAAIAAgACAAIAAgAGUAbgBkAHMALABNAEEAUAAoAHMAdABhAHIAdABzACwAUABlAHIAaQBvAGQARQBuAGQAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAdABhAGcALABJAEYAKABzAHQAYQByAHQAcwA9AFIAZQBwAG8AcgB0AGkAbgBnAEMAeQBjAGwAZQBTAHQAYQByAHQALABcACIAIAAoAFQAaABpAHMAIAByAGUAcABvAHIAdABpAG4AZwAgAGMAeQBjAGwAZQApAFwAIgAsAFwAIgBcACIAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAcwB0AGEAcgB0AHMAVABlAHgAdAAsAFQARQBYAFQAKABzAHQAYQByAHQAcwAsAFwAIgBkAGQAIABtAG0AbQAgAHkAeQB5AHkAXAAiACkALABcAG4AIAAgACAAIAAgACAAIAAgAGUAbgBkAHMAVABlAHgAdAAsAFQARQBYAFQAKABlAG4AZABzACwAXAAiAGQAZAAgAG0AbQBtACAAeQB5AHkAeQBcACIAKQAsAFwAbgAgACAAIAAgACAAIAAgACAASQBGACgAbgA9ADAALABcACIAXAAiACwASABTAFQAQQBDAEsAKABzAHQAYQByAHQAcwBUAGUAeAB0ACAAXAB1ADAAMAAyADYAIABcACIAIAB0AG8AIABcACIAIABcAHUAMAAwADIANgAgAGUAbgBkAHMAVABlAHgAdAAgAFwAdQAwADAAMgA2ACAAdABhAGcAKQApAFwAbgAgACAAIAAgACkAXABuACkAOwBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBEAGkAcwBwAGwAYQB5AEYAdQBuAGMAdABpAG8AbgBOAGEAbQBlAFwAbgA9AEwAQQBNAEIARABBACgARgB1AG4AYwB0AGkAbwBuACwAIABGAE8AUgBNAFUATABBAFQARQBYAFQAKABGAHUAbgBjAHQAaQBvAG4AKQApADsAIgB9ACwAewAiAHAAYQB0AGgAIgA6ACIALwBwAHIAbwBqAGUAYwB0AHMALwBDAG8AbQBtAG8AbgBfAEUAcQB1AGEAdABpAG8AbgBzACIALAAiAHQAZQB4AHQAIgA6ACIAXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQBcAG4AQwBvAG4AdgBlAHIAdAAgAG4AaQB0AHIAbwB1AHMAIABvAHgAaQBkAGUAIABlAG0AaQBzAHMAaQBvAG4AcwAgAHQAbwAgAGMAYQByAGIAbwBuACAAZABpAG8AeABpAGQAZQAgAGUAcQB1AGkAdgBhAGwAZQBuAHQAIABlAG0AaQBzAHMAaQBvAG4AcwBcAG4ARQBOADIATwAgAEMATwAyAGUAXABuAHQAIABDAE8AMgBlAFwAbgBFAE4AMgBPADoAIABuAGkAdAByAG8AdQBzACAAbwB4AGkAZABlACAAZQBtAGkAcwBzAGkAbwBuAHMAIAAoAHQAIABOADIATwApAFwAbgBHAFcAUABOADIATwA6ACAAZwBsAG8AYgBhAGwAIAB3AGEAcgBtAGkAbgBnACAAcABvAHQAZQBuAHQAaQBhAGwAIABmAG8AcgAgAG4AaQB0AHIAbwB1AHMAIABvAHgAaQBkAGUAIAAoAHQAIABDAE8AMgAtAGUAIAAvACAAdAAgAE4AMgBPACkAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABFAF8ATgAyAE8ALAAgAEcAVwBQAF8ATgAyAE8ALABcAG4AIAAgACAAIABFAF8ATgAyAE8AIAAqACAARwBXAFAAXwBOADIATwBcAG4AIAAgACkAXABuADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQATgAyAE8AVABvAEMATwAyAGUAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEMAbwBuAHYAZQByAHQAIABuAGkAdAByAG8AdQBzACAAbwB4AGkAZABlACAAZQBtAGkAcwBzAGkAbwBuAHMAIAB0AG8AIABjAGEAcgBiAG8AbgAgAGQAaQBvAHgAaQBkAGUAIABlAHEAdQBpAHYAYQBsAGUAbgB0ACAAZQBtAGkAcwBzAGkAbwBuAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARQBOADIATwAgAEMATwAyAGUAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAHQAIABDAE8AMgBlAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQATgAyAE8AVABvAEMATwAyAGUAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQBfAEwAYQB0AGUAeABFAHEAdQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEMATwAyAF8AZQAgAD0AIABFAF8AewBOADIATwB9ACAAXABcAHQAaQBtAGUAcwAgAEcAVwBQAF8AewBOADIATwB9AFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQATgAyAE8AVABvAEMATwAyAGUAXwBBAHIAZwB1AG0AZQBuAHQAcwBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADIALAAgADIALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEUATgAyAE8AXAAiACwAXAAiAE4AaQB0AHIAbwB1AHMAIABvAHgAaQBkAGUAIABlAG0AaQBzAHMAaQBvAG4AcwAgACgAdAAgAE4AMgBPACkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEcAVwBQAE4AMgBPAFwAIgAsAFwAIgBHAGwAbwBiAGEAbAAgAHcAYQByAG0AaQBuAGcAIABwAG8AdABlAG4AdABpAGEAbAAgAGYAbwByACAAbgBpAHQAcgBvAHUAcwAgAG8AeABpAGQAZQAgACgAdAAgAEMATwAyAC0AZQAgAC8AIAB0ACAATgAyAE8AKQBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQBcAG4AQwBvAG4AdgBlAHIAdAAgAG0AZQB0AGgAYQBuAGUAIABlAG0AaQBzAHMAaQBvAG4AcwAgAHQAbwAgAGMAYQByAGIAbwBuACAAZABpAG8AeABpAGQAZQAgAGUAcQB1AGkAdgBhAGwAZQBuAHQAIABlAG0AaQBzAHMAaQBvAG4AcwBcAG4ARQBDAEgANAAgAEMATwAyAGUAXABuAHQAIABDAE8AMgBlAFwAbgBFAEMASAA0ADoAIABtAGUAdABoAGEAbgBlACAAZQBtAGkAcwBzAGkAbwBuAHMAIAAoAHQAIABDAEgANAApAFwAbgBHAFcAUABDAEgANAA6ACAAZwBsAG8AYgBhAGwAIAB3AGEAcgBtAGkAbgBnACAAcABvAHQAZQBuAHQAaQBhAGwAIABmAG8AcgAgAG0AZQB0AGgAYQBuAGUAIAAoAHQAIABDAE8AMgAtAGUAIAAvACAAdAAgAEMASAA0ACkAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABFAF8AQwBIADQALAAgAEcAVwBQAF8AQwBIADQALABcAG4AIAAgACAAIABFAF8AQwBIADQAIAAqACAARwBXAFAAXwBDAEgANABcAG4AIAAgACkAXABuADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQAQwBIADQAVABvAEMATwAyAGUAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEMAbwBuAHYAZQByAHQAIABtAGUAdABoAGEAbgBlACAAZQBtAGkAcwBzAGkAbwBuAHMAIAB0AG8AIABjAGEAcgBiAG8AbgAgAGQAaQBvAHgAaQBkAGUAIABlAHEAdQBpAHYAYQBsAGUAbgB0ACAAZQBtAGkAcwBzAGkAbwBuAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARQBDAEgANAAgAEMATwAyAGUAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAHQAIABDAE8AMgBlAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQAQwBIADQAVABvAEMATwAyAGUAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQBfAEwAYQB0AGUAeABFAHEAdQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEMATwAyAF8AZQAgAD0AIABFAF8AewBDAEgANAB9ACAAXABcAHQAaQBtAGUAcwAgAEcAVwBQAF8AewBDAEgANAB9AFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQAQwBIADQAVABvAEMATwAyAGUAXwBBAHIAZwB1AG0AZQBuAHQAcwBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADIALAAgADIALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEUAQwBIADQAXAAiACwAXAAiAE0AZQB0AGgAYQBuAGUAIABlAG0AaQBzAHMAaQBvAG4AcwAgACgAdAAgAEMASAA0ACkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEcAVwBQAEMASAA0AFwAIgAsAFwAIgBHAGwAbwBiAGEAbAAgAHcAYQByAG0AaQBuAGcAIABwAG8AdABlAG4AdABpAGEAbAAgAGYAbwByACAAbQBlAHQAaABhAG4AZQAgACgAdAAgAEMATwAyAC0AZQAgAC8AIAB0ACAAQwBIADQAKQBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwAiAH0AXQAsACIAcAByAG8AagBlAGMAdABOAGEAbQBlAHMAIgA6AFsAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGUAbgBzAGkAdAB5AE8AZgBNAGUAdABoAGEAbgBlAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAZQBuAHMAaQB0AHkATwBmAE0AZQB0AGgAYQBuAGUAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAZQBuAHMAaQB0AHkATwBmAE0AZQB0AGgAYQBuAGUAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGUAbgBzAGkAdAB5AE8AZgBNAGUAdABoAGEAbgBlAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AE4AMgBvAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBDAGcAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABOADIAbwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAQwBnAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQATgAyAG8ARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAEMAZwBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABOADIAbwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAQwBnAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABOADIAbwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAQwBnAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AEcAYQBzAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AEcAYQBzAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AEcAYQBzAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AEcAYQBzAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARwBXAFAAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARwBXAFAAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARwBXAFAAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEcAVwBQAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARwBXAFAAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEEAdQBzAHQAcgBhAGwAaQBhAG4AUwB0AGEAdABlAHMAVABlAHIAcgBpAHQAbwByAGkAZQBzAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEEAdQBzAHQAcgBhAGwAaQBhAG4AUwB0AGEAdABlAHMAVABlAHIAcgBpAHQAbwByAGkAZQBzAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEEAdQBzAHQAcgBhAGwAaQBhAG4AUwB0AGEAdABlAHMAVABlAHIAcgBpAHQAbwByAGkAZQBzAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBBAHUAcwB0AHIAYQBsAGkAYQBuAFMAdABhAHQAZQBzAFQAZQByAHIAaQB0AG8AcgBpAGUAcwBfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEEAdQBzAHQAcgBhAGwAaQBhAG4AUwB0AGEAdABlAHMAVABlAHIAcgBpAHQAbwByAGkAZQBzAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAEEAUwBBADQAQQByAGUAYQBzAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAQQBTAEEANABBAHIAZQBhAHMAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBBAFMAQQA0AEEAcgBlAGEAcwBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBBAFMAQQA0AEEAcgBlAGEAcwBfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAQQBTAEEANABBAHIAZQBhAHMAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAZQB0AEEAbgBkAEQAcgB5AFoAbwBuAGUAcwBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAGUAdABBAG4AZABEAHIAeQBaAG8AbgBlAHMAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBlAHQAQQBuAGQARAByAHkAWgBvAG4AZQBzAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAGUAdABBAG4AZABEAHIAeQBaAG8AbgBlAHMAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAGUAdABBAG4AZABEAHIAeQBaAG8AbgBlAHMAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAGUAdABBAG4AZABEAHIAeQBaAG8AbgBlAHMAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbABpAG0AYQB0AGUAWgBvAG4AZQBzAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbABpAG0AYQB0AGUAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbABpAG0AYQB0AGUAWgBvAG4AZQBzAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbABpAG0AYQB0AGUAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBsAGkAbQBhAHQAZQBaAG8AbgBlAHMAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbABpAG0AYQB0AGUAWgBvAG4AZQBzAF8AQQBwAHAAZQBuAGQAaQBjAGUAcwAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBzAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAHMAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAcwBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAcwBfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAHMAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBzAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBzAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlAHMAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUAcwBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUAcwBfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlAHMAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBzAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBzAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlAHMAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlAHMAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBzAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQB0AGEAUwBjAG8AcgBlAHMAXwBTAGMAbwBwAGUAMwBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAdABhAFMAYwBvAHIAZQBzAF8AUwBjAG8AcABlADMAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAHQAYQBTAGMAbwByAGUAcwBfAFMAYwBvAHAAZQAzAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAdABhAFMAYwBvAHIAZQBzAF8AUwBjAG8AcABlADMAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAdABhAFMAYwBvAHIAZQBzAF8AUwBjAG8AcABlADMAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAdABhAFMAYwBvAHIAZQBzAF8AUwBjAG8AcABlADMAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMATABFAEEAQwBIAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMATABFAEEAQwBIAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAEwARQBBAEMASABfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMATABFAEEAQwBIAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMATABFAEEAQwBIAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAGwAZQBhAGMAaABfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAbABlAGEAYwBoAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAbABlAGEAYwBoAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAGwAZQBhAGMAaABfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBsAGUAYQBjAGgAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBsAGUAYQBjAGgAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBHAGUAdABBAHIAcgBhAHkAVABhAGIAbABlAFIAbwB3AFMAdABhAHIAdABOAHUAbQBiAGUAcgAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBHAGUAdABBAHIAcgBhAHkAVABhAGIAbABlAEMAbwBsAHUAbQBuAFMAdABhAHIAdABOAHUAbQBiAGUAcgAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBEAGkAcwBwAGwAYQB5AEEAcgByAGEAeQBJAG4AVABhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQBJAG4AVABhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQBJAG4AVABhAGIAbABlAE4AdQBtAGIAZQByACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAFMAcABsAGkAdABTAHQAcgBpAG4AZwBJAG4AdABvAEEAcgByAGEAeQAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBHAGUAdABDAGwAaQBtAGEAdABlAFoAbwBuAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8ATABvAG8AawB1AHAASQB0AGUAbQBGAHIAbwBtAE0AaQBuAE0AYQB4ACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAFMAdQBtAFEAdQBhAG4AdABpAHQAeQBGAHIAbwBtAEMAcgBpAHQAZQByAGkAYQAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAGcAZQB0AE8AdgBlAHIAbABhAHAAcABpAG4AZwBSAGUAcABvAHIAdABpAG4AZwBDAHkAYwBsAGUAcwAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAGcAZQB0AE8AdgBlAHIAbABhAHAAcABpAG4AZwBSAGUAcABvAHIAdABpAG4AZwBQAGUAcgBpAG8AZABzACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAEQAaQBzAHAAbABhAHkARgB1AG4AYwB0AGkAbwBuAE4AYQBtAGUAIgBdACwAIgBsAG8AYwBhAGwAZQAiADoAewAiAGwAaQBzAHQAUwBlAHAAYQByAGEAdABvAHIAIgA6ACIALAAiACwAIgByAG8AdwBTAGUAcABhAHIAYQB0AG8AcgAiADoAIgA7ACIALAAiAGMAbwBsAHUAbQBuAFMAZQBwAGEAcgBhAHQAbwByACIAOgAiACwAIgAsACIAdABoAG8AdQBzAGEAbgBkAHMAUwBlAHAAYQByAGEAdABvAHIAIgA6ACIALAAiACwAIgB0AGgAbwB1AHMAYQBuAGQAcwBQAG8AcwBpAHQAaQBvAG4AcwAiADoAWwAzAF0ALAAiAGQAZQBjAGkAbQBhAGwAUwBlAHAAYQByAGEAdABvAHIAIgA6ACIALgAiACwAIgBkAGEAdABlAE8AcgBkAGUAcgAiADoAIgBEAE0AWQAiACwAIgBjAHUAcgByAGUAbgBjAHkAUwB5AG0AYgBvAGwAIgA6ACIAJAAiACwAIgBpAHMAQwB1AHIAcgBlAG4AYwB5AFMAeQBtAGIAbwBsAEwAZQBhAGQAIgA6AHQAcgB1AGUALAAiAGkAcwBDAHUAcgByAGUAbgBjAHkAUwBlAHAAQgB5AFMAcABhAGMAZQAiADoAZgBhAGwAcwBlACwAIgByAG8AdwBMAGUAdAB0AGUAcgAiADoAIgBSACIALAAiAGMAbwBsAHUAbQBuAEwAZQB0AHQAZQByACIAOgAiAEMAIgAsACIAcgBjAEwAZQBmAHQAQgByAGEAYwBrAGUAdAAiADoAIgBbACIALAAiAHIAYwBSAGkAZwBoAHQAQgByAGEAYwBrAGUAdAAiADoAIgBdACIALAAiAHMAdABhAHQAZQBtAGUAbgB0AFMAZQBwAGEAcgBhAHQAbwByACIAOgAiADsAIgAsACIAbABvAGMAYQBsAGUATgBhAG0AZQAiADoAIgBlAG4ALQB1AHMAIgB9AH0A</AFEJSONBlob>
+<AFEJSONBlob xmlns="http://schemas.advancedformulaenvironment.officeapps.live.com/afejsonblob/1.0">ewAiAHMAYwBoAGUAbQBhACIAOgAiAGgAdAB0AHAAOgAvAC8AcwBjAGgAZQBtAGEAcwAuAGEAZAB2AGEAbgBjAGUAZABmAG8AcgBtAHUAbABhAGUAbgB2AGkAcgBvAG4AbQBlAG4AdAAuAG8AZgBmAGkAYwBlAGEAcABwAHMALgBsAGkAdgBlAC4AYwBvAG0ALwBhAGYAZQBwAHIAbwBqAGUAYwB0AHMALwAwAC4AMgAiACwAIgBmAGkAbABlAHMAIgA6AFsAewAiAHAAYQB0AGgAIgA6ACIALwBwAHIAbwBqAGUAYwB0AHMALwBXAG8AcgBrAGIAbwBvAGsAIgAsACIAdABlAHgAdAAiADoAIgAvAC8AIAAtAC0ALQAgAFcAbwByAGsAYgBvAG8AawAgAG0AbwBkAHUAbABlACAALQAtAC0AXABuAC8ALwAgAEEAIABmAGkAbABlACAAbwBmACAAbgBhAG0AZQAgAGQAZQBmAGkAbgBpAHQAaQBvAG4AcwAgAG8AZgAgAHQAaABlACAAZgBvAHIAbQA6AFwAbgAvAC8AIAAgACAAIABuAGEAbQBlACAAPQAgAGQAZQBmAGkAbgBpAHQAaQBvAG4AOwBcAG4AIgB9ACwAewAiAHAAYQB0AGgAIgA6ACIALwBwAHIAbwBqAGUAYwB0AHMALwBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAIgAsACIAdABlAHgAdAAiADoAIgAvACoAXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuAFMAbwB1AHIAYwBlACAAZABhAHQAYQAgAHQAaABhAHQAIABpAHMAIABjAG8AbQBtAG8AbgAgAGEAYwByAG8AcwBzACAAYQBsAGwAIABlAG4AdABlAHIAcAByAGkAcwBlACAAdAB5AHAAZQBzAFwAbgBFAHgAYwBlAGwAIABtAG8AZAB1AGwAZQAgAG4AYQBtAGUAOgAgAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBcAG4APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQBcAG4APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQBcAG4AKgAvAFwAbgBcAG4ALwAqAFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQBcAG4AUwBvAHUAcgBjAGUAOgAgAE4AYQB0AGkAbwBuAGEAbAAgAEkAbgB2AGUAbgB0AG8AcgB5ACAAUgBlAHAAbwByAHQAIAAyADAAMgAzACAAVgBvAGwAdQBtAGUAIAAxAFwAbgBOAEkAUgBfADIAMAAyADMAXwBWAG8AbAAxAFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQBcAG4AKgAvAFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABlAG4AcwBpAHQAeQBPAGYATQBlAHQAaABhAG4AZQBcAG4AcAAgAD0AIABkAGUAbgBzAGkAdAB5ACAAbwBmACAAbQBlAHQAaABhAG4AZQAgACgAMAAuADYANwA4ADQAIABrAGcALwBtADMAKQBcAG4AVABhAGsAZQBuACAAZgByAG8AbQAgAHQAaABlACAATgBhAHQAaQBvAG4AYQBsACAARwByAGUAZQBuAGgAbwB1AHMAZQAgAGEAbgBkACAARQBuAGUAcgBnAHkAIABSAGUAcABvAHIAdABpAG4AZwAgAFwAbgAoAE0AZQBhAHMAdQByAGUAbQBlAG4AdAApACAARABlAHQAZQByAG0AaQBuAGEAdABpAG8AbgAgADIAMAAwADgAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABlAG4AcwBpAHQAeQBPAGYATQBlAHQAaABhAG4AZQBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAcAAgAD0AIABkAGUAbgBzAGkAdAB5ACAAbwBmACAAbQBlAHQAaABhAG4AZQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABlAG4AcwBpAHQAeQBPAGYATQBlAHQAaABhAG4AZQBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAGsAZwAvAG0AMwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABlAG4AcwBpAHQAeQBPAGYATQBlAHQAaABhAG4AZQBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBOAGEAdABpAG8AbgBhAGwAIABJAG4AdgBlAG4AdABvAHIAeQAgAFIAZQBwAG8AcgB0ACAAMgAwADIAMwAgAFYAbwBsAHUAbQBlACAAMQA6ACAARQBxAHUAYQB0AGkAbwBuAHMAIAAzAC4AQgAuADEAYQBfADIALAAgADMALgBCAC4AMQBjAF8AMgAsACAAMwAuAEIALgAzAF8AMQAsACAAMwAuAEIALgA0AGcAXwAyAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGUAbgBzAGkAdAB5AE8AZgBNAGUAdABoAGEAbgBlAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKAAwAC4ANgA3ADgANAApADsAXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AE4AMgBvAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBDAGcAXABuAEMAZwAgAD0AIAA0ADQALwAyADgAIABmAGEAYwB0AG8AcgAgAHQAbwAgAGMAbwBuAHYAZQByAHQAIABlAGwAZQBtAGUAbgB0AGEAbAAgAG0AYQBzAHMAIABvAGYAIABOADIATwAgAHQAbwAgAG0AbwBsAGUAYwB1AGwAYQByACAAbQBhAHMAcwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AE4AMgBvAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBDAGcAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEYAYQBjAHQAbwByACAAdABvACAAYwBvAG4AdgBlAHIAdAAgAGUAbABlAG0AZQBuAHQAYQBsACAAbQBhAHMAcwAgAG8AZgAgAE4AMgBPACAAdABvACAAbQBvAGwAZQBjAHUAbABhAHIAIABtAGEAcwBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AE4AMgBvAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBDAGcAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEMAZwBOADIATwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABOADIAbwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAQwBnAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAZgBhAGMAdABvAHIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQATgAyAG8ARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAEMAZwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBOAGEAdABpAG8AbgBhAGwAIABJAG4AdgBlAG4AdABvAHIAeQAgAFIAZQBwAG8AcgB0ACAAMgAwADIAMwAgAFYAbwBsAHUAbQBlACAAMQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABOADIAbwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAQwBnAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKAA0ADQALwAyADgAKQA7AFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXABuAEYAYQBjAHQAbwByACAAdABvACAAYwBvAG4AdgBlAHIAdAAgAGUAbABlAG0AZQBuAHQAYQBsACAAbQBhAHMAcwAgAG8AZgAgAGcAYQBzACAAdABvACAAbQBvAGwAZQBjAHUAbABhAHIAIABtAGEAcwBzAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQARwBhAHMARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBGAGEAYwB0AG8AcgAgAHQAbwAgAGMAbwBuAHYAZQByAHQAIABlAGwAZQBtAGUAbgB0AGEAbAAgAG0AYQBzAHMAIABvAGYAIABnAGEAcwAgAHQAbwAgAG0AbwBsAGUAYwB1AGwAYQByACAAbQBhAHMAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEMAZwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBmAGEAYwB0AG8AcgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAWABYAFgAWABYAFgAWABcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAOAAsACAANAAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARwBhAHMAXAAiACwAIABcACIAQwBvAG4AdgBlAHIAcwBpAG8AbgAgAGYAYQBjAHQAbwByAFwAIgAsACAAXAAiAEMAbwBuAHYAZQByAHMAaQBvAG4AIABmAGEAYwB0AG8AcgAgADEAXAAiACwAIABcACIAQwBvAG4AdgBlAHIAcwBpAG8AbgAgAGYAYQBjAHQAbwByACAAMgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBPADIAXAAiACwAIABcACIANAA0AC8AMQAyAFwAIgAsACAANAA0ACwAIAAxADIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBIADQAXAAiACwAIABcACIAMQA2AC8AMQAyAFwAIgAsACAAMQA2ACwAIAAxADIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgAyAE8AXAAiACwAIABcACIANAA0AC8AMgA4AFwAIgAsACAANAA0ACwAIAAyADgAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgBvAHgAXAAiACwAIABcACIANAA2AC8AMQA0AFwAIgAsACAANAA2ACwAIAAxADQAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBPAFwAIgAsACAAXAAiADIAOAAvADEAMgBcACIALAAgADIAOAAsACAAMQAyADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMATwAyACAATABpAG0AZQBcACIALAAgAFwAIgA0ADQALwAxADIAXAAiACwAIAA0ADQALAAgADEAMgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOAE0AVgBPAEMAXAAiACwAIABcACIAMQA0AC8AMQAyAFwAIgAsACAAMQA0ACwAIAAxADIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEcAVwBQAE4AMgBPAFwAbgBHAGwAbwBiAGEAbAAgAHcAYQByAG0AaQBuAGcAIABwAG8AdABlAG4AdABpAGEAbAAgAGYAbwByACAAZwByAGUAZQBuAGgAbwB1AHMAZQAgAGcAYQBzAGUAcwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBHAFcAUABfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARwBsAG8AYgBhAGwAIAB3AGEAcgBtAGkAbgBnACAAcABvAHQAZQBuAHQAaQBhAGwAIABmAG8AcgAgAGcAcgBlAGUAbgBoAG8AdQBzAGUAIABnAGEAcwBlAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEcAVwBQAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBHAFcAUABOADIATwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARwBXAFAAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBmAGEAYwB0AG8AcgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARwBXAFAAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAWABYAFgAWABYAFgAWABcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARwBXAFAAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAOAAsACAAMgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARwBhAHMAXAAiACwAIABcACIAQwBPADIALQBlACAAZgBhAGMAdABvAHIAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMATwAyAFwAIgAsACAAMQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAEgANABcACIALAAgADIAOAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOADIATwBcACIALAAgADIANgA1ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMARgA0AFwAIgAsACAANgA2ADMAMAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDADIARgA2AFwAIgAsACAAMQAyADIAMAAwADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFMARgA2AFwAIgAsACAAMgAyADgAMAAwADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE4ARgAzAFwAIgAsACAAMQA3ADIAMAAwAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQQB1AHMAdAByAGEAbABpAGEAbgBTAHQAYQB0AGUAcwBUAGUAcgByAGkAdABvAHIAaQBlAHMAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQQB1AHMAdAByAGEAbABpAGEAbgBTAHQAYQB0AGUAcwBUAGUAcgByAGkAdABvAHIAaQBlAHMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEEAdQBzAHQAcgBhAGwAaQBhAG4AIABzAHQAYQB0AGUAcwAgAGEAbgBkACAAdABlAHIAcgBpAHQAbwByAGkAZQBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBBAHUAcwB0AHIAYQBsAGkAYQBuAFMAdABhAHQAZQBzAFQAZQByAHIAaQB0AG8AcgBpAGUAcwBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEEAdQBzAHQAcgBhAGwAaQBhAG4AUwB0AGEAdABlAHMAVABlAHIAcgBpAHQAbwByAGkAZQBzAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEEAdQBzAHQAcgBhAGwAaQBhAG4AUwB0AGEAdABlAHMAVABlAHIAcgBpAHQAbwByAGkAZQBzAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBBAHUAcwB0AHIAYQBsAGkAYQBuAFMAdABhAHQAZQBzAFQAZQByAHIAaQB0AG8AcgBpAGUAcwBfAEQAYQB0AGEAXABuACAAIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADkALAAgADMALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFMAdABhAHQAZQAvAFQAZQByAHIAaQB0AG8AcgB5AFwAIgAsACAAXAAiAEMAbwBtAG0AbwBuACAATgBhAG0AZQBcACIALAAgAFwAIgBBAGIAYgByAGUAdgBpAGEAdABpAG8AbgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgBlAHcAIABTAG8AdQB0AGgAIABXAGEAbABlAHMAXAAiACwAIABcACIATgBlAHcAIABTAG8AdQB0AGgAIABXAGEAbABlAHMAXAAiACwAIABcACIATgBTAFcAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEEAdQBzAHQAcgBhAGwAaQBhAG4AIABDAGEAcABpAHQAYQBsACAAVABlAHIAcgBpAHQAbwByAHkAXAAiACwAIABcACIAQQBDAFQAXAAiACwAIABcACIAQQBDAFQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFYAaQBjAHQAbwByAGkAYQBcACIALAAgAFwAIgBWAGkAYwB0AG8AcgBpAGEAXAAiACwAIABcACIAVgBJAEMAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFEAdQBlAGUAbgBzAGwAYQBuAGQAXAAiACwAIABcACIAUQB1AGUAZQBuAHMAbABhAG4AZABcACIALAAgAFwAIgBRAEwARABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUwBvAHUAdABoACAAQQB1AHMAdAByAGEAbABpAGEAXAAiACwAIABcACIAUwBvAHUAdABoACAAQQB1AHMAdAByAGEAbABpAGEAXAAiACwAIABcACIAUwBBAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGUAcwB0AGUAcgBuACAAQQB1AHMAdAByAGEAbABpAGEAXAAiACwAIABcACIAVwBlAHMAdABlAHIAbgAgAEEAdQBzAHQAcgBhAGwAaQBhAFwAIgAsACAAXAAiAFcAQQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVABhAHMAbQBhAG4AaQBhAFwAIgAsACAAXAAiAFQAYQBzAG0AYQBuAGkAYQBcACIALAAgAFwAIgBUAEEAUwBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgBvAHIAdABoAGUAcgBuACAAVABlAHIAcgBpAHQAbwByAHkAXAAiACwAIABcACIATgBvAHIAdABoAGUAcgBuACAAVABlAHIAcgBpAHQAbwByAHkAXAAiACwAIABcACIATgBUAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBBAFMAQQA0AEEAcgBlAGEAcwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAEEAUwBBADQAQQByAGUAYQBzAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBBAEIAUwAgAFMAdABhAHQAaQBzAHQAYwBhAGwAIABBAHIAZQBhAHMAIABMAGUAdgBlAGwAIAA0ACAALQAgAFcAZQBzAHQAZQByAG4AIABBAHUAcwB0AHIAYQBsAGkAYQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBBAFMAQQA0AEEAcgBlAGEAcwBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAQQBTAEEANABBAHIAZQBhAHMAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBBAFMAQQA0AEEAcgBlAGEAcwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBBAHUAcwB0AHIAYQBsAGkAYQBuACAAQgB1AHIAZQBhAHUAIABvAGYAIABTAHQAYQB0AGkAcwB0AGkAYwBzACAAKABBAEIAUwApACAALQAgAFMAdABhAHQAaQBzAHQAaQBjAGEAbAAgAEEAcgBlAGEAcwAgAEwAZQB2AGUAbAAgADIAIAAtACAAMgAwADIAMQAgAC0AIABTAGgAYQBwAGUAZgBpAGwAZQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBBAFMAQQA0AEEAcgBlAGEAcwBfAEQAYQB0AGEAXABuACAAIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADEAMQAsACAAMQAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUwBBACAANAAgAE4AYQBtAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEIAdQBuAGIAdQByAHkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE0AYQBuAGQAdQByAGEAaABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUABlAHIAdABoACAALQAgAEkAbgBuAGUAcgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUABlAHIAdABoACAALQAgAE4AbwByAHQAaAAgAEUAYQBzAHQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFAAZQByAHQAaAAgAC0AIABOAG8AcgB0AGgAIABXAGUAcwB0AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBQAGUAcgB0AGgAIAAtACAAUwBvAHUAdABoACAARQBhAHMAdABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUABlAHIAdABoACAALQAgAFMAbwB1AHQAaAAgAFcAZQBzAHQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAZQBzAHQAZQByAG4AIABBAHUAcwB0AHIAYQBsAGkAYQAgAC0AIABXAGgAZQBhAHQAIABCAGUAbAB0AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGUAcwB0AGUAcgBuACAAQQB1AHMAdAByAGEAbABpAGEAIAAtACAATwB1AHQAYgBhAGMAawAgACgATgBvAHIAdABoACkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAZQBzAHQAZQByAG4AIABBAHUAcwB0AHIAYQBsAGkAYQAgAC0AIABPAHUAdABiAGEAYwBrACAAKABTAG8AdQB0AGgAKQBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAZQB0AEEAbgBkAEQAcgB5AFoAbwBuAGUAcwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAGUAdABBAG4AZABEAHIAeQBaAG8AbgBlAHMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgAEEAdQBzAHQAcgBhAGwAaQBhAG4AIAB3AGUAdAAgAGEAbgBkACAAZAByAHkAIAB6AG8AbgBlAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAZQB0AEEAbgBkAEQAcgB5AFoAbwBuAGUAcwBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAZQB0AEEAbgBkAEQAcgB5AFoAbwBuAGUAcwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAGUAdABBAG4AZABEAHIAeQBaAG8AbgBlAHMAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAVABhAGIAbABlACAAMQAuADIAOgAgAFQAcgBhAG4AcwBsAGEAdABpAG4AZwAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAHMAIAB0AG8AIAB3AGUAdAAgAGEAbgBkACAAZAByAHkAIAB6AG8AbgBlAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAZQB0AEEAbgBkAEQAcgB5AFoAbwBuAGUAcwBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAzACwAIAAxACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBWAEEAUgBJAEEAVABJAE8ATgAgAE8ARgAgAFMATwBVAFIAQwBFACAARABBAFQAQQA6AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBBAGQAZABlAGQAIAB3AGEAcgBtACAALwAgAGMAbwBvAGwAIAB0AGUAbQBwAGUAcgBhAHQAZQAgAG0AbwBpAHMAdAAgAC8AIABkAHIAeQAgAC0AIABsAG8AdwAgAGYAcgBvAHMAdAAgAGEAbgBkACAAaABpAGcAaAAgAHQAZQBtAHAAIABjAGwAYQBzAHMAZQBzACAAdABvACAAYQBjAGMAbwBtAG0AbwBkAGEAdABlACAAYwBsAGkAbQBhAHQAZQAgAHMAYwBlAG4AYQByAGkAbwBzACAAZQB4AGMAbAB1AGQAZQBkACAAYgB5ACAAVgBFAEUAUgBHACAAYwByAGkAdABlAHIAaQBhAC4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEYAaQB4AGUAZAAgAHQAeQBwAG8AIAAtACAAQwBoAGEAbgBnAGUAZAAgAFwAdQAwADAAMgA3AEYAcgB5AFwAdQAwADAAMgA3ACAAdABvACAAXAB1ADAAMAAyADcARAByAHkAXAB1ADAAMAAyADcALgBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAZQB0AEEAbgBkAEQAcgB5AFoAbwBuAGUAcwBfAEQAYQB0AGEAXABuACAAIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADEANQAsACAAMgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBsAGkAbQBhAHQAZQAgAFoAbwBuAGUAXAAiACwAIABcACIAVwBlAHQAIABvAHIAIABEAHIAeQAgAFoAbwBuAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAcgBvAHAAaQBjAGEAbAAgAG0AbwBuAHQAYQBuAGUAXAAiACwAIABcACIAVwBlAHQAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVAByAG8AcABpAGMAYQBsACAAdwBlAHQAXAAiACwAIABcACIAVwBlAHQAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVAByAG8AcABpAGMAYQBsACAAbQBvAGkAcwB0AFwAIgAsACAAXAAiAFcAZQB0ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAcgBvAHAAaQBjAGEAbAAgAGQAcgB5AFwAIgAsACAAXAAiAEQAcgB5ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAYQByAG0AIAB0AGUAbQBwAGUAcgBhAHQAZQAgAG0AbwBpAHMAdABcACIALAAgAFwAIgBXAGUAdAAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGEAcgBtACAAdABlAG0AcABlAHIAYQB0AGUAIABkAHIAeQBcACIALAAgAFwAIgBEAHIAeQAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AbwBsACAAdABlAG0AcABlAHIAYQB0AGUAIABtAG8AaQBzAHQAXAAiACwAIABcACIAVwBlAHQAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBvAG8AbAAgAHQAZQBtAHAAZQByAGEAdABlACAAZAByAHkAXAAiACwAIABcACIARAByAHkAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBhAHIAbQAgAHQAZQBtAHAAZQByAGEAdABlACAAbQBvAGkAcwB0ACAALQAgAGwAbwB3ACAAZgByAG8AcwB0AFwAIgAsACAAXAAiAFcAZQB0ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAYQByAG0AIAB0AGUAbQBwAGUAcgBhAHQAZQAgAGQAcgB5ACAALQAgAGwAbwB3ACAAZgByAG8AcwB0AFwAIgAsACAAXAAiAEQAcgB5ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAYQByAG0AIAB0AGUAbQBwAGUAcgBhAHQAZQAgAG0AbwBpAHMAdAAgAC0AIABoAGkAZwBoACAAdABlAG0AcABcACIALAAgAFwAIgBXAGUAdAAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGEAcgBtACAAdABlAG0AcABlAHIAYQB0AGUAIABkAHIAeQAgAC0AIABoAGkAZwBoACAAdABlAG0AcABcACIALAAgAFwAIgBEAHIAeQAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AbwBsACAAdABlAG0AcABlAHIAYQB0AGUAIABtAG8AaQBzAHQAIAAtACAAbABvAHcAIABmAHIAbwBzAHQAXAAiACwAIABcACIAVwBlAHQAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBvAG8AbAAgAHQAZQBtAHAAZQByAGEAdABlACAAZAByAHkAIAAtACAAbABvAHcAIABmAHIAbwBzAHQAXAAiACwAIABcACIARAByAHkAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbABpAG0AYQB0AGUAWgBvAG4AZQBzAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbABpAG0AYQB0AGUAWgBvAG4AZQBzAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIABBAHUAcwB0AHIAYQBsAGkAYQBuACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBsAGkAbQBhAHQAZQBaAG8AbgBlAHMAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABUAGEAYgBsAGUAIAAxAC4AMwA6ACAAQwBsAGkAbQBhAHQAZQAgAGEAbgBkACAAUgBhAGkAbgBmAGEAbABsACAAegBvAG4AZQAgAGMAbABhAHMAcwBpAGYAaQBjAGEAdABpAG8AbgBzACAAYQBuAGQAIABkAGUAZgBpAG4AaQB0AGkAbwBuAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbABpAG0AYQB0AGUAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADUALAAgADEALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFYAQQBSAEkAQQBUAEkATwBOACAATwBGACAAUwBPAFUAUgBDAEUAIABEAEEAVABBADoAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEEAZABkAGUAZAAgAHcAYQByAG0AIAAvACAAYwBvAG8AbAAgAHQAZQBtAHAAZQByAGEAdABlACAAbQBvAGkAcwB0ACAALwAgAGQAcgB5ACAALQAgAGwAbwB3ACAAZgByAG8AcwB0ACAAYQBuAGQAIABoAGkAZwBoACAAdABlAG0AcAAgAGMAbABhAHMAcwBlAHMAIAB0AG8AIABhAGMAYwBvAG0AbQBvAGQAYQB0AGUAIABjAGwAaQBtAGEAdABlACAAcwBjAGUAbgBhAHIAaQBvAHMAIABlAHgAYwBsAHUAZABlAGQAIABiAHkAIABWAEUARQBSAEcAIABjAHIAaQB0AGUAcgBpAGEALgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARgBpAHgAZQBkACAAdAB5AHAAbwAgAGkAbgAgAE0AQQBUACAAdgBhAGwAdQBlACAAZgBvAHIAIAB3AGEAcgBtACAAdABlAG0AcABlAHIAYQB0AGUAIABkAHIAeQAgAC0AIABjAGgAYQBuAGcAZQBkACAAMQAwACAAdABvACAAMQAxAC4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEEAZABkAGUAZAAgAG0AaQBuACAAYQBuAGQAIABtAGEAeAAgAGMAbwBsAHUAbQBuAHMAIABmAG8AcgAgAE0AQQBUACwAIABNAEEAUAAsACAAZgByAG8AcwB0ACAAZABhAHkAcwAgAHAAZQByACAAeQBlAGEAcgAsACAAZQBsAGUAdgBhAHQAaQBvAG4ALAAgAE0AQQBQADoAUABFAFQAIAB0AG8AIABjAGEAbABjAHUAbABhAHQAZQAgAHoAbwBuAGUAcwAgAGYAcgBvAG0AIAByAGUAYQBsACAAYwBsAGkAbQBhAHQAZQAgAGQAYQB0AGEALgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARwBBAEYAIABhAGMAYwBlAHAAdABzACAAcgBhAGkAbgBmAGEAbABsACAAYQBzACAAYQAgAHAAcgBvAHgAeQAgAGYAbwByACAAcAByAGUAYwBpAHAAaQB0AGEAdABpAG8AbgAuAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBsAGkAbQBhAHQAZQBaAG8AbgBlAHMAXwBEAGEAdABhAFwAbgAgACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAA5ACwAIAAxADYALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAbABpAG0AYQB0AGUAIABaAG8AbgBlAFwAIgAsACAAXAAiAE0AQQBUAFwAIgAsACAAXAAiAE0AQQBQAFwAIgAsACAAXAAiAEYAcgBvAHMAdAAgAGQAYQB5AHMAIABwAGUAcgAgAHkAZQBhAHIAXAAiACwAIABcACIARQBsAGUAdgBhAHQAaQBvAG4AXAAiACwAIABcACIATQBBAFAAOgBQAEUAVABcACIALAAgAFwAIgBNAGkAbgAgAHQAZQBtAHAAXAAiACwAIABcACIATQBhAHgAIAB0AGUAbQBwAFwAIgAsACAAXAAiAE0AaQBuACAAcgBhAGkAbgBmAGEAbABsAFwAIgAsACAAXAAiAE0AYQB4ACAAcgBhAGkAbgBmAGEAbABsAFwAIgAsACAAXAAiAE0AaQBuACAAZgByAG8AcwB0ACAAZABhAHkAcwBcACIALAAgAFwAIgBNAGEAeAAgAGYAcgBvAHMAdAAgAGQAYQB5AHMAXAAiACwAIABcACIATQBpAG4AIABlAGwAZQB2AGEAdABpAG8AbgBcACIALAAgAFwAIgBNAGEAeAAgAGUAbABlAHYAYQB0AGkAbwBuAFwAIgAsACAAXAAiAE0AaQBuACAATQBBAFAAOgBQAEUAVABcACIALAAgAFwAIgBNAGkAbgAgAE0AQQBQADoAUABFAFQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAcgBvAHAAaQBjAGEAbAAgAG0AbwBuAHQAYQBuAGUAXAAiACwAIABcACIAXAB1ADAAMAAzAGUAIAAxADgAIABDAFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAGQiIAA3AFwAIgAsACAAXAAiAFwAdQAwADAAMwBlACAAMQAwADAAMAAgAG0AXAAiACwAIABcACIAQQBuAHkAXAAiACwAIAAxADgALgAwADAAMQAsACAAOQA5ADkAOQA5ADkALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA3ACwAIAAxADAAMAAwACwAIAA5ADkAOQA5ADkAOQAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVAByAG8AcABpAGMAYQBsACAAdwBlAHQAXAAiACwAIABcACIAXAB1ADAAMAAzAGUAIAAxADgAIABDAFwAIgAsACAAXAAiAFwAdQAwADAAMwBlACAAMgAwADAAMAAgAG0AbQBcACIALAAgAFwAIgBkIiAANwBcACIALAAgAFwAIgBkIiAAMQAwADAAMAAgAG0AXAAiACwAIABcACIAQQBuAHkAXAAiACwAIAAxADgALgAwADAAMQAsACAAOQA5ADkAOQA5ADkALAAgADIAMAAwADAALgAwADAAMQAsACAAOQA5ADkAOQA5ADkALAAgAC0AOQA5ADkAOQA5ADkALAAgADcALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5AC4AOQA5ADkALAAgACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVAByAG8AcABpAGMAYQBsACAAbQBvAGkAcwB0AFwAIgAsACAAXAAiAFwAdQAwADAAMwBlACAAMQA4ACAAQwBcACIALAAgAFwAIgBcAHUAMAAwADMAZQAgADEAMAAwADAAIABtAG0AIAAtACAAZCIgADIAMAAwADAAIABtAG0AXAAiACwAIABcACIAZCIgADcAXAAiACwAIABcACIAZCIgADEAMAAwADAAIABtAFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAMQA4AC4AMAAwADEALAAgADkAOQA5ADkAOQA5ACwAIAAxADAAMAAwAC4AMAAwADEALAAgADIAMAAwADAALAAgAC0AOQA5ADkAOQA5ADkALAAgADcALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5AC4AOQA5ADkALAAgACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVAByAG8AcABpAGMAYQBsACAAZAByAHkAXAAiACwAIABcACIAXAB1ADAAMAAzAGUAIAAxADgAIABDAFwAIgAsACAAXAAiAGQiIAAxADAAMAAwACAAbQBtAFwAIgAsACAAXAAiAGQiIAA3AFwAIgAsACAAXAAiAGQiIAAxADAAMAAwACAAbQBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgADEAOAAuADAAMAAxACwAIAA5ADkAOQA5ADkAOQAsACAALQA5ADkAOQA5ADkAOQAsACAAMQAwADAAMAAsACAALQA5ADkAOQA5ADkAOQAsACAANwAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkALgA5ADkAOQAsACAAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQA5ADkAOQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGEAcgBtACAAdABlAG0AcABlAHIAYQB0AGUAIABtAG8AaQBzAHQAXAAiACwAIABcACIAXAB1ADAAMAAzAGUAIAAxADAAIABDAFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAFwAdQAwADAAMwBlACAAMQBcACIALAAgADEAMAAuADAAMAAxACwAIAA5ADkAOQA5ADkAOQAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQA5ADkAOQAsACAAMQAuADAAMAAxACwAIAA5ADkAOQA5ADkAOQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGEAcgBtACAAdABlAG0AcABlAHIAYQB0AGUAIABkAHIAeQBcACIALAAgAFwAIgBcAHUAMAAwADMAZQAgADEAMAAgAEMAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAZCIgADEAXAAiACwAIAAxADAALgAwADAAMQAsACAAOQA5ADkAOQA5ADkALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQA5ADkAOQAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkALAAgACAALQA5ADkAOQA5ADkAOQAsACAAMQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AbwBsACAAdABlAG0AcABlAHIAYQB0AGUAIABtAG8AaQBzAHQAXAAiACwAIABcACIAXAB1ADAAMAAzAGUAIAAwACAAQwAgAC0AIABkIiAAMQAwACAAQwBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBcAHUAMAAwADMAZQAgADEAXAAiACwAIAAtADkAOQA5ADkAOQA5ACwAIAAxADAALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQA5ADkAOQAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkALAAgADEALgAwADAAMQAsACAAOQA5ADkAOQA5ADkAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBvAG8AbAAgAHQAZQBtAHAAZQByAGEAdABlACAAZAByAHkAXAAiACwAIABcACIAXAB1ADAAMAAzAGUAIAAwACAAQwAgAC0AIABkIiAAMQAwACAAQwBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBkIiAAMQBcACIALAAgAC0AOQA5ADkAOQA5ADkALAAgADEAMAAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQA5ADkAOQAsACAAIAAtADkAOQA5ADkAOQA5ACwAIAAxAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAEEAcABwAGUAbgBkAGkAYwBlAHMAXABuACAAIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADQALAAgADEALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE4AbwB0AGUAOgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATQBBAFQAIAA9ACAAbQBlAGEAbgAgAGEAbgBuAHUAYQBsACAAdABlAG0AcABlAHIAYQB0AHUAcgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBNAEEAUAAgAD0AIABtAGUAYQBuACAAYQBuAG4AdQBhAGwAIABwAHIAZQBjAGkAcABpAHQAYQB0AGkAbwBuAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBQAEUAVAAgAD0AIABwAG8AdABlAG4AdABpAGEAbAAgAGUAdgBhAHAAbwB0AHIAYQBuAHMAcABpAHIAYQB0AGkAbwBuAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAHMAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAcwBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAQQB1AHMAdAByAGEAbABpAGEAbgAgAHQAZQBtAHAAZQByAGEAdAB1AHIAZQAgAHoAbwBuAGUAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAcwBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAHMAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAcwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABUAGEAYgBsAGUAIAAxAC4AMwA6ACAAQwBsAGkAbQBhAHQAZQAgAGEAbgBkACAAUgBhAGkAbgBmAGEAbABsACAAegBvAG4AZQAgAGMAbABhAHMAcwBpAGYAaQBjAGEAdABpAG8AbgBzACAAYQBuAGQAIABkAGUAZgBpAG4AaQB0AGkAbwBuAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAHMAXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBBAFIASQBBAFQASQBPAE4AIABPAEYAIABTAE8AVQBSAEMARQAgAEQAQQBUAEEAOgAgAEEAZABkAGUAZAAgAGUAeAB0AHIAYQAgAE0AQQBUACAAbQBpAG4AIABhAG4AZAAgAE0AQQBUACAAbQBhAHgAIABjAG8AbAB1AG0AbgBzACAAdABvACAAYwBhAGwAYwB1AGwAYQB0AGUAIAB6AG8AbgBlACAAZgByAG8AbQAgAHIAZQBhAGwAIAB0AGUAbQBwAGUAcgBhAHQAdQByAGUAIABkAGEAdABhAC4AXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAHMAXwBEAGEAdABhAFwAbgAgACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAA0ACwAIAA0ACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAGUAbQBwAGUAcgBhAHQAdQByAGUAIABaAG8AbgBlAFwAIgAsACAAXAAiAE0AZQBkAGkAYQBuACAAQQBuAG4AdQBhAGwAIABUAGUAbQBwAGUAcgBhAHQAdQByAGUAIAAoAE0AQQBUACkAXAAiACwAIABcACIATQBpAG4AIABNAEEAVABcACIALAAgAFwAIgBNAGEAeAAgAE0AQQBUAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGEAcgBtAFwAIgAsACAAXAAiAGUiIAAyADYAIABDAFwAIgAsACAAMgA2ACwAIAA5ADkAOQA5ADkAOQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAGUAbQBwAGUAcgBhAHQAZQBcACIALAAgAFwAIgAxADUAIAAtACAAMgA1ACAAQwBcACIALAAgADEANQAsACAAMgA1AC4AOQA5ADkAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBvAG8AbABcACIALAAgAFwAIgBkIiAAMQA0ACAAQwBcACIALAAgAC0AOQA5ADkAOQA5ADkALAAgADEANAAuADkAOQA5AFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBzAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlAHMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgAEEAdQBzAHQAcgBhAGwAaQBhAG4AIAByAGEAaQBuAGYAYQBsAGwAIAB6AG8AbgBlAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlAHMAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBzAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlAHMAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAVABhAGIAbABlACAAMQAuADMAOgAgAEMAbABpAG0AYQB0AGUAIABhAG4AZAAgAFIAYQBpAG4AZgBhAGwAbAAgAHoAbwBuAGUAIABjAGwAYQBzAHMAaQBmAGkAYwBhAHQAaQBvAG4AcwAgAGEAbgBkACAAZABlAGYAaQBuAGkAdABpAG8AbgBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYAQQBSAEkAQQBUAEkATwBOACAATwBGACAAUwBPAFUAUgBDAEUAIABEAEEAVABBADoAIABBAGQAZABlAGQAIABlAHgAdAByAGEAIABSAGEAaQBuAGYAYQBsAGwAIABtAGkAbgAgAGEAbgBkACAAUgBhAGkAbgBmAGEAbABsACAAbQBhAHgAIABjAG8AbAB1AG0AbgBzACAAdABvACAAYwBhAGwAYwB1AGwAYQB0AGUAIAB6AG8AbgBlACAAZgByAG8AbQAgAHIAZQBhAGwAIAByAGEAaQBuAGYAYQBsAGwAIABkAGEAdABhAC4AXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlAHMAXwBEAGEAdABhAFwAbgAgACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAzACwAIAA0ACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBSAGEAaQBuAGYAYQBsAGwAIABaAG8AbgBlAFwAIgAsACAAXAAiAEEAbgBuAHUAYQBsACAAcgBhAGkAbgBmAGEAbABsAFwAIgAsACAAXAAiAFIAYQBpAG4AZgBhAGwAbAAgAG0AaQBuAFwAIgAsACAAXAAiAFIAYQBpAG4AZgBhAGwAbAAgAG0AYQB4AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBIAGkAZwBoACAAcgBhAGkAbgBmAGEAbABsAFwAIgAsACAAXAAiAEEAbgBuAHUAYQBsACAAcgBhAGkAbgBmAGEAbABsACAAXAB1ADAAMAAzAGUAIAA2ADAAMABtAG0AXAAiACwAIAA2ADAAMAAuADAAMAAxACwAIAA5ADkAOQA5ADkAOQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBMAG8AdwAgAHIAYQBpAG4AZgBhAGwAbABcACIALAAgAFwAIgBBAG4AbgB1AGEAbAAgAHIAYQBpAG4AZgBhAGwAbAAgAGQiIAA2ADAAMABtAG0AXAAiACwAIAAtADkAOQA5ADkAOQA5ACwAIAA2ADAAMABcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBzAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIABBAHUAcwB0AHIAYQBsAGkAYQBuACAAbABlAGEAYwBoAGkAbgBnACAAegBvAG4AZQBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBzAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgAFQAYQBiAGwAZQAgADEALgAzADoAIABDAGwAaQBtAGEAdABlACAAYQBuAGQAIABSAGEAaQBuAGYAYQBsAGwAIAB6AG8AbgBlACAAYwBsAGEAcwBzAGkAZgBpAGMAYQB0AGkAbwBuAHMAIABhAG4AZAAgAGQAZQBmAGkAbgBpAHQAaQBvAG4AcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBfAEQAYQB0AGEAXABuACAAIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADQALAAgADIALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEwAZQBhAGMAaABpAG4AZwAgAFoAbwBuAGUAXAAiACwAIABcACIATABlAGEAYwBoAGkAbgBnACAAYwByAGkAdABlAHIAaQBhAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBMAGUAYQBjAGgAaQBuAGcAIABvAGMAYwB1AHIAcwBcACIALAAgAFwAIgCjAygANdhf3DXYTtw12FbcNdhb3CkAXAB1ADAAMAAzAGUAowMoADXYONw12EfcMAApACsANdhg3DXYXNw12FbcNdhZ3CAANdhk3DXYTtw12GHcNdhS3DXYX9wgAA4hNdhc3DXYWdw12FHcNdhW3DXYW9w12FTcIAA12FDcNdhO3DXYXdw12E7cNdhQ3DXYVtw12GHcNdhm3FwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBMAGUAYQBjAGgAaQBuAGcAIABkAG8AZQBzACAAbgBvAHQAIABvAGMAYwB1AHIAXAAiACwAIABcACIAowMoADXYX9w12E7cNdhW3DXYW9wpAGQiowMoADXYONw12EfcMAApACsANdhg3DXYXNw12FbcNdhZ3CAANdhk3DXYTtw12GHcNdhS3DXYX9wgAA4hNdhc3DXYWdw12FHcNdhW3DXYW9w12FTcIAA12FDcNdhO3DXYXdw12E7cNdhQ3DXYVtw12GHcNdhm3FwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABcAG4ANQAuADUALgAyAC4AMwAgAEMAbwBuAHMAdABhAG4AdAAgAFAAYQByAGEAbQBlAHQAZQByAHMAXABuAEYAcgBhAGMAdABpAG8AbgAgAG8AZgAgAE4AIAB0AGgAYQB0ACAAaQBzACAAYQB2AGEAaQBsAGEAYgBsAGUAIABmAG8AcgAgAGwAZQBhAGMAaABpAG4AZwAgAGEAbgBkACAAcgB1AG4AbwBmAGYAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARgByAGEAYwB0AGkAbwBuACAAbwBmACAATgAgAHQAaABhAHQAIABpAHMAIABhAHYAYQBpAGwAYQBiAGwAZQAgAGYAbwByACAAbABlAGEAYwBoAGkAbgBnACAAYQBuAGQAIAByAHUAbgBvAGYAZgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiACgARABpAG0AZQBuAHMAaQBvAG4AbABlAHMAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoANQAuADUALgAyAC4AMwAgAEMAbwBuAHMAdABhAG4AdAAgAFAAYQByAGEAbQBlAHQAZQByAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMwAsACAAMgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIASQBzACAAaQBuACAAbABlAGEAYwBoAGkAbgBnACAAegBvAG4AZQBcACIALABcACIARgByAGEAYwBXAEUAVABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAWQBlAHMAIAAtACAAaQBuACAAbABlAGEAYwBoAGkAbgBnACAAegBvAG4AZQBcACIALAAgADEAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgBvACAALQAgAG4AbwB0ACAAaQBuACAAbABlAGEAYwBoAGkAbgBnACAAegBvAG4AZQBcACIALAAgADAAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuACAAIABDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAKABcACIAXAAiACkAKQA7AFwAbgBcAG4AXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAdABhAFMAYwBvAHIAZQBzAF8AUwBjAG8AcABlADMAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAHQAYQBTAGMAbwByAGUAcwBfAFMAYwBvAHAAZQAzAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBBAHUAcwB0AHIAYQBsAGkAYQBuACAAZABhAHQAYQAgAHMAYwBvAHIAZQBzACAAZgBvAHIAIABzAGMAbwBwAGUAIAAzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAdABhAFMAYwBvAHIAZQBzAF8AUwBjAG8AcABlADMAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAdABhAFMAYwBvAHIAZQBzAF8AUwBjAG8AcABlADMAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAHQAYQBTAGMAbwByAGUAcwBfAFMAYwBvAHAAZQAzAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgAFgAWABYAFgAWABYAFgAWABcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAHQAYQBTAGMAbwByAGUAcwBfAFMAYwBvAHAAZQAzAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAdABhAFMAYwBvAHIAZQBzAF8AUwBjAG8AcABlADMAXwBEAGEAdABhAFwAbgAgACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAA2ACwAIAAyACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBEAGEAdABhACAAcwBvAHUAcgBjAGUAXAAiACwAIABcACIARABhAHQAYQAgAHMAYwBvAHIAZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIASQBuAHQAZQByAG4AYQB0AGkAbwBuAGEAbAAgAHMAYwBvAHAAZQAgADMAIABkAGEAdABhAGIAYQBzAGUAXAAiACwAIAAxADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEEAdQBzAHQAcgBhAGwAaQBhAG4AIABzAGMAbwBwAGUAIAAzACAAZABhAHQAYQBiAGEAcwBlAFwAIgAsACAAMgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBTAHQAYQB0AGUAIABvAHIAIAByAGUAZwBpAG8AbgBhAGwAIABzAGMAbwBwAGUAIAAzACAAZABhAHQAYQBiAGEAcwBlAFwAIgAsACAAMwA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBFAG0AaQBzAHMAaQBvAG4AcwAgAGkAbgB0AGUAbgBzAGkAdAB5ACAAYwBhAGwAYwB1AGwAYQB0AGUAZAAgAGYAcgBvAG0AIABhAHAAcAByAG8AdgBlAGQAIABtAGUAdABoAG8AZABcACIALAAgADQAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVgBlAHIAaQBmAGkAZQBkACAAYwByAGUAZABlAG4AdABpAGEAbAAgAG0AYQB0AGMAaABpAG4AZwAgAEkAUwBPADEANAAwADYANwBcACIALAAgADUAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAFwAbgAgACAALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBMAEUAQQBDAEgAXABuADUALgA1AC4AMgAuADMAIABDAG8AbgBzAHQAYQBuAHQAIABQAGEAcgBhAG0AZQB0AGUAcgBzAFwAbgBGAHIAYQBjAHQAaQBvAG4AIABvAGYAIABOACAAdABoAGEAdAAgAGkAcwAgAGEAdgBhAGkAbABhAGIAbABlACAAZgBvAHIAIABsAGUAYQBjAGgAaQBuAGcAIABhAG4AZAAgAHIAdQBuAG8AZgBmAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMATABFAEEAQwBIAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBGAHIAYQBjAHQAaQBvAG4AIABvAGYAIABOACAAdABoAGEAdAAgAGkAcwAgAGEAdgBhAGkAbABhAGIAbABlACAAZgBvAHIAIABsAGUAYQBjAGgAaQBuAGcAIABhAG4AZAAgAHIAdQBuAG8AZgBmAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAEwARQBBAEMASABfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiACgARABpAG0AZQBuAHMAaQBvAG4AbABlAHMAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ADUALgA1AC4AMgAuADMAIABDAG8AbgBzAHQAYQBuAHQAIABQAGEAcgBhAG0AZQB0AGUAcgBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAEwARQBBAEMASABfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBOAGEAdABpAG8AbgBhAGwAIABJAG4AdgBlAG4AdABvAHIAeQAgAFIAZQBwAG8AcgB0ACAAVgBvAGwAdQBtAGUAIAAxADoAIABMAGUAYQBjAGgAaQBuAGcAIABhAG4AZAAgAHIAdQBuAG8AZgBmACAAKAAzAC4ARAAuAGIALgAyACkAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMATABFAEEAQwBIAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADEALAAgADIALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEYAcgBhAGMATABFAEEAQwBIAFwAIgAsADAALgAyADQAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuACAAIABDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAEwARQBBAEMASABfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoACgAXAAiAFwAIgApACkAOwBcAG4AXABuAFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAGwAZQBhAGMAaABcAG4ANQAuADUALgAyAC4AMwAgAEMAbwBuAHMAdABhAG4AdAAgAFAAYQByAGEAbQBlAHQAZQByAHMAXABuAEUAbQBpAHMAcwBpAG8AbgAgAGYAYQBjAHQAbwByACAAZgBvAHIAIABuAGkAdAByAG8AZwBlAG4AIABsAGUAYQBjAGgAaQBuAGcAIABhAG4AZAAgAHIAdQBuAG8AZgBmAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBsAGUAYQBjAGgAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEUAbQBpAHMAcwBpAG8AbgAgAGYAYQBjAHQAbwByACAAZgBvAHIAIABuAGkAdAByAG8AZwBlAG4AIABsAGUAYQBjAGgAaQBuAGcAIABhAG4AZAAgAHIAdQBuAG8AZgBmAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAbABlAGEAYwBoAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAKABrAGcAIABOADIATwAtAE4AIAAvACAAawBnACAATgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAGwAZQBhAGMAaABfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoANQAuADUALgAyAC4AMwAgAEMAbwBuAHMAdABhAG4AdAAgAFAAYQByAGEAbQBlAHQAZQByAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBsAGUAYQBjAGgAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIATgBhAHQAaQBvAG4AYQBsACAASQBuAHYAZQBuAHQAbwByAHkAIABSAGUAcABvAHIAdAAgAFYAbwBsAHUAbQBlACAAMQA6ACAARQBxAHUAYQB0AGkAbwBuACAAMwAuAEQALgBCAF8AMQAwAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAbABlAGEAYwBoAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADEALAAgADIALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEUARgBsAGUAYQBjAGgAXAAiACwAMAAuADAAMQAxAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgAgACAAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAGwAZQBhAGMAaABfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoACgAXAAiAFwAIgApACkAOwBcAG4AXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATgAyAE8AXABuAFQAYQBiAGwAZQAgAEEALgAyAC4AMgAuADEAXABuAE4AaQB0AHIAbwB1AHMAIABvAHgAaQBkAGUAIABlAG0AaQBzAHMAaQBvAG4AIABmAGEAYwB0AG8AcgBzACAAZgBvAHIAIABpAG4AbwByAGcAYQBuAGkAYwAgAGYAZQByAHQAaQBsAGkAcwBlAHIAIABhAHAAcABsAGkAYwBhAHQAaQBvAG4AIAAoAGsAZwAgAE4AMgBPAC0ATgAvAGsAZwAgAE4AKQAgACgARQBGAE4AMgBPACkAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE4AMgBPAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBOAGkAdAByAG8AdQBzACAAbwB4AGkAZABlACAAZQBtAGkAcwBzAGkAbwBuACAAZgBhAGMAdABvAHIAcwAgAGYAbwByACAAaQBuAG8AcgBnAGEAbgBpAGMAIABmAGUAcgB0AGkAbABpAHMAZQByACAAYQBwAHAAbABpAGMAYQB0AGkAbwBuAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATgAyAE8AXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgAoAGsAZwAgAE4AMgBPAC0ATgAgAC8AIABrAGcAIABOAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATgAyAE8AXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAVABhAGIAbABlACAAQQAuADIALgAyAC4AMQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE4AMgBPAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATgAyAE8AXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMQA1ACwAIAA1ACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBQAHIAbwBkAHUAYwB0AGkAbwBuACAAcwB5AHMAdABlAG0AIABqAFwAIgAsAFwAIgBFAEYATgAyAE8AXAAiACwAIABcACIAUAByAG8AZAB1AGMAdABpAG8AbgAgAHMAeQBzAHQAZQBtACAAbwBuAGwAeQBcACIALAAgAFwAIgBJAHIAcgBpAGcAYQB0AGkAbwBuACAAbQBlAHQAaABvAGQAXAAiACwAIABcACIAUgBhAGkAbgBmAGEAbABsACAAegBvAG4AZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIASQByAHIAaQBnAGEAdABlAGQAIABwAGEAcwB0AHUAcgBlAFwAIgAsADAALgAwADAANQA5ACwAIABcACIAUABhAHMAdAB1AHIAZQBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBBAG4AeQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIASQByAHIAaQBnAGEAdABlAGQAIABjAHIAbwBwAFwAIgAsADAALgAwADAANwAsACAAXAAiAEMAcgBvAHAAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAQQBuAHkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE4AbwBuAC0AaQByAHIAaQBnAGEAdABlAGQAIABwAGEAcwB0AHUAcgBlAFwAIgAsADAALgAwADAAMQA4ACwAIABcACIAUABhAHMAdAB1AHIAZQBcACIALAAgAFwAIgBOAG8AdAAgAGkAcgByAGkAZwBhAHQAZQBkAFwAIgAsACAAXAAiAEwAbwB3ACAAcgBhAGkAbgBmAGEAbABsAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOAG8AbgAtAGkAcgByAGkAZwBhAHQAZQBkACAAcABhAHMAdAB1AHIAZQBcACIALAAwAC4AMAAwADEAOAAsACAAXAAiAFAAYQBzAHQAdQByAGUAXAAiACwAIABcACIATgBvAHQAIABpAHIAcgBpAGcAYQB0AGUAZABcACIALAAgAFwAIgBIAGkAZwBoACAAcgBhAGkAbgBmAGEAbABsAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOAG8AbgAtAGkAcgByAGkAZwBhAHQAZQBkACAAYwByAG8AcAAgACgAbABvAHcAIAByAGEAaQBuAGYAYQBsAGwAKQBcACIALAAwAC4AMAAwADIAOQAsACAAXAAiAEMAcgBvAHAAXAAiACwAIABcACIATgBvAHQAIABpAHIAcgBpAGcAYQB0AGUAZABcACIALAAgAFwAIgBMAG8AdwAgAHIAYQBpAG4AZgBhAGwAbABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgBvAG4ALQBpAHIAcgBpAGcAYQB0AGUAZAAgAGMAcgBvAHAAIAAoAGgAaQBnAGgAIAByAGEAaQBuAGYAYQBsAGwAKQBcACIALAAwAC4AMAAwADgALAAgAFwAIgBDAHIAbwBwAFwAIgAsACAAXAAiAE4AbwB0ACAAaQByAHIAaQBnAGEAdABlAGQAXAAiACwAIABcACIASABpAGcAaAAgAHIAYQBpAG4AZgBhAGwAbABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUwB1AGcAYQByAFwAIgAsADAALgAwADEAOQA5ACwAIABcACIAUwB1AGcAYQByAFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAEEAbgB5AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AdAB0AG8AbgBcACIALAAwAC4AMAAwADUAMwAsACAAXAAiAEMAbwB0AHQAbwBuAFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAEEAbgB5AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBIAG8AcgB0AGkAYwB1AGwAdAB1AHIAYQBsACAAYwByAG8AcABzAFwAIgAsADAALgAwADAANgA0ACwAIABcACIASABvAHIAdABpAGMAdQBsAHQAdQByAGEAbAAgAGMAcgBvAHAAcwBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBBAG4AeQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUgBpAGMAZQAgACgAYwBvAG4AdABpAG4AdQBvAHUAcwAgAGYAbABvAG8AZABpAG4AZwApAFwAIgAsADAALgAwADAAMwAsACAAXAAiAFIAaQBjAGUAXAAiACwAIABcACIAQwBvAG4AdABpAG4AdQBvAHUAcwAgAGYAbABvAG8AZABpAG4AZwBcACIALAAgAFwAIgBBAG4AeQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUgBpAGMAZQAgACgAcwBpAG4AZwBsAGUAIABhAG4AZAAgAG0AdQBsAHQAaQBwAGwAZQAgAGQAcgBhAGkAbgBhAGcAZQAsACAAbwByACAAYQBsAHQAZQByAG4AYQB0AGUAIAB3AGUAdAB0AGkAbgBnACAAYQBuAGQAIABkAHIAeQBpAG4AZwApAFwAIgAsADAALgAwADAANQAsACAAXAAiAFIAaQBjAGUAXAAiACwAIABcACIAUwBpAG4AZwBsAGUAIABhAG4AZAAgAG0AdQBsAHQAaQBwAGwAZQAgAGQAcgBhAGkAbgBhAGcAZQAsACAAbwByACAAYQBsAHQAZQByAG4AYQB0AGUAIAB3AGUAdAB0AGkAbgBnACAAYQBuAGQAIABkAHIAeQBpAG4AZwBcACIALAAgAFwAIgBBAG4AeQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQQBxAHUAYQBjAHUAbAB0AHUAcgBlAFwAIgAsADAALgAwADAAMgA2ACwAIABcACIAQQBxAHUAYQBjAHUAbAB0AHUAcgBlAFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAEEAbgB5AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBGAG8AcgBlAHMAdAByAHkAXAAiACwAMAAuADAAMAAxADgALAAgAFwAIgBGAG8AcgBlAHMAdAByAHkAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAQQBuAHkAXAAiAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgAgACAAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE4AMgBPAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAA1ACwAIAAxACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBWAEEAUgBJAEEAVABJAE8ATgAgAE8ARgAgAFMATwBVAFIAQwBFACAARABBAFQAQQA6AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBSAGUAbQBvAHYAZQBkACAAZAB1AHAAbABpAGMAYQB0AGUAIABcAHUAMAAwADIANwBBAHEAdQBhAGMAdQBsAHQAdQByAGUAXAB1ADAAMAAyADcAIAByAG8AdwAuAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBSAGUAbQBvAHYAZQBkACAAYQBzAHQAZQByAGkAcwBrAHMAIAB0AG8AIABhAGkAZAAgAGwAbwBvAGsAdQBwAC4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEEAZABkAGUAZAAgAFwAdQAwADAAMgA3AHAAcgBvAGQAdQBjAHQAaQBvAG4AIABzAHkAcwB0AGUAbQAgAG8AbgBsAHkAXAB1ADAAMAAyADcALAAgAFwAdQAwADAAMgA3AHIAYQBpAG4AZgBhAGwAbAAgAHoAbwBuAGUAXAB1ADAAMAAyADcAIABhAG4AZAAgAFwAdQAwADAAMgA3AGkAcgByAGkAZwBhAHQAaQBvAG4AIABtAGUAdABoAG8AZABcAHUAMAAwADIANwAgAGMAbwBsAHUAbQBuAHMAIAB0AG8AIABhAGkAZAAgAGwAbwBvAGsAdQBwAC4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEQAdQBwAGwAaQBjAGEAdABlAGQAIABcAHUAMAAwADIANwBuAG8AbgAtAGkAcgByAGkAZwBhAHQAZQBkACAAcABhAHMAdAB1AHIAZQBcAHUAMAAwADIANwAgAHIAbwB3ACAAdwBpAHQAaAAgAHMAYQBtAGUAIABFAEYAIABmAG8AcgAgAGwAbwB3ACAAYQBuAGQAIABoAGkAZwBoACAAcgBhAGkAbgBmAGEAbABsACAAegBvAG4AZQBzACAAdABvACAAYQBpAGQAIABsAG8AbwBrAHUAcAAuAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7ACIAfQAsAHsAIgBwAGEAdABoACIAOgAiAC8AcAByAG8AagBlAGMAdABzAC8AQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMAIgAsACIAdABlAHgAdAAiADoAIgBVAHQAaQBsAGkAdAB5AF8ARwBlAHQAQQByAHIAYQB5AFQAYQBiAGwAZQBSAG8AdwBTAHQAYQByAHQATgB1AG0AYgBlAHIAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABUAGEAYgBsAGUAaABlAGEAZABlAHIAQwBlAGwAbAAsAFIAbwB3AHMAQgBlAHQAdwBlAGUAbgBIAGUAYQBkAGUAcgBhAG4AZABBAHIAcgBhAHkALABcAG4AIAAgACAAIABSAE8AVwAoAFQAYQBiAGwAZQBoAGUAYQBkAGUAcgBDAGUAbABsACkAIAArACAAUgBvAHcAcwBCAGUAdAB3AGUAZQBuAEgAZQBhAGQAZQByAGEAbgBkAEEAcgByAGEAeQAgAC0AIAAxAFwAbgApADsAXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8ARwBlAHQAQQByAHIAYQB5AFQAYQBiAGwAZQBDAG8AbAB1AG0AbgBTAHQAYQByAHQATgB1AG0AYgBlAHIAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgAFQAYQBiAGwAZQBIAGUAYQBkAGUAcgBDAGUAbABsACwAXABuACAAIABDAE8ATABVAE0ATgAoAFQAYQBiAGwAZQBIAGUAYQBkAGUAcgBDAGUAbABsACkAXABuACkAOwBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBEAGkAcwBwAGwAYQB5AEEAcgByAGEAeQBJAG4AVABhAGIAbABlAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAQQByAHIAYQB5AEQAYQB0AGEALAAgAFQAYQBiAGwAZQBoAGUAYQBkAGUAcgBDAGUAbABsACwAIABSAG8AdwBzAEIAZQB0AHcAZQBlAG4ASABlAGEAZABlAHIAYQBuAGQAQQByAHIAYQB5ACwAIABbAEMAbwBsAHUAbQBuAHMAQgBlAHQAdwBlAGUAbgBIAGUAYQBkAGUAcgBBAG4AZABBAHIAcgBhAHkAXQAsAFwAbgAgAEkARgBFAFIAUgBPAFIAKABcAG4AIAAgACAAIAAgAEkATgBEAEUAWAAoAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABVAE4ASQBRAFUARQAoAEEAcgByAGEAeQBEAGEAdABhACkALAAgAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABSAE8AVwAoACkALQBVAHQAaQBsAGkAdAB5AF8ARwBlAHQAQQByAHIAYQB5AFQAYQBiAGwAZQBSAG8AdwBTAHQAYQByAHQATgB1AG0AYgBlAHIAKABUAGEAYgBsAGUAaABlAGEAZABlAHIAQwBlAGwAbAAsACAAUgBvAHcAcwBCAGUAdAB3AGUAZQBuAEgAZQBhAGQAZQByAGEAbgBkAEEAcgByAGEAeQApACwAIABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAQwBPAEwAVQBNAE4AKAApAC0AVQB0AGkAbABpAHQAeQBfAEcAZQB0AEEAcgByAGEAeQBUAGEAYgBsAGUAQwBvAGwAdQBtAG4AUwB0AGEAcgB0AE4AdQBtAGIAZQByACgAVABhAGIAbABlAGgAZQBhAGQAZQByAEMAZQBsAGwAKQAgACsAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAEkARgAoAEkAUwBPAE0ASQBUAFQARQBEACgAQwBvAGwAdQBtAG4AcwBCAGUAdAB3AGUAZQBuAEgAZQBhAGQAZQByAEEAbgBkAEEAcgByAGEAeQApACwAIAAxACwAIABDAG8AbAB1AG0AbgBzAEIAZQB0AHcAZQBlAG4ASABlAGEAZABlAHIAQQBuAGQAQQByAHIAYQB5ACkAXABuACAAIAAgACAAIAAgACAAIAApACwAIABcACIAXAAiAFwAbgAgACAAIAAgACkAXABuACkAOwBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBMAG8AbwBrAHUAcABWAGEAbAB1AGUASQBuAFQAYQBiAGwAZQBcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQAsACAATABvAG8AawB1AHAAQQByAHIAYQB5ACwAIABSAGUAdAB1AHIAbgBBAHIAcgBhAHkALABcAG4AIAAgACAAIABYAEwATwBPAEsAVQBQACgATABvAG8AawB1AHAAVgBhAGwAdQBlACwAIABMAG8AbwBrAHUAcABBAHIAcgBhAHkALAAgAFIAZQB0AHUAcgBuAEEAcgByAGEAeQAsACAAXAAiAFwAIgApAFwAbgApADsAXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8ATABvAG8AawB1AHAAVgBhAGwAdQBlAEkAbgBUAGEAYgBsAGUATgB1AG0AYgBlAHIAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABMAG8AbwBrAHUAcABWAGEAbAB1AGUALAAgAEwAbwBvAGsAdQBwAEEAcgByAGEAeQAsACAAUgBlAHQAdQByAG4AQQByAHIAYQB5ACwAXABuACAAIAAgACAASQBGACgASQBTAE4AVQBNAEIARQBSACgAXABuACAAIAAgACAAIAAgACAAIABYAEwATwBPAEsAVQBQACgATABvAG8AawB1AHAAVgBhAGwAdQBlACwAIABMAG8AbwBrAHUAcABBAHIAcgBhAHkALAAgAFIAZQB0AHUAcgBuAEEAcgByAGEAeQAsACAAXAAiAFwAIgApAFwAbgAgACAAIAAgACkALAAgAFgATABPAE8ASwBVAFAAKABMAG8AbwBrAHUAcABWAGEAbAB1AGUALAAgAEwAbwBvAGsAdQBwAEEAcgByAGEAeQAsACAAUgBlAHQAdQByAG4AQQByAHIAYQB5ACwAIABcACIAXAAiACkALAAgADAAKQBcAG4AKQA7AFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAFMAcABsAGkAdABTAHQAcgBpAG4AZwBJAG4AdABvAEEAcgByAGEAeQBcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAEMAZQBsAGwALAAgAEQAZQBsAGkAbQBpAHQAZQByACwAIABbAEMAaABhAHIAYQBjAHQAZQByAFQAbwBSAGUAbQBvAHYAZQAxAF0ALAAgAFsAQwBoAGEAcgBhAGMAdABlAHIAVABvAFIAZQBtAG8AdgBlADIAXQAsAFwAbgAgACAAIAAgACAAIAAgACAARgBJAEwAVABFAFIAWABNAEwAKABcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBcAHUAMAAwADMAYwB0AFwAdQAwADAAMwBlAFwAdQAwADAAMwBjAHMAXAB1ADAAMAAzAGUAXAAiACAAXAB1ADAAMAAyADYAXABuACAAIAAgACAAIAAgACAAIABTAFUAQgBTAFQASQBUAFUAVABFACgAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFMAVQBCAFMAVABJAFQAVQBUAEUAKABTAFUAQgBTAFQASQBUAFUAVABFACgAQwBlAGwAbAAsAEMAaABhAHIAYQBjAHQAZQByAFQAbwBSAGUAbQBvAHYAZQAxACwAXAAiAFwAIgApACwAQwBoAGEAcgBhAGMAdABlAHIAVABvAFIAZQBtAG8AdgBlADIALABcACIAXAAiACkALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAARABlAGwAaQBtAGkAdABlAHIALABcACIAXAB1ADAAMAAzAGMALwBzAFwAdQAwADAAMwBlAFwAdQAwADAAMwBjAHMAXAB1ADAAMAAzAGUAXAAiAFwAbgAgACAAIAAgACAAIAAgACAAKQAgAFwAdQAwADAAMgA2AFwAbgAgACAAIAAgACAAIAAgACAAXAAiAFwAdQAwADAAMwBjAC8AcwBcAHUAMAAwADMAZQBcAHUAMAAwADMAYwAvAHQAXAB1ADAAMAAzAGUAXAAiACwAXABuACAAIAAgACAAIAAgACAAIABcACIALwAvAHMAXAAiAFwAbgAgACAAIAAgACkAXABuACkAOwBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBHAGUAdABDAGwAaQBtAGEAdABlAFoAbwBuAGUAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABhAHYAZwBUAGUAbQBwACwAYQB2AGcAUgBhAGkAbgAsAGYAcgBvAHMAdABEAGEAeQBzACwAZQBsAGUAdgAsAG0AYQBwAF8AcABlAHQALABcAG4AIAAgACAAIABtAGkAbgBUAGUAbQBwAEEAcgByAGEAeQAsAG0AYQB4AFQAZQBtAHAAQQByAHIAYQB5ACwAXABuACAAIAAgACAAbQBpAG4AUgBhAGkAbgBmAGEAbABsAEEAcgByAGEAeQAsAG0AYQB4AFIAYQBpAG4AZgBhAGwAbABBAHIAcgBhAHkALABcAG4AIAAgACAAIABtAGkAbgBGAHIAbwBzAHQAQQByAHIAYQB5ACwAbQBhAHgARgByAG8AcwB0AEEAcgByAGEAeQAsAFwAbgAgACAAIAAgAG0AaQBuAEUAbABlAHYAYQB0AGkAbwBuAEEAcgByAGEAeQAsAG0AYQB4AEUAbABlAHYAYQB0AGkAbwBuAEEAcgByAGEAeQAsAFwAbgAgACAAIAAgAG0AaQBuAFAARQBUAEEAcgByAGEAeQAsAG0AYQB4AFAARQBUAEEAcgByAGEAeQAsAFwAbgAgACAAIAAgAGMAbABpAG0AYQB0AGUAWgBvAG4AZQBBAHIAcgBhAHkALABcAG4AIAAgACAAIABMAEUAVAAoAFwAbgAgACAAIAAgACAAIAAgACAAbQBhAHMAawAsAFwAbgAgACAAIAAgACAAIAAgACAAKABWAEEATABVAEUAKABtAGkAbgBUAGUAbQBwAEEAcgByAGEAeQApAFwAdQAwADAAMwBjAD0AYQB2AGcAVABlAG0AcAApACoAXABuACAAIAAgACAAIAAgACAAIAAoAFYAQQBMAFUARQAoAG0AYQB4AFQAZQBtAHAAQQByAHIAYQB5ACkAXAB1ADAAMAAzAGUAPQBhAHYAZwBUAGUAbQBwACkAKgBcAG4AIAAgACAAIAAgACAAIAAgACgAVgBBAEwAVQBFACgAbQBpAG4AUgBhAGkAbgBmAGEAbABsAEEAcgByAGEAeQApAFwAdQAwADAAMwBjAD0AYQB2AGcAUgBhAGkAbgApACoAXABuACAAIAAgACAAIAAgACAAIAAoAFYAQQBMAFUARQAoAG0AYQB4AFIAYQBpAG4AZgBhAGwAbABBAHIAcgBhAHkAKQBcAHUAMAAwADMAZQA9AGEAdgBnAFIAYQBpAG4AKQAqAFwAbgAgACAAIAAgACAAIAAgACAAKABWAEEATABVAEUAKABtAGkAbgBGAHIAbwBzAHQAQQByAHIAYQB5ACkAXAB1ADAAMAAzAGMAPQBmAHIAbwBzAHQARABhAHkAcwApACoAXABuACAAIAAgACAAIAAgACAAIAAoAFYAQQBMAFUARQAoAG0AYQB4AEYAcgBvAHMAdABBAHIAcgBhAHkAKQBcAHUAMAAwADMAZQA9AGYAcgBvAHMAdABEAGEAeQBzACkAKgBcAG4AIAAgACAAIAAgACAAIAAgACgAVgBBAEwAVQBFACgAbQBpAG4ARQBsAGUAdgBhAHQAaQBvAG4AQQByAHIAYQB5ACkAXAB1ADAAMAAzAGMAPQBlAGwAZQB2ACkAKgBcAG4AIAAgACAAIAAgACAAIAAgACgAVgBBAEwAVQBFACgAbQBhAHgARQBsAGUAdgBhAHQAaQBvAG4AQQByAHIAYQB5ACkAXAB1ADAAMAAzAGUAPQBlAGwAZQB2ACkAKgBcAG4AIAAgACAAIAAgACAAIAAgACgAVgBBAEwAVQBFACgAbQBpAG4AUABFAFQAQQByAHIAYQB5ACkAXAB1ADAAMAAzAGMAPQBtAGEAcABfAHAAZQB0ACkAKgBcAG4AIAAgACAAIAAgACAAIAAgACgAVgBBAEwAVQBFACgAbQBhAHgAUABFAFQAQQByAHIAYQB5ACkAXAB1ADAAMAAzAGUAPQBtAGEAcABfAHAAZQB0ACkALABcAG4AIAAgACAAIAAgACAAIAAgAFQAQQBLAEUAKABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAARgBJAEwAVABFAFIAKABjAGwAaQBtAGEAdABlAFoAbwBuAGUAQQByAHIAYQB5ACwAbQBhAHMAawAsACAAXAAiAE4AbwAgAG0AYQB0AGMAaABcACIAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAxAFwAbgAgACAAIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgApADsAXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8ATABvAG8AawB1AHAASQB0AGUAbQBGAHIAbwBtAE0AaQBuAE0AYQB4AFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATABvAG8AawB1AHAAVgBhAGwAdQBlACwAIABNAGkAbgBBAHIAcgBhAHkALAAgAE0AYQB4AEEAcgByAGEAeQAsACAASQB0AGUAbQBBAHIAcgBhAHkALABcAG4AIAAgACAAIABMAEUAVAAoAFwAbgAgACAAIAAgACAAIAAgACAAbQBhAHMAawAsAFwAbgAgACAAIAAgACAAIAAgACAAKABWAEEATABVAEUAKABNAGkAbgBBAHIAcgBhAHkAKQBcAHUAMAAwADMAYwA9AEwAbwBvAGsAdQBwAFYAYQBsAHUAZQApACoAXABuACAAIAAgACAAIAAgACAAIAAoAFYAQQBMAFUARQAoAE0AYQB4AEEAcgByAGEAeQApAFwAdQAwADAAMwBlAD0ATABvAG8AawB1AHAAVgBhAGwAdQBlACkALABcAG4AIAAgACAAIAAgACAAIAAgAEYASQBMAFQARQBSACgASQB0AGUAbQBBAHIAcgBhAHkALAAgAG0AYQBzAGsALAAgAFwAIgBOAG8AIABtAGEAdABjAGgAXAAiACkAXABuACAAIAAgACAAKQBcAG4AKQA7AFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAFMAdQBtAFEAdQBhAG4AdABpAHQAeQBGAHIAbwBtAEMAcgBpAHQAZQByAGkAYQBcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgACAAQwByAGkAdABlAHIAaQBhADEALAAgAEMAcgBpAHQAZQByAGkAYQAxAFQAeQBwAGUAQQByAHIAYQB5ACwAIABRAHUAYQBuAHQAaQB0AHkALAAgAFsATQB1AGwAdABpAHAAbABpAGUAcgBdACwAIABbAEMAcgBpAHQAZQByAGkAYQAyAF0ALABbAEMAcgBpAHQAZQByAGkAYQAyAEEAcgByAGEAeQBdACwAXABuACAAIABMAEUAVAAoAFwAbgAgACAAIAAgAG0AdQBsAHQAaQBwAGwAaQBlAHIALAAgAEkARgAoAEkAUwBPAE0ASQBUAFQARQBEACgATQB1AGwAdABpAHAAbABpAGUAcgApACwAMQAsAE0AdQBsAHQAaQBwAGwAaQBlAHIAKQAsAFwAbgAgACAAIAAgAHEAdQBhAG4AdABpAHQAeQAsACAAUQB1AGEAbgB0AGkAdAB5ACoATQB1AGwAdABpAHAAbABpAGUAcgAsAFwAbgAgACAAIAAgAGMAcgBpAHQAZQByAGkAYQAxACwALQAtACgAQwByAGkAdABlAHIAaQBhADEAVAB5AHAAZQBBAHIAcgBhAHkAPQBDAHIAaQB0AGUAcgBpAGEAMQApACwAXABuACAAIAAgACAAYwByAGkAdABlAHIAaQBhADIALABJAEYAKABJAFMATwBNAEkAVABUAEUARAAoAEMAcgBpAHQAZQByAGkAYQAyACkALAAxACwALQAtACgAQwByAGkAdABlAHIAaQBhADIAQQByAHIAYQB5AD0AQwByAGkAdABlAHIAaQBhADIAKQApACwAXABuACAAIAAgACAAUwBVAE0AUABSAE8ARABVAEMAVAAoAGMAcgBpAHQAZQByAGkAYQAxACoAYwByAGkAdABlAHIAaQBhADIAKgBxAHUAYQBuAHQAaQB0AHkAKQBcAG4AIAAgACkAXABuACkAOwBcAG4AXABuAGcAZQB0AE8AdgBlAHIAbABhAHAAcABpAG4AZwBSAGUAcABvAHIAdABpAG4AZwBDAHkAYwBsAGUAcwBcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAFAAcgBvAGQAdQBjAHQAaQBvAG4AQwB5AGMAbABlAFMAdABhAHIAdAAsAFAAcgBvAGQAdQBjAHQAaQBvAG4AQwB5AGMAbABlAEUAbgBkACwAUgBlAHAAbwByAHQAaQBuAGcAQwB5AGMAbABlAFMAdABhAHIAdAAsAFwAbgAgACAAIAAgAEwARQBUACgAXABuACAAIAAgACAAIAAgACAAIABTACwAUAByAG8AZAB1AGMAdABpAG8AbgBDAHkAYwBsAGUAUwB0AGEAcgB0ACwAXABuACAAIAAgACAAIAAgACAAIABFACwAUAByAG8AZAB1AGMAdABpAG8AbgBDAHkAYwBsAGUARQBuAGQALABcAG4AIAAgACAAIAAgACAAIAAgAG0ALABNAE8ATgBUAEgAKABSAGUAcABvAHIAdABpAG4AZwBDAHkAYwBsAGUAUwB0AGEAcgB0ACkALABcAG4AIAAgACAAIAAgACAAIAAgAGQALABEAEEAWQAoAFIAZQBwAG8AcgB0AGkAbgBnAEMAeQBjAGwAZQBTAHQAYQByAHQAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAUABlAHIAaQBvAGQARQBuAGQALABMAEEATQBCAEQAQQAoAHMAdAAsAEUARABBAFQARQAoAHMAdAAsADEAMgApAC0AMQApACwAXABuACAAIAAgACAAIAAgACAAIABBACwAUwAtADMANgA1ACwAXABuACAAIAAgACAAIAAgACAAIAB5AGEALABZAEUAQQBSACgAQQApACwAXABuACAAIAAgACAAIAAgACAAIAB5AGIALABZAEUAQQBSACgARQApACwAXABuACAAIAAgACAAIAAgACAAIABmAGkAcgBzAHQAWQBlAGEAcgAsAHkAYQArACgAUABlAHIAaQBvAGQARQBuAGQAKABEAEEAVABFACgAeQBhACwAbQAsAGQAKQApAFwAdQAwADAAMwBjACAAUwApACwAXABuACAAIAAgACAAIAAgACAAIABsAGEAcwB0AFkAZQBhAHIALAB5AGIALQAoAEQAQQBUAEUAKAB5AGIALABtACwAZAApAFwAdQAwADAAMwBlACAARQApACwAXABuACAAIAAgACAAIAAgACAAIABNAEEAWAAoADAALABsAGEAcwB0AFkAZQBhAHIALQBmAGkAcgBzAHQAWQBlAGEAcgArADEAKQBcAG4AIAAgACAAIAApAFwAbgApADsAXABuAFwAbgBnAGUAdABPAHYAZQByAGwAYQBwAHAAaQBuAGcAUgBlAHAAbwByAHQAaQBuAGcAUABlAHIAaQBvAGQAcwBcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAFAAcgBvAGQAdQBjAHQAaQBvAG4AQwB5AGMAbABlAFMAdABhAHIAdAAsAFAAcgBvAGQAdQBjAHQAaQBvAG4AQwB5AGMAbABlAEUAbgBkACwAUgBlAHAAbwByAHQAaQBuAGcAQwB5AGMAbABlAFMAdABhAHIAdAAsAFwAbgAgACAAIAAgAEwARQBUACgAXABuACAAIAAgACAAIAAgACAAIABTACwAUAByAG8AZAB1AGMAdABpAG8AbgBDAHkAYwBsAGUAUwB0AGEAcgB0ACwAXABuACAAIAAgACAAIAAgACAAIABFACwAUAByAG8AZAB1AGMAdABpAG8AbgBDAHkAYwBsAGUARQBuAGQALABcAG4AIAAgACAAIAAgACAAIAAgAG0ALABNAE8ATgBUAEgAKABSAGUAcABvAHIAdABpAG4AZwBDAHkAYwBsAGUAUwB0AGEAcgB0ACkALABcAG4AIAAgACAAIAAgACAAIAAgAGQALABEAEEAWQAoAFIAZQBwAG8AcgB0AGkAbgBnAEMAeQBjAGwAZQBTAHQAYQByAHQAKQAsACAALwAqAGgAZQBsAHAAZQByADoAIABlAG4AZAAgAGQAYQB0AGUAIABmAG8AcgAgAGEAIAByAGUAcABvAHIAdABpAG4AZwAgAHAAZQByAGkAbwBkACAAcwB0AGEAcgB0AGkAbgBnACAAYQB0ACAAYQAgAGcAaQB2AGUAbgAgAGQAYQB0AGUAKgAvAFwAbgAgACAAIAAgACAAIAAgACAAUABlAHIAaQBvAGQARQBuAGQALABMAEEATQBCAEQAQQAoAHMAdAAsAEUARABBAFQARQAoAHMAdAAsADEAMgApAC0AMQApACwAIAAvACoAbwBuAGwAeQAgAG4AZQBlAGQAIAB0AG8AIABsAG8AbwBrACAAYgBhAGMAawAgADMANgA1ACAAZABhAHkAcwAoAG0AYQB4ACAAbwB2AGUAcgBsAGEAcAAgAHcAaQBuAGQAbwB3ACkAKgAvAFwAbgAgACAAIAAgACAAIAAgACAAQQAsAFMALQAzADYANQAsAFwAbgAgACAAIAAgACAAIAAgACAAeQBhACwAWQBFAEEAUgAoAEEAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAeQBiACwAWQBFAEEAUgAoAEUAKQAsACAALwAqAGkAZgAgAHQAaABlACAAYQBuAGMAaABvAHIAIABmAG8AcgAgAHkAYQAgAGUAbgBkAHMAIABiAGUAZgBvAHIAZQAgAFMALABpAHQAIABjAGEAbgBcAHUAMAAwADIANwB0ACAAbwB2AGUAcgBsAGEAcAA7ACAAbQBvAHYAZQAgAHQAbwAgAG4AZQB4AHQAIAB5AGUAYQByACoALwBcAG4AIAAgACAAIAAgACAAIAAgAGYAaQByAHMAdABZAGUAYQByACwAeQBhACsAKABQAGUAcgBpAG8AZABFAG4AZAAoAEQAQQBUAEUAKAB5AGEALABtACwAZAApACkAXAB1ADAAMAAzAGMAUwApACwAIAAvACoAaQBmACAAdABoAGUAIABhAG4AYwBoAG8AcgAgAGYAbwByACAAeQBiACAAcwB0AGEAcgB0AHMAIABhAGYAdABlAHIAIABFACwAaQB0ACAAYwBhAG4AXAB1ADAAMAAyADcAdAAgAG8AdgBlAHIAbABhAHAAOwAgAG0AbwB2AGUAIAB0AG8AIABwAHIAZQB2AGkAbwB1AHMAIAB5AGUAYQByACoALwBcAG4AIAAgACAAIAAgACAAIAAgAGwAYQBzAHQAWQBlAGEAcgAsAHkAYgAtACgARABBAFQARQAoAHkAYgAsAG0ALABkACkAXAB1ADAAMAAzAGUARQApACwAXABuACAAIAAgACAAIAAgACAAIABuACwATQBBAFgAKAAwACwAbABhAHMAdABZAGUAYQByAC0AZgBpAHIAcwB0AFkAZQBhAHIAKwAxACkALABcAG4AIAAgACAAIAAgACAAIAAgAHkAcgBzACwAUwBFAFEAVQBFAE4AQwBFACgAbgAsADEALABmAGkAcgBzAHQAWQBlAGEAcgAsADEAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAcwB0AGEAcgB0AHMALABEAEEAVABFACgAeQByAHMALABtACwAZAApACwAXABuACAAIAAgACAAIAAgACAAIABlAG4AZABzACwATQBBAFAAKABzAHQAYQByAHQAcwAsAFAAZQByAGkAbwBkAEUAbgBkACkALABcAG4AIAAgACAAIAAgACAAIAAgAHQAYQBnACwASQBGACgAcwB0AGEAcgB0AHMAPQBSAGUAcABvAHIAdABpAG4AZwBDAHkAYwBsAGUAUwB0AGEAcgB0ACwAXAAiACAAKABUAGgAaQBzACAAcgBlAHAAbwByAHQAaQBuAGcAIABjAHkAYwBsAGUAKQBcACIALABcACIAXAAiACkALABcAG4AIAAgACAAIAAgACAAIAAgAHMAdABhAHIAdABzAFQAZQB4AHQALABUAEUAWABUACgAcwB0AGEAcgB0AHMALABcACIAZABkACAAbQBtAG0AIAB5AHkAeQB5AFwAIgApACwAXABuACAAIAAgACAAIAAgACAAIABlAG4AZABzAFQAZQB4AHQALABUAEUAWABUACgAZQBuAGQAcwAsAFwAIgBkAGQAIABtAG0AbQAgAHkAeQB5AHkAXAAiACkALABcAG4AIAAgACAAIAAgACAAIAAgAEkARgAoAG4APQAwACwAXAAiAFwAIgAsAEgAUwBUAEEAQwBLACgAcwB0AGEAcgB0AHMAVABlAHgAdAAgAFwAdQAwADAAMgA2ACAAXAAiACAAdABvACAAXAAiACAAXAB1ADAAMAAyADYAIABlAG4AZABzAFQAZQB4AHQAIABcAHUAMAAwADIANgAgAHQAYQBnACkAKQBcAG4AIAAgACAAIAApAFwAbgApADsAXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8ARABpAHMAcABsAGEAeQBGAHUAbgBjAHQAaQBvAG4ATgBhAG0AZQBcAG4APQBMAEEATQBCAEQAQQAoAEYAdQBuAGMAdABpAG8AbgAsACAAVABFAFgAVABCAEUARgBPAFIARQAoAEYATwBSAE0AVQBMAEEAVABFAFgAVAAoAEYAdQBuAGMAdABpAG8AbgApACwAIABcACIAKABcACIAKQApADsAXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8ATABvAG8AawB1AHAATgAyAE8ARQBGAEYAcgBvAG0AUAByAG8AZABJAHIAcgBpAGcAYQB0AGkAbwBuAFIAYQBpAG4AZgBhAGwAbABcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAFAAcgBvAGQAdQBjAHQAaQBvAG4AUwB5AHMAdABlAG0ALAAgAEkAcgByAGkAZwBhAHQAaQBvAG4ATQBlAHQAaABvAGQALAAgAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlACwAXABuACAAIAAgACAAUAByAG8AZAB1AGMAdABpAG8AbgBTAHkAcwB0AGUAbQBBAHIAcgBhAHkALAAgAEkAcgByAGkAZwBhAHQAaQBvAG4ATQBlAHQAaABvAGQAQQByAHIAYQB5ACwAIABSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBBAHIAcgBhAHkALABSAGUAdAB1AHIAbgBBAHIAcgBhAHkALABcAG4AIAAgACAAIABMAEUAVAAoAFwAbgAgACAAIAAgACAAIAAgACAASQByAHIAaQBnAGEAdABpAG8AbgBNAGUAdABoAG8AZAAsACAASQBGACgASQByAHIAaQBnAGEAdABpAG8AbgBNAGUAdABoAG8AZAA9AFwAIgBOAG8AdAAgAGkAcgByAGkAZwBhAHQAZQBkAFwAIgAsACAAXAAiAE4AbwB0ACAAaQByAHIAaQBnAGEAdABlAGQAXAAiACwAIABcACIAQQBuAHkAXAAiACkALABcAG4AIAAgACAAIAAgACAAIAAgAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlACwAIABJAEYAKABJAHIAcgBpAGcAYQB0AGkAbwBuAE0AZQB0AGgAbwBkACAAPQAgAFwAIgBOAG8AdAAgAGkAcgByAGkAZwBhAHQAZQBkAFwAIgAsACAAUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUALAAgAFwAIgBBAG4AeQBcACIAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAWABMAE8ATwBLAFUAUAAoADEALAAgAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAoAFAAcgBvAGQAdQBjAHQAaQBvAG4AUwB5AHMAdABlAG0AQQByAHIAYQB5AD0AUAByAG8AZAB1AGMAdABpAG8AbgBTAHkAcwB0AGUAbQApACoAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACgASQByAHIAaQBnAGEAdABpAG8AbgBNAGUAdABoAG8AZABBAHIAcgBhAHkAPQBJAHIAcgBpAGcAYQB0AGkAbwBuAE0AZQB0AGgAbwBkACkAKgBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAKABSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBBAHIAcgBhAHkAPQBSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQApACwAIABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAUgBlAHQAdQByAG4AQQByAHIAYQB5ACkAXABuACAAIAAgACAAKQBcAG4AKQA7ACIAfQAsAHsAIgBwAGEAdABoACIAOgAiAC8AcAByAG8AagBlAGMAdABzAC8AQwBvAG0AbQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAiACwAIgB0AGUAeAB0ACIAOgAiAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQATgAyAE8AVABvAEMATwAyAGUAXABuAEMAbwBuAHYAZQByAHQAIABuAGkAdAByAG8AdQBzACAAbwB4AGkAZABlACAAZQBtAGkAcwBzAGkAbwBuAHMAIAB0AG8AIABjAGEAcgBiAG8AbgAgAGQAaQBvAHgAaQBkAGUAIABlAHEAdQBpAHYAYQBsAGUAbgB0ACAAZQBtAGkAcwBzAGkAbwBuAHMAXABuAEUATgAyAE8AIABDAE8AMgBlAFwAbgB0ACAAQwBPADIAZQBcAG4ARQBOADIATwA6ACAAbgBpAHQAcgBvAHUAcwAgAG8AeABpAGQAZQAgAGUAbQBpAHMAcwBpAG8AbgBzACAAKAB0ACAATgAyAE8AKQBcAG4ARwBXAFAATgAyAE8AOgAgAGcAbABvAGIAYQBsACAAdwBhAHIAbQBpAG4AZwAgAHAAbwB0AGUAbgB0AGkAYQBsACAAZgBvAHIAIABuAGkAdAByAG8AdQBzACAAbwB4AGkAZABlACAAKAB0ACAAQwBPADIALQBlACAALwAgAHQAIABOADIATwApAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAFwAbgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQATgAyAE8AVABvAEMATwAyAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAARQBfAE4AMgBPACwAIABHAFcAUABfAE4AMgBPACwAXABuACAAIAAgACAARQBfAE4AMgBPACAAKgAgAEcAVwBQAF8ATgAyAE8AXABuACAAIAApAFwAbgA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AE4AMgBPAFQAbwBDAE8AMgBlAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBDAG8AbgB2AGUAcgB0ACAAbgBpAHQAcgBvAHUAcwAgAG8AeABpAGQAZQAgAGUAbQBpAHMAcwBpAG8AbgBzACAAdABvACAAYwBhAHIAYgBvAG4AIABkAGkAbwB4AGkAZABlACAAZQBxAHUAaQB2AGEAbABlAG4AdAAgAGUAbQBpAHMAcwBpAG8AbgBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQATgAyAE8AVABvAEMATwAyAGUAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEUATgAyAE8AIABDAE8AMgBlAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQATgAyAE8AVABvAEMATwAyAGUAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgB0ACAAQwBPADIAZQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AE4AMgBPAFQAbwBDAE8AMgBlAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQATgAyAE8AVABvAEMATwAyAGUAXwBMAGEAdABlAHgARQBxAHUAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBDAE8AMgBfAGUAIAA9ACAARQBfAHsATgAyAE8AfQAgAFwAXAB0AGkAbQBlAHMAIABHAFcAUABfAHsATgAyAE8AfQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AE4AMgBPAFQAbwBDAE8AMgBlAF8AQQByAGcAdQBtAGUAbgB0AHMAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAyACwAIAAyACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBFAE4AMgBPAFwAIgAsAFwAIgBOAGkAdAByAG8AdQBzACAAbwB4AGkAZABlACAAZQBtAGkAcwBzAGkAbwBuAHMAIAAoAHQAIABOADIATwApAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBHAFcAUABOADIATwBcACIALABcACIARwBsAG8AYgBhAGwAIAB3AGEAcgBtAGkAbgBnACAAcABvAHQAZQBuAHQAaQBhAGwAIABmAG8AcgAgAG4AaQB0AHIAbwB1AHMAIABvAHgAaQBkAGUAIAAoAHQAIABDAE8AMgAtAGUAIAAvACAAdAAgAE4AMgBPACkAXAAiAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQAQwBIADQAVABvAEMATwAyAGUAXABuAEMAbwBuAHYAZQByAHQAIABtAGUAdABoAGEAbgBlACAAZQBtAGkAcwBzAGkAbwBuAHMAIAB0AG8AIABjAGEAcgBiAG8AbgAgAGQAaQBvAHgAaQBkAGUAIABlAHEAdQBpAHYAYQBsAGUAbgB0ACAAZQBtAGkAcwBzAGkAbwBuAHMAXABuAEUAQwBIADQAIABDAE8AMgBlAFwAbgB0ACAAQwBPADIAZQBcAG4ARQBDAEgANAA6ACAAbQBlAHQAaABhAG4AZQAgAGUAbQBpAHMAcwBpAG8AbgBzACAAKAB0ACAAQwBIADQAKQBcAG4ARwBXAFAAQwBIADQAOgAgAGcAbABvAGIAYQBsACAAdwBhAHIAbQBpAG4AZwAgAHAAbwB0AGUAbgB0AGkAYQBsACAAZgBvAHIAIABtAGUAdABoAGEAbgBlACAAKAB0ACAAQwBPADIALQBlACAALwAgAHQAIABDAEgANAApAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAFwAbgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQAQwBIADQAVABvAEMATwAyAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAARQBfAEMASAA0ACwAIABHAFcAUABfAEMASAA0ACwAXABuACAAIAAgACAARQBfAEMASAA0ACAAKgAgAEcAVwBQAF8AQwBIADQAXABuACAAIAApAFwAbgA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AEMASAA0AFQAbwBDAE8AMgBlAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBDAG8AbgB2AGUAcgB0ACAAbQBlAHQAaABhAG4AZQAgAGUAbQBpAHMAcwBpAG8AbgBzACAAdABvACAAYwBhAHIAYgBvAG4AIABkAGkAbwB4AGkAZABlACAAZQBxAHUAaQB2AGEAbABlAG4AdAAgAGUAbQBpAHMAcwBpAG8AbgBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQAQwBIADQAVABvAEMATwAyAGUAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEUAQwBIADQAIABDAE8AMgBlAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQAQwBIADQAVABvAEMATwAyAGUAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgB0ACAAQwBPADIAZQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AEMASAA0AFQAbwBDAE8AMgBlAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQAQwBIADQAVABvAEMATwAyAGUAXwBMAGEAdABlAHgARQBxAHUAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBDAE8AMgBfAGUAIAA9ACAARQBfAHsAQwBIADQAfQAgAFwAXAB0AGkAbQBlAHMAIABHAFcAUABfAHsAQwBIADQAfQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AEMASAA0AFQAbwBDAE8AMgBlAF8AQQByAGcAdQBtAGUAbgB0AHMAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAyACwAIAAyACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBFAEMASAA0AFwAIgAsAFwAIgBNAGUAdABoAGEAbgBlACAAZQBtAGkAcwBzAGkAbwBuAHMAIAAoAHQAIABDAEgANAApAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBHAFcAUABDAEgANABcACIALABcACIARwBsAG8AYgBhAGwAIAB3AGEAcgBtAGkAbgBnACAAcABvAHQAZQBuAHQAaQBhAGwAIABmAG8AcgAgAG0AZQB0AGgAYQBuAGUAIAAoAHQAIABDAE8AMgAtAGUAIAAvACAAdAAgAEMASAA0ACkAXAAiAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAIgB9AF0ALAAiAHAAcgBvAGoAZQBjAHQATgBhAG0AZQBzACIAOgBbACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABlAG4AcwBpAHQAeQBPAGYATQBlAHQAaABhAG4AZQBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGUAbgBzAGkAdAB5AE8AZgBNAGUAdABoAGEAbgBlAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGUAbgBzAGkAdAB5AE8AZgBNAGUAdABoAGEAbgBlAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABlAG4AcwBpAHQAeQBPAGYATQBlAHQAaABhAG4AZQBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABOADIAbwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAQwBnAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQATgAyAG8ARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAEMAZwBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AE4AMgBvAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBDAGcAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQATgAyAG8ARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAEMAZwBfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQATgAyAG8ARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAEMAZwBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQARwBhAHMARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEcAVwBQAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEcAVwBQAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEcAVwBQAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBHAFcAUABfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEcAVwBQAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBBAHUAcwB0AHIAYQBsAGkAYQBuAFMAdABhAHQAZQBzAFQAZQByAHIAaQB0AG8AcgBpAGUAcwBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBBAHUAcwB0AHIAYQBsAGkAYQBuAFMAdABhAHQAZQBzAFQAZQByAHIAaQB0AG8AcgBpAGUAcwBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBBAHUAcwB0AHIAYQBsAGkAYQBuAFMAdABhAHQAZQBzAFQAZQByAHIAaQB0AG8AcgBpAGUAcwBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQQB1AHMAdAByAGEAbABpAGEAbgBTAHQAYQB0AGUAcwBUAGUAcgByAGkAdABvAHIAaQBlAHMAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBBAHUAcwB0AHIAYQBsAGkAYQBuAFMAdABhAHQAZQBzAFQAZQByAHIAaQB0AG8AcgBpAGUAcwBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBBAFMAQQA0AEEAcgBlAGEAcwBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAEEAUwBBADQAQQByAGUAYQBzAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAQQBTAEEANABBAHIAZQBhAHMAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAQQBTAEEANABBAHIAZQBhAHMAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAEEAUwBBADQAQQByAGUAYQBzAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAGUAdABBAG4AZABEAHIAeQBaAG8AbgBlAHMAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBlAHQAQQBuAGQARAByAHkAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAZQB0AEEAbgBkAEQAcgB5AFoAbwBuAGUAcwBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBlAHQAQQBuAGQARAByAHkAWgBvAG4AZQBzAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBlAHQAQQBuAGQARAByAHkAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBlAHQAQQBuAGQARAByAHkAWgBvAG4AZQBzAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBsAGkAbQBhAHQAZQBaAG8AbgBlAHMAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbABpAG0AYQB0AGUAWgBvAG4AZQBzAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAEEAcABwAGUAbgBkAGkAYwBlAHMAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAcwBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAHMAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAHMAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAcwBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUAcwBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlAHMAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlAHMAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUAcwBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlAHMAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlAHMAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAdABhAFMAYwBvAHIAZQBzAF8AUwBjAG8AcABlADMAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAHQAYQBTAGMAbwByAGUAcwBfAFMAYwBvAHAAZQAzAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQB0AGEAUwBjAG8AcgBlAHMAXwBTAGMAbwBwAGUAMwBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAHQAYQBTAGMAbwByAGUAcwBfAFMAYwBvAHAAZQAzAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAHQAYQBTAGMAbwByAGUAcwBfAFMAYwBvAHAAZQAzAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAHQAYQBTAGMAbwByAGUAcwBfAFMAYwBvAHAAZQAzAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAEwARQBBAEMASABfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAEwARQBBAEMASABfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAEwARQBBAEMASABfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMATABFAEEAQwBIAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAEwARQBBAEMASABfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBsAGUAYQBjAGgAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAGwAZQBhAGMAaABfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAGwAZQBhAGMAaABfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBsAGUAYQBjAGgAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAbABlAGEAYwBoAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAbABlAGEAYwBoAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8ARwBlAHQAQQByAHIAYQB5AFQAYQBiAGwAZQBSAG8AdwBTAHQAYQByAHQATgB1AG0AYgBlAHIAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8ARwBlAHQAQQByAHIAYQB5AFQAYQBiAGwAZQBDAG8AbAB1AG0AbgBTAHQAYQByAHQATgB1AG0AYgBlAHIAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8ARABpAHMAcABsAGEAeQBBAHIAcgBhAHkASQBuAFQAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBMAG8AbwBrAHUAcABWAGEAbAB1AGUASQBuAFQAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBMAG8AbwBrAHUAcABWAGEAbAB1AGUASQBuAFQAYQBiAGwAZQBOAHUAbQBiAGUAcgAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBTAHAAbABpAHQAUwB0AHIAaQBuAGcASQBuAHQAbwBBAHIAcgBhAHkAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8ARwBlAHQAQwBsAGkAbQBhAHQAZQBaAG8AbgBlACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAEwAbwBvAGsAdQBwAEkAdABlAG0ARgByAG8AbQBNAGkAbgBNAGEAeAAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBTAHUAbQBRAHUAYQBuAHQAaQB0AHkARgByAG8AbQBDAHIAaQB0AGUAcgBpAGEAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBnAGUAdABPAHYAZQByAGwAYQBwAHAAaQBuAGcAUgBlAHAAbwByAHQAaQBuAGcAQwB5AGMAbABlAHMAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBnAGUAdABPAHYAZQByAGwAYQBwAHAAaQBuAGcAUgBlAHAAbwByAHQAaQBuAGcAUABlAHIAaQBvAGQAcwAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBEAGkAcwBwAGwAYQB5AEYAdQBuAGMAdABpAG8AbgBOAGEAbQBlACIAXQAsACIAbABvAGMAYQBsAGUAIgA6AHsAIgBsAGkAcwB0AFMAZQBwAGEAcgBhAHQAbwByACIAOgAiACwAIgAsACIAcgBvAHcAUwBlAHAAYQByAGEAdABvAHIAIgA6ACIAOwAiACwAIgBjAG8AbAB1AG0AbgBTAGUAcABhAHIAYQB0AG8AcgAiADoAIgAsACIALAAiAHQAaABvAHUAcwBhAG4AZABzAFMAZQBwAGEAcgBhAHQAbwByACIAOgAiACwAIgAsACIAdABoAG8AdQBzAGEAbgBkAHMAUABvAHMAaQB0AGkAbwBuAHMAIgA6AFsAMwBdACwAIgBkAGUAYwBpAG0AYQBsAFMAZQBwAGEAcgBhAHQAbwByACIAOgAiAC4AIgAsACIAZABhAHQAZQBPAHIAZABlAHIAIgA6ACIARABNAFkAIgAsACIAYwB1AHIAcgBlAG4AYwB5AFMAeQBtAGIAbwBsACIAOgAiACQAIgAsACIAaQBzAEMAdQByAHIAZQBuAGMAeQBTAHkAbQBiAG8AbABMAGUAYQBkACIAOgB0AHIAdQBlACwAIgBpAHMAQwB1AHIAcgBlAG4AYwB5AFMAZQBwAEIAeQBTAHAAYQBjAGUAIgA6AGYAYQBsAHMAZQAsACIAcgBvAHcATABlAHQAdABlAHIAIgA6ACIAUgAiACwAIgBjAG8AbAB1AG0AbgBMAGUAdAB0AGUAcgAiADoAIgBDACIALAAiAHIAYwBMAGUAZgB0AEIAcgBhAGMAawBlAHQAIgA6ACIAWwAiACwAIgByAGMAUgBpAGcAaAB0AEIAcgBhAGMAawBlAHQAIgA6ACIAXQAiACwAIgBzAHQAYQB0AGUAbQBlAG4AdABTAGUAcABhAHIAYQB0AG8AcgAiADoAIgA7ACIALAAiAGwAbwBjAGEAbABlAE4AYQBtAGUAIgA6ACIAZQBuAC0AdQBzACIAfQB9AA==</AFEJSONBlob>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9A9CF321-0D35-4044-BC72-33748FE2B865}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{CD460F9D-420A-4723-B323-396E4D19EC9B}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="09eef6d6-daa8-4301-8f9f-b1ec38079286"/>
+    <ds:schemaRef ds:uri="7291119c-fce9-4911-96ae-b800be5dccd8"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -4456,12 +4893,9 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{CD460F9D-420A-4723-B323-396E4D19EC9B}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9A9CF321-0D35-4044-BC72-33748FE2B865}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="09eef6d6-daa8-4301-8f9f-b1ec38079286"/>
-    <ds:schemaRef ds:uri="7291119c-fce9-4911-96ae-b800be5dccd8"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>